<commit_message>
Expand 황우중 W30 directive to 10 task rows (ch.2 split by section)
Expand §3 task table and completion-report sheet from 5 to 10 rows,
re-linking formulas, merges, data validations, and approval block.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPtt2MinYXH5T7wMFXyfVt
</commit_message>
<xml_diff>
--- a/out/BRING_주간_황우중_2026-W30.xlsx
+++ b/out/BRING_주간_황우중_2026-W30.xlsx
@@ -1544,7 +1544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:K47"/>
+  <dimension ref="B1:K52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="24.7109375" customWidth="1" style="49" min="2" max="2"/>
@@ -1694,8 +1694,8 @@
       <c r="C8" s="70" t="inlineStr">
         <is>
           <t>TRL 1 연구개발보고서에서 대표가 제1장(기술개발 방향·연구개발 목표)을 확정하였다. 제1장의 최상위 기준은 '노후 소형건축물 입구 1개소'를 초기 적용대상으로 하는 Scan-to-Fit 리트로핏 MVP이며, 표준 프레임+맞춤형 공차보정 연결부, 탈부착형 기능 카세트, BIM–BOM–제작도면 연계, 공장 사전제작·현장 건식설치, FM·Building Passport 연계를 핵심 축으로 한다.
-그러나 기존 TRL 1 작성 가이드(제2~11장)에는 방 1개·창호 1~2개 중심 MVP와 센서·창호 중심 표현이 다수 남아 있어, 제1장 확정 방향과 정합되지 않는다.
-따라서 이번 주에는 후속 작성의 1차로, 제1장 확정 MVP를 최상위 기준으로 제2장(문제 정의 및 기술 개념)을 전면 작성하고, 제3·4장 작성을 위한 연구가설·시스템 모듈·제품구조·필수 산출물 초안을 확보한다.</t>
+기존 TRL 1 작성 가이드(제2~11장)에는 방 1개·창호 1~2개 중심 MVP와 센서·창호 중심 표현이 다수 남아 있어 제1장 확정 방향과 정합되지 않는다.
+따라서 이번 주에는 후속 작성의 1차로, 제1장 확정 MVP를 최상위 기준으로 제2장(문제 정의 및 기술 개념)을 절 단위로 전면 작성하고, 제3·4장 작성을 위한 연구가설·시스템 모듈·제품구조·필수 산출물 초안을 확보한다.</t>
         </is>
       </c>
       <c r="D8" s="41" t="n"/>
@@ -1716,7 +1716,7 @@
       </c>
       <c r="C9" s="73" t="inlineStr">
         <is>
-          <t>제1장에서 확정된 입구 1개소 중심 Scan-to-Fit 리트로핏 MVP를 최상위 기준으로, TRL 1 보고서 제2장을 전면 작성하고 제3·4장 작성을 위한 연구가설·시스템 모듈·제품구조·산출물 초안을 확정한다.</t>
+          <t>제1장에서 확정된 입구 1개소 중심 Scan-to-Fit 리트로핏 MVP를 최상위 기준으로, TRL 1 보고서 제2장을 절 단위로 전면 작성하고 제3·4장 작성을 위한 연구가설·시스템 모듈·제품구조·산출물 초안을 확정한다.</t>
         </is>
       </c>
       <c r="D9" s="41" t="n"/>
@@ -1737,8 +1737,8 @@
       </c>
       <c r="C10" s="73" t="inlineStr">
         <is>
-          <t>제2장 문제정의·기술개념이 입구 MVP 기준으로 정합되지 않으면, 이후 전 장이 방·창호 중심 표현과 뒤섞여 연구개발보고서 전체 논리가 흔들린다.
-또한 문제·원인·기술논리·검증계획의 연결이 확보되지 않으면 TRL 2 개념검증 계획과 1:1 목업·시제품 일정이 연쇄적으로 지연되고, 후속 장의 재작성 부담이 발생한다.</t>
+          <t>제2장 문제정의·기술개념이 입구 MVP 기준으로 정합되지 않으면 이후 전 장이 방·창호 중심 표현과 뒤섞여 연구개발보고서 전체 논리가 흔들린다.
+또한 문제·원인·기술논리·검증계획의 연결이 확보되지 않으면 TRL 2 개념검증 계획과 1:1 목업·시제품 일정이 연쇄적으로 지연되고 후속 장의 재작성 부담이 발생한다.</t>
         </is>
       </c>
       <c r="D10" s="41" t="n"/>
@@ -1825,7 +1825,7 @@
       <c r="B16" s="112" t="n"/>
       <c r="C16" s="111" t="inlineStr">
         <is>
-          <t>제2장 5개 절(입구·공용부 구조 / 기존 공정 / 기존 기술 한계 / 핵심 문제 / 기술 개념) 전면 작성</t>
+          <t>제2장 5개 절을 절 단위로 각각 전면 작성</t>
         </is>
       </c>
       <c r="D16" s="41" t="n"/>
@@ -1873,7 +1873,7 @@
       <c r="B19" s="112" t="n"/>
       <c r="C19" s="113" t="inlineStr">
         <is>
-          <t>제4장 시스템 모듈(5~6개) 정의 및 제품구조·데이터 흐름 초안 작성</t>
+          <t>제4장 시스템 모듈(5~6개) 정의·구성방식 비교·제품구조·데이터 흐름 초안 작성</t>
         </is>
       </c>
       <c r="D19" s="41" t="n"/>
@@ -1889,7 +1889,7 @@
       <c r="B20" s="112" t="n"/>
       <c r="C20" s="111" t="inlineStr">
         <is>
-          <t>제2장 필수 산출물(표·그림) 및 미확인 가정·쟁점 정리</t>
+          <t>제2장 필수 산출물(표·그림) 및 미확인 가정·대표 검토 쟁점·용어/약어 정리</t>
         </is>
       </c>
       <c r="D20" s="41" t="n"/>
@@ -1949,9 +1949,10 @@
       <c r="C23" s="105" t="inlineStr">
         <is>
           <t>· 제1장(대표 확정)의 기술개발 방향·연구개발 목표를 최상위 기준으로 삼는다
-· TRL 1 수준을 유지한다: 문제 관찰·기술원리 정립·시스템 개념 정의·연구가설 설정·적용/제외조건·후보 성능지표·TRL 2 계획까지만 작성
+· TRL 1 수준 유지: 문제 관찰·기술원리 정립·시스템 개념 정의·연구가설 설정·적용/제외조건·후보 성능지표·TRL 2 계획까지만 작성
 · '성능 달성·스마트공장 구축·자동설계 완성·원가 절감 완료·센서만으로 원인 확정' 등 달성형 표현 금지
-· 첨부 작성 가이드는 참고자료이며, 입구 MVP와 상충하면 입구 MVP를 우선한다</t>
+· 서술은 □핵심주제/○세부주제/•현황·원인·기술필요성·대응방향·TRL1 정립사항 구조로 작성
+· 첨부 작성 가이드는 참고자료이며 입구 MVP와 상충 시 입구 MVP 우선</t>
         </is>
       </c>
       <c r="D23" s="41" t="n"/>
@@ -1975,7 +1976,7 @@
       </c>
       <c r="C24" s="102" t="inlineStr">
         <is>
-          <t>제1장 확정 MVP와 상충하거나 TRL 1 수준을 넘는 작성이 필요하다고 판단되면, 변경 사유·영향을 문서화하여 대표 승인 후 반영한다.</t>
+          <t>제1장 확정 MVP와 상충하거나 TRL 1 수준을 넘는 작성이 필요하다고 판단되면 변경 사유·영향을 문서화하여 대표 승인 후 반영한다.</t>
         </is>
       </c>
       <c r="D24" s="41" t="n"/>
@@ -2074,15 +2075,15 @@
       </c>
       <c r="D28" s="47" t="inlineStr">
         <is>
-          <t>기존 TRL 1 작성 가이드에 남아 있는 방·창호·외벽 중심 표현을 입구 1개소 MVP 기준으로 전수 식별·수정하고, 초기 MVP와 후속 확장범위를 명확히 구분한다.</t>
+          <t>기존 TRL 1 작성 가이드의 방·창호·외벽 중심 표현을 입구 1개소 MVP 기준으로 전수 식별·수정하고 초기 MVP와 후속 확장범위를 구분한다.</t>
         </is>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>① 가이드 내 방·창호·외벽 중심 표현의 위치를 전수 식별한 목록 작성
-② 각 표현을 입구 1개소 MVP 기준으로 수정한 대조표(기존→수정) 작성
-③ 초기 MVP / 후속 확장범위(센서·창호·외벽) 구분표 작성
-④ 기술 중심축 순서(현장·고객조사→입구 3D실측→As-is BIM→문제분석→To-be 기획→Scan-to-Fit→표준/맞춤 분리→BIM–BOM–제작도면→공장 사전제작→현장 건식설치→검증→FM/Building Passport)를 1개 흐름도로 고정</t>
+          <t>① 가이드 내 방·창호·외벽 중심 표현 위치 전수 식별 목록
+② 기존→수정 대조표(입구 1개소 MVP 기준)
+③ 초기 MVP / 후속 확장범위(센서·창호·외벽) 구분표
+④ 기술 중심축 순서(현장·고객조사→입구 3D실측→As-is BIM→문제분석→To-be 기획→Scan-to-Fit→표준/맞춤 분리→BIM–BOM–제작도면→공장 사전제작→현장 건식설치→검증→FM/Building Passport) 흐름도 1개</t>
         </is>
       </c>
       <c r="F28" s="47" t="inlineStr">
@@ -2097,7 +2098,7 @@
       </c>
       <c r="H28" s="107" t="inlineStr">
         <is>
-          <t>07-21(화) 18:00</t>
+          <t>07-21(화) 12:00</t>
         </is>
       </c>
       <c r="I28" s="47" t="inlineStr">
@@ -2106,10 +2107,10 @@
         </is>
       </c>
       <c r="J28" s="114" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="29" ht="123" customHeight="1" s="49">
@@ -2118,26 +2119,25 @@
       </c>
       <c r="C29" s="47" t="inlineStr">
         <is>
-          <t>제2장 문제 정의 및 기술 개념 전면 작성</t>
+          <t>제2장 1절 — 노후건축물 입구·공용부 구조 분석</t>
         </is>
       </c>
       <c r="D29" s="47" t="inlineStr">
         <is>
-          <t>제1장에서 선언한 기술개발 필요성을 입구 리트로핏 현장에서 실제로 발생하는 문제로 구체화하고, 왜 표준제품을 그대로 적용하기 어려운지를 구조적으로 설명한다.</t>
+          <t>노후 소형건축물 입구·공용부의 구조와 간섭요소를 분석하고, 왜 표준제품을 그대로 적용하기 어려운지를 구조적으로 설명한다.</t>
         </is>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>① 제1절 입구·공용부 구조 분석(구조·간섭요소·체결가능위치 및 표준제품 적용 곤란 근거)
-② 제2절 기존 공간기획·실측·제작·설치 공정의 비효율 분석표
-③ 제3절 기존 기술 8종 비교표(해결문제/강점/입구적용 한계/브링 보완방향)
-④ 제4절 핵심 문제문장 1개 확정 + 하위 7개 문제 분해도
-⑤ 제5절 기술 개념 흐름도 작성</t>
+          <t>① 입구 구성요소(벽체·바닥·천장·출입문·계단·캐노피·공용설비) 분류표
+② 벽면 요철·바닥 경사·단차·벽체 기울기 등 시공오차 요인 정리
+③ 배관·배선·계량기·실외기 등 간섭요소 및 구조체 체결 가능 위치 정리
+④ 표준제품 직접 적용이 어려운 근거를 구조적으로 서술 + 운반·반입·조립 영향 조건</t>
         </is>
       </c>
       <c r="F29" s="47" t="inlineStr">
         <is>
-          <t>02_황우중_제2장_문제정의_기술개념_W30_v1.pdf</t>
+          <t>02_황우중_2장1절_입구구조분석_W30_v1.pdf</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="H29" s="107" t="inlineStr">
         <is>
-          <t>07-23(목) 18:00</t>
+          <t>07-21(화) 18:00</t>
         </is>
       </c>
       <c r="I29" s="47" t="inlineStr">
@@ -2156,10 +2156,10 @@
         </is>
       </c>
       <c r="J29" s="114" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="30" ht="84" customHeight="1" s="49">
@@ -2168,231 +2168,408 @@
       </c>
       <c r="C30" s="47" t="inlineStr">
         <is>
-          <t>제3장 연구가설 및 개념검증 논리 초안</t>
+          <t>제2장 2절 — 기존 공간기획·실측·제작·설치 공정 분석</t>
         </is>
       </c>
       <c r="D30" s="47" t="inlineStr">
         <is>
-          <t>각 기술요소가 왜 필요한지 인과관계로 설명하고, 검증 가능한 연구가설로 전환한다.</t>
+          <t>기존 입구 개선공사 공정의 흐름과 비효율을 분석한다.</t>
         </is>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>① 최소 6개 연구가설 목록(실측·BIM 연계·표준/맞춤 분리·공장 사전조립·탈부착 카세트·Building Passport)
+          <t>① 현장방문→실측→공간기획→개별도면→재실측→주문제작→현장 절단·천공·용접→설치→재작업 공정 흐름도
+② 비효율 8항목(기획-제작 분리, 실측 누락·반복, 정보단절, 현장 추가가공, 업체 일정조정, 부품 재제작, 부분교체 곤란, 이력 미관리) 분석표
+③ 정보단절·재작업 발생 지점 표기</t>
+        </is>
+      </c>
+      <c r="F30" s="47" t="inlineStr">
+        <is>
+          <t>03_황우중_2장2절_공정비효율분석_W30_v1.pdf</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>브링 구글 드라이브</t>
+        </is>
+      </c>
+      <c r="H30" s="107" t="inlineStr">
+        <is>
+          <t>07-22(수) 18:00</t>
+        </is>
+      </c>
+      <c r="I30" s="47" t="inlineStr">
+        <is>
+          <t>높음</t>
+        </is>
+      </c>
+      <c r="J30" s="114" t="n">
+        <v>3</v>
+      </c>
+      <c r="K30" s="19" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="31" ht="90" customHeight="1" s="49">
+      <c r="B31" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C31" s="47" t="inlineStr">
+        <is>
+          <t>제2장 3절 — 기존 기술 8종 비교 및 한계</t>
+        </is>
+      </c>
+      <c r="D31" s="47" t="inlineStr">
+        <is>
+          <t>관련 기존 기술을 비교하여 입구 리트로핏 적용 시 한계와 브링 기술의 보완지점을 도출한다.</t>
+        </is>
+      </c>
+      <c r="E31" s="1" t="inlineStr">
+        <is>
+          <t>① 기존 기술 8종(현장 인테리어·리모델링/프리패브·OSC/모듈러 신축/Scan-to-BIM/파라메트릭 설계/3D프린팅/시설관리 앱/BIM·디지털트윈 FM) 비교표
+② 각 기술의 해결문제·강점·노후건축물 입구 적용 한계·브링 보완방향 작성</t>
+        </is>
+      </c>
+      <c r="F31" s="47" t="inlineStr">
+        <is>
+          <t>04_황우중_2장3절_기존기술비교_W30_v1.xlsx</t>
+        </is>
+      </c>
+      <c r="G31" s="108" t="inlineStr">
+        <is>
+          <t>브링 구글 드라이브</t>
+        </is>
+      </c>
+      <c r="H31" s="107" t="inlineStr">
+        <is>
+          <t>07-22(수) 18:00</t>
+        </is>
+      </c>
+      <c r="I31" s="47" t="inlineStr">
+        <is>
+          <t>높음</t>
+        </is>
+      </c>
+      <c r="J31" s="114" t="n">
+        <v>4</v>
+      </c>
+      <c r="K31" s="19" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="32" ht="69" customHeight="1" s="49">
+      <c r="B32" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="C32" s="47" t="inlineStr">
+        <is>
+          <t>제2장 4절 — 핵심 문제 정의 및 분해</t>
+        </is>
+      </c>
+      <c r="D32" s="47" t="inlineStr">
+        <is>
+          <t>보고서 전체의 핵심 문제를 한 문장으로 고정하고 하위 문제로 분해한다.</t>
+        </is>
+      </c>
+      <c r="E32" s="1" t="inlineStr">
+        <is>
+          <t>① 핵심 문제문장 1개 확정(형상 상이·시공오차·정보 분리·현장 맞춤가공·재작업 반복)
+② 하위 7개 문제(형상정보 부족/기획-제작 단절/현장 공차 대응 부족/표준·맞춤 구분 부재/공장 사전제작률 부족/탈부착·부분교체 부족/설치 후 이력관리 부족) 분해도
+③ 각 하위문제의 근거</t>
+        </is>
+      </c>
+      <c r="F32" s="47" t="inlineStr">
+        <is>
+          <t>05_황우중_2장4절_핵심문제정의_W30_v1.pdf</t>
+        </is>
+      </c>
+      <c r="G32" s="108" t="inlineStr">
+        <is>
+          <t>브링 구글 드라이브</t>
+        </is>
+      </c>
+      <c r="H32" s="107" t="inlineStr">
+        <is>
+          <t>07-22(수) 18:00</t>
+        </is>
+      </c>
+      <c r="I32" s="47" t="inlineStr">
+        <is>
+          <t>높음</t>
+        </is>
+      </c>
+      <c r="J32" s="114" t="n">
+        <v>3</v>
+      </c>
+      <c r="K32" s="19" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="33" ht="90" customHeight="1" s="49">
+      <c r="B33" s="17" t="n"/>
+      <c r="C33" s="47" t="inlineStr">
+        <is>
+          <t>제2장 5절 — 기술 개념 정의 및 흐름도</t>
+        </is>
+      </c>
+      <c r="D33" s="47" t="inlineStr">
+        <is>
+          <t>입구 리트로핏 기술흐름을 개념 수준에서 정의한다.</t>
+        </is>
+      </c>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>① 기술 개념 흐름도(입구 현장조사→형상·공차 실측→As-is BIM→공간·성능 문제 분석→To-be 공간기획→Scan-to-Fit 설계→표준 프레임 선정→맞춤 연결부 설계→기능 카세트 조합→BOM·제작도면→공장 사전제작·조립→현장 건식설치→품질·탈착 검증→FM/Building Passport 등록)
+② 각 단계 입력·출력 정의
+③ 초기 MVP·후속 확장범위 표</t>
+        </is>
+      </c>
+      <c r="F33" s="47" t="inlineStr">
+        <is>
+          <t>06_황우중_2장5절_기술개념흐름_W30_v1.pdf</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>브링 구글 드라이브</t>
+        </is>
+      </c>
+      <c r="H33" s="107" t="inlineStr">
+        <is>
+          <t>07-23(목) 18:00</t>
+        </is>
+      </c>
+      <c r="I33" s="47" t="inlineStr">
+        <is>
+          <t>높음</t>
+        </is>
+      </c>
+      <c r="J33" s="114" t="n">
+        <v>4</v>
+      </c>
+      <c r="K33" s="19" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="34" ht="90" customHeight="1" s="49">
+      <c r="B34" s="17" t="n"/>
+      <c r="C34" s="47" t="inlineStr">
+        <is>
+          <t>제3장 — 연구가설 및 개념검증 논리 초안</t>
+        </is>
+      </c>
+      <c r="D34" s="47" t="inlineStr">
+        <is>
+          <t>각 기술요소가 왜 필요한지 인과관계로 설명하고 검증 가능한 연구가설로 전환한다.</t>
+        </is>
+      </c>
+      <c r="E34" s="1" t="inlineStr">
+        <is>
+          <t>① 최소 6개 연구가설(디지털 실측/BIM 기반 기획-제작 연계/표준·맞춤 분리 반복성/공장 사전조립 작업·재작업 절감/탈부착 카세트 부분교체·기능추가/Building Passport 이력관리)
 ② 가설별 표: 연구가설 / 논리적 근거 / 확인해야 할 데이터 / TRL 2 검증방법 / 예상 산출물
 ③ 완전주문제작·완전표준화·혼합생산 비교표
 ④ 기술요소별 필요성 표</t>
         </is>
       </c>
-      <c r="F30" s="47" t="inlineStr">
-        <is>
-          <t>03_황우중_제3장_연구가설_검증초안_W30_v1.xlsx</t>
-        </is>
-      </c>
-      <c r="G30" s="6" t="inlineStr">
+      <c r="F34" s="47" t="inlineStr">
+        <is>
+          <t>07_황우중_3장_연구가설_검증초안_W30_v1.xlsx</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
         <is>
           <t>브링 구글 드라이브</t>
         </is>
       </c>
-      <c r="H30" s="107" t="inlineStr">
+      <c r="H34" s="107" t="inlineStr">
         <is>
           <t>07-23(목) 18:00</t>
         </is>
       </c>
-      <c r="I30" s="47" t="inlineStr">
+      <c r="I34" s="47" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
       </c>
-      <c r="J30" s="114" t="n">
-        <v>7</v>
-      </c>
-      <c r="K30" s="19" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="31" ht="90" customHeight="1" s="49">
-      <c r="B31" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="C31" s="47" t="inlineStr">
-        <is>
-          <t>제4장 시스템 구조 및 제품구조 초안</t>
-        </is>
-      </c>
-      <c r="D31" s="47" t="inlineStr">
-        <is>
-          <t>TRL 1 수준에서 시스템을 5~6개 모듈로 정리하고, 표준 프레임·맞춤 연결부·기능 카세트로 구성되는 혼합생산형 입구 리트로핏 구조를 개념안으로 도출한다.</t>
-        </is>
-      </c>
-      <c r="E31" s="1" t="inlineStr">
-        <is>
-          <t>① 5~6개 모듈 정의표(역할/입력/처리/출력/HW/SW/수행주체/초기MVP 포함여부/후속확장)
-② 구성방식 6후보 비교표(현장적합성·제작난이도·원가·표준화·운송·설치·탈착·확장성·스마트공장 연계 기준)
-③ 최적 구조 선정 근거표(혼합생산형 입구 리트로핏 — 단 TRL 2에서 변경 가능한 개념안으로 표기)
-④ 전체 시스템 구성도 + 데이터 흐름도 초안</t>
-        </is>
-      </c>
-      <c r="F31" s="47" t="inlineStr">
-        <is>
-          <t>04_황우중_제4장_시스템제품구조_초안_W30_v1.pdf</t>
-        </is>
-      </c>
-      <c r="G31" s="108" t="inlineStr">
+      <c r="J34" s="114" t="n">
+        <v>6</v>
+      </c>
+      <c r="K34" s="19" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="35" ht="90" customHeight="1" s="49">
+      <c r="B35" s="17" t="n"/>
+      <c r="C35" s="47" t="inlineStr">
+        <is>
+          <t>제4장 — 시스템 구조·구성방식·최적구조 초안</t>
+        </is>
+      </c>
+      <c r="D35" s="47" t="inlineStr">
+        <is>
+          <t>TRL 1 수준에서 시스템을 5~6개 모듈로 정리하고 혼합생산형 입구 리트로핏 구조를 개념안으로 도출한다.</t>
+        </is>
+      </c>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>① 모듈 5~6개 정의표(역할/입력/처리/출력/HW/SW/수행주체/초기MVP 포함여부/후속확장)
+② 구성방식 6후보 비교표(현장적합성·제작난이도·원가·표준화·운송·설치·탈착·확장성·스마트공장 연계)
+③ 최적 구조 선정 근거표(혼합생산형 입구 리트로핏 — TRL 2에서 변경 가능한 개념안으로 표기)
+④ 전체 시스템 구성도</t>
+        </is>
+      </c>
+      <c r="F35" s="47" t="inlineStr">
+        <is>
+          <t>08_황우중_4장_시스템구조_초안_W30_v1.pdf</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
         <is>
           <t>브링 구글 드라이브</t>
         </is>
       </c>
-      <c r="H31" s="107" t="inlineStr">
+      <c r="H35" s="107" t="inlineStr">
+        <is>
+          <t>07-24(금) 12:00</t>
+        </is>
+      </c>
+      <c r="I35" s="47" t="inlineStr">
+        <is>
+          <t>높음</t>
+        </is>
+      </c>
+      <c r="J35" s="114" t="n">
+        <v>6</v>
+      </c>
+      <c r="K35" s="19" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="36" ht="90" customHeight="1" s="49">
+      <c r="B36" s="17" t="n"/>
+      <c r="C36" s="47" t="inlineStr">
+        <is>
+          <t>제4장 — 제품구조·데이터 흐름 + 제2장 필수 산출물 패키지</t>
+        </is>
+      </c>
+      <c r="D36" s="47" t="inlineStr">
+        <is>
+          <t>제품 분해구조와 데이터 흐름을 초안화하고 제2장 필수 산출물을 완비한다.</t>
+        </is>
+      </c>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>① 제품 분해구조도(표준 프레임–맞춤 공차보정 연결부–탈부착 기능 카세트)
+② 데이터 흐름도(BIM–BOM–제작도면–부품 ID–품질검사–FM/Passport)
+③ 제2장 필수 산출물 6종 완비(입구 구조 분류표/기존 공정 비효율표/기존 기술 비교표/핵심 문제 분해도/기술개념 흐름도/초기 MVP·후속확장 표)</t>
+        </is>
+      </c>
+      <c r="F36" s="47" t="inlineStr">
+        <is>
+          <t>09_황우중_4장제품구조_2장산출물_W30_v1.pdf</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>브링 구글 드라이브</t>
+        </is>
+      </c>
+      <c r="H36" s="107" t="inlineStr">
         <is>
           <t>07-24(금) 15:00</t>
         </is>
       </c>
-      <c r="I31" s="47" t="inlineStr">
+      <c r="I36" s="47" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
       </c>
-      <c r="J31" s="114" t="n">
-        <v>8</v>
-      </c>
-      <c r="K31" s="19" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="32" ht="69" customHeight="1" s="49">
-      <c r="B32" s="17" t="n">
+      <c r="J36" s="114" t="n">
         <v>5</v>
       </c>
-      <c r="C32" s="47" t="inlineStr">
-        <is>
-          <t>제2장 필수 산출물 패키지 및 미확인 가정·쟁점 정리</t>
-        </is>
-      </c>
-      <c r="D32" s="47" t="inlineStr">
-        <is>
-          <t>제2장 필수 산출물을 완비하고, TRL 1 단계에서 확정되지 않은 가정과 대표 검토가 필요한 쟁점을 분리하여 정리한다.</t>
-        </is>
-      </c>
-      <c r="E32" s="1" t="inlineStr">
-        <is>
-          <t>① 제2장 필수 산출물 6종 완비(입구 구조 분류표 / 기존 공정 비효율표 / 기존 기술 비교표 / 핵심 문제 분해도 / 기술개념 흐름도 / 초기 MVP·후속확장 표)
-② 확인되지 않은 가정 목록
-③ 대표 검토가 필요한 쟁점 목록
-④ 용어정의·약어목록 초안</t>
-        </is>
-      </c>
-      <c r="F32" s="47" t="inlineStr">
-        <is>
-          <t>05_황우중_제2장산출물_쟁점정리_W30_v1.pdf</t>
-        </is>
-      </c>
-      <c r="G32" s="108" t="inlineStr">
+      <c r="K36" s="19" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="37" ht="90" customHeight="1" s="49">
+      <c r="B37" s="17" t="n"/>
+      <c r="C37" s="47" t="inlineStr">
+        <is>
+          <t>미확인 가정·대표 검토 쟁점·용어/약어 정리</t>
+        </is>
+      </c>
+      <c r="D37" s="47" t="inlineStr">
+        <is>
+          <t>TRL 1 단계에서 확정되지 않은 가정과 대표 검토가 필요한 쟁점을 분리하고 부속자료를 정리한다.</t>
+        </is>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>① 확인되지 않은 가정 목록
+② 대표 검토가 필요한 쟁점 목록
+③ 용어정의·약어목록 초안
+④ 참고문헌·근거자료 출처 목록</t>
+        </is>
+      </c>
+      <c r="F37" s="47" t="inlineStr">
+        <is>
+          <t>10_황우중_가정_쟁점_용어정리_W30_v1.pdf</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
         <is>
           <t>브링 구글 드라이브</t>
         </is>
       </c>
-      <c r="H32" s="107" t="inlineStr">
+      <c r="H37" s="107" t="inlineStr">
         <is>
           <t>07-24(금) 17:00</t>
         </is>
       </c>
-      <c r="I32" s="47" t="inlineStr">
+      <c r="I37" s="47" t="inlineStr">
         <is>
           <t>보통</t>
         </is>
       </c>
-      <c r="J32" s="114" t="n">
-        <v>4</v>
-      </c>
-      <c r="K32" s="19" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="33" ht="69" customHeight="1" s="49">
-      <c r="B33" s="45" t="inlineStr">
+      <c r="J37" s="114" t="n">
+        <v>3</v>
+      </c>
+      <c r="K37" s="19" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="38" ht="69" customHeight="1" s="49">
+      <c r="B38" s="45" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="C33" s="51" t="n"/>
-      <c r="D33" s="41" t="n"/>
-      <c r="E33" s="41" t="n"/>
-      <c r="F33" s="41" t="n"/>
-      <c r="G33" s="41" t="n"/>
-      <c r="H33" s="41" t="n"/>
-      <c r="I33" s="42" t="n"/>
-      <c r="J33" s="115">
-        <f>SUM(J28:J32)</f>
-        <v/>
-      </c>
-      <c r="K33" s="21">
-        <f>SUM(K28:K32)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" ht="24" customHeight="1" s="49">
-      <c r="B34" s="45" t="inlineStr">
-        <is>
-          <t>발행 검증</t>
-        </is>
-      </c>
-      <c r="C34" s="116">
-        <f>IF(COUNTA(C28:C32)=0,"업무 미입력",IF(COUNTA(E28:E32)&lt;COUNTA(C28:C32),"발행 불가 — 완료기준 누락 업무 있음",IF(COUNTA(F28:F32)&lt;COUNTA(C28:C32),"발행 불가 — 산출물 누락 업무 있음",IF(SUM(K28:K32)&lt;&gt;1,"발행 불가 — 가중치 합계 "&amp;TEXT(SUM(K28:K32),"0%")&amp;" (100% 필요)","발행 가능 — 완료기준·산출물·가중치 충족"))))</f>
-        <v/>
-      </c>
-      <c r="D34" s="41" t="n"/>
-      <c r="E34" s="41" t="n"/>
-      <c r="F34" s="41" t="n"/>
-      <c r="G34" s="41" t="n"/>
-      <c r="H34" s="41" t="n"/>
-      <c r="I34" s="41" t="n"/>
-      <c r="J34" s="41" t="n"/>
-      <c r="K34" s="42" t="n"/>
-    </row>
-    <row r="35" ht="24" customHeight="1" s="49"/>
-    <row r="36" ht="24" customHeight="1" s="49"/>
-    <row r="37" ht="18" customHeight="1" s="49">
-      <c r="B37" s="89" t="inlineStr">
-        <is>
-          <t>담당자 접수확인  —  월요일 12:00까지 담당자 직접 작성 (미작성 = 업무 미이해로 간주, 재지시)</t>
-        </is>
-      </c>
-      <c r="C37" s="64" t="n"/>
-      <c r="D37" s="64" t="n"/>
-      <c r="E37" s="64" t="n"/>
-      <c r="F37" s="64" t="n"/>
-      <c r="G37" s="64" t="n"/>
-      <c r="H37" s="64" t="n"/>
-      <c r="I37" s="64" t="n"/>
-      <c r="J37" s="64" t="n"/>
-      <c r="K37" s="64" t="n"/>
-    </row>
-    <row r="38" ht="36" customHeight="1" s="49">
-      <c r="B38" s="45" t="inlineStr">
-        <is>
-          <t>내가 이해한 업무
-(본인 언어로 재작성)</t>
-        </is>
-      </c>
-      <c r="C38" s="117" t="n"/>
+      <c r="C38" s="51" t="n"/>
       <c r="D38" s="41" t="n"/>
       <c r="E38" s="41" t="n"/>
       <c r="F38" s="41" t="n"/>
       <c r="G38" s="41" t="n"/>
       <c r="H38" s="41" t="n"/>
-      <c r="I38" s="41" t="n"/>
-      <c r="J38" s="41" t="n"/>
-      <c r="K38" s="42" t="n"/>
-    </row>
-    <row r="39" ht="19.5" customHeight="1" s="49">
+      <c r="I38" s="42" t="n"/>
+      <c r="J38" s="115">
+        <f>SUM(J28:J37)</f>
+        <v/>
+      </c>
+      <c r="K38" s="21">
+        <f>SUM(K28:K37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="24" customHeight="1" s="49">
       <c r="B39" s="45" t="inlineStr">
         <is>
-          <t>완료기준 재확인
-(무엇이 되면 끝인가)</t>
-        </is>
-      </c>
-      <c r="C39" s="118" t="n"/>
+          <t>발행 검증</t>
+        </is>
+      </c>
+      <c r="C39" s="116">
+        <f>IF(COUNTA(C28:C37)=0,"업무 미입력",IF(COUNTA(E28:E37)&lt;COUNTA(C28:C37),"발행 불가 — 완료기준 누락 업무 있음",IF(COUNTA(F28:F37)&lt;COUNTA(C28:C37),"발행 불가 — 산출물 누락 업무 있음",IF(SUM(K28:K37)&lt;&gt;1,"발행 불가 — 가중치 합계 "&amp;TEXT(SUM(K28:K37),"0%")&amp;" (100% 필요)","발행 가능 — 완료기준·산출물·가중치 충족"))))</f>
+        <v/>
+      </c>
       <c r="D39" s="41" t="n"/>
       <c r="E39" s="41" t="n"/>
       <c r="F39" s="41" t="n"/>
@@ -2403,61 +2580,37 @@
       <c r="K39" s="42" t="n"/>
     </row>
     <row r="40" ht="24" customHeight="1" s="49">
-      <c r="B40" s="45" t="inlineStr">
-        <is>
-          <t>예상 리스크
-(막힐 것 같은 지점)</t>
-        </is>
-      </c>
+      <c r="B40" s="45" t="n"/>
       <c r="C40" s="43" t="n"/>
-      <c r="D40" s="41" t="n"/>
-      <c r="E40" s="41" t="n"/>
-      <c r="F40" s="41" t="n"/>
-      <c r="G40" s="41" t="n"/>
-      <c r="H40" s="41" t="n"/>
-      <c r="I40" s="41" t="n"/>
-      <c r="J40" s="41" t="n"/>
-      <c r="K40" s="42" t="n"/>
     </row>
     <row r="41" ht="24" customHeight="1" s="49">
-      <c r="B41" s="45" t="inlineStr">
-        <is>
-          <t>필요한 지원·의사결정</t>
-        </is>
-      </c>
+      <c r="B41" s="45" t="n"/>
       <c r="C41" s="43" t="n"/>
-      <c r="D41" s="41" t="n"/>
-      <c r="E41" s="41" t="n"/>
-      <c r="F41" s="41" t="n"/>
-      <c r="G41" s="41" t="n"/>
-      <c r="H41" s="41" t="n"/>
-      <c r="I41" s="41" t="n"/>
-      <c r="J41" s="41" t="n"/>
-      <c r="K41" s="42" t="n"/>
-    </row>
-    <row r="42" ht="24" customHeight="1" s="49">
-      <c r="B42" s="45" t="inlineStr">
-        <is>
-          <t>실행 계획 (요일 배분)</t>
-        </is>
-      </c>
-      <c r="C42" s="43" t="n"/>
-      <c r="D42" s="41" t="n"/>
-      <c r="E42" s="41" t="n"/>
-      <c r="F42" s="41" t="n"/>
-      <c r="G42" s="41" t="n"/>
-      <c r="H42" s="41" t="n"/>
-      <c r="I42" s="41" t="n"/>
-      <c r="J42" s="41" t="n"/>
-      <c r="K42" s="42" t="n"/>
-    </row>
-    <row r="43" ht="24" customHeight="1" s="49">
+    </row>
+    <row r="42" ht="18" customHeight="1" s="49">
+      <c r="B42" s="89" t="inlineStr">
+        <is>
+          <t>담당자 접수확인  —  월요일 12:00까지 담당자 직접 작성 (미작성 = 업무 미이해로 간주, 재지시)</t>
+        </is>
+      </c>
+      <c r="C42" s="64" t="n"/>
+      <c r="D42" s="64" t="n"/>
+      <c r="E42" s="64" t="n"/>
+      <c r="F42" s="64" t="n"/>
+      <c r="G42" s="64" t="n"/>
+      <c r="H42" s="64" t="n"/>
+      <c r="I42" s="64" t="n"/>
+      <c r="J42" s="64" t="n"/>
+      <c r="K42" s="64" t="n"/>
+    </row>
+    <row r="43" ht="36" customHeight="1" s="49">
       <c r="B43" s="45" t="inlineStr">
         <is>
-          <t>접수 확인 일시 / 서명</t>
-        </is>
-      </c>
-      <c r="C43" s="47" t="n"/>
+          <t>내가 이해한 업무
+(본인 언어로 재작성)</t>
+        </is>
+      </c>
+      <c r="C43" s="117" t="n"/>
       <c r="D43" s="41" t="n"/>
       <c r="E43" s="41" t="n"/>
       <c r="F43" s="41" t="n"/>
@@ -2467,14 +2620,31 @@
       <c r="J43" s="41" t="n"/>
       <c r="K43" s="42" t="n"/>
     </row>
-    <row r="44" ht="24" customHeight="1" s="49"/>
+    <row r="44" ht="19.5" customHeight="1" s="49">
+      <c r="B44" s="45" t="inlineStr">
+        <is>
+          <t>완료기준 재확인
+(무엇이 되면 끝인가)</t>
+        </is>
+      </c>
+      <c r="C44" s="118" t="n"/>
+      <c r="D44" s="41" t="n"/>
+      <c r="E44" s="41" t="n"/>
+      <c r="F44" s="41" t="n"/>
+      <c r="G44" s="41" t="n"/>
+      <c r="H44" s="41" t="n"/>
+      <c r="I44" s="41" t="n"/>
+      <c r="J44" s="41" t="n"/>
+      <c r="K44" s="42" t="n"/>
+    </row>
     <row r="45" ht="24" customHeight="1" s="49">
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>결   재</t>
-        </is>
-      </c>
-      <c r="C45" s="41" t="n"/>
+      <c r="B45" s="45" t="inlineStr">
+        <is>
+          <t>예상 리스크
+(막힐 것 같은 지점)</t>
+        </is>
+      </c>
+      <c r="C45" s="43" t="n"/>
       <c r="D45" s="41" t="n"/>
       <c r="E45" s="41" t="n"/>
       <c r="F45" s="41" t="n"/>
@@ -2487,80 +2657,140 @@
     <row r="46" ht="24" customHeight="1" s="49">
       <c r="B46" s="45" t="inlineStr">
         <is>
+          <t>필요한 지원·의사결정</t>
+        </is>
+      </c>
+      <c r="C46" s="43" t="n"/>
+      <c r="D46" s="41" t="n"/>
+      <c r="E46" s="41" t="n"/>
+      <c r="F46" s="41" t="n"/>
+      <c r="G46" s="41" t="n"/>
+      <c r="H46" s="41" t="n"/>
+      <c r="I46" s="41" t="n"/>
+      <c r="J46" s="41" t="n"/>
+      <c r="K46" s="42" t="n"/>
+    </row>
+    <row r="47" ht="24" customHeight="1" s="49">
+      <c r="B47" s="45" t="inlineStr">
+        <is>
+          <t>실행 계획 (요일 배분)</t>
+        </is>
+      </c>
+      <c r="C47" s="43" t="n"/>
+      <c r="D47" s="41" t="n"/>
+      <c r="E47" s="41" t="n"/>
+      <c r="F47" s="41" t="n"/>
+      <c r="G47" s="41" t="n"/>
+      <c r="H47" s="41" t="n"/>
+      <c r="I47" s="41" t="n"/>
+      <c r="J47" s="41" t="n"/>
+      <c r="K47" s="42" t="n"/>
+    </row>
+    <row r="48" ht="24" customHeight="1" s="49">
+      <c r="B48" s="45" t="inlineStr">
+        <is>
+          <t>접수 확인 일시 / 서명</t>
+        </is>
+      </c>
+      <c r="C48" s="47" t="n"/>
+      <c r="D48" s="41" t="n"/>
+      <c r="E48" s="41" t="n"/>
+      <c r="F48" s="41" t="n"/>
+      <c r="G48" s="41" t="n"/>
+      <c r="H48" s="41" t="n"/>
+      <c r="I48" s="41" t="n"/>
+      <c r="J48" s="41" t="n"/>
+      <c r="K48" s="42" t="n"/>
+    </row>
+    <row r="49" ht="24" customHeight="1" s="49"/>
+    <row r="50" ht="24" customHeight="1" s="49">
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>결   재</t>
+        </is>
+      </c>
+      <c r="C50" s="41" t="n"/>
+      <c r="D50" s="41" t="n"/>
+      <c r="E50" s="41" t="n"/>
+      <c r="F50" s="41" t="n"/>
+      <c r="G50" s="41" t="n"/>
+      <c r="H50" s="41" t="n"/>
+      <c r="I50" s="41" t="n"/>
+      <c r="J50" s="41" t="n"/>
+      <c r="K50" s="42" t="n"/>
+    </row>
+    <row r="51" ht="24" customHeight="1" s="49">
+      <c r="B51" s="45" t="inlineStr">
+        <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="C46" s="45" t="inlineStr">
+      <c r="C51" s="45" t="inlineStr">
         <is>
           <t>작성 (지시자)</t>
         </is>
       </c>
-      <c r="D46" s="42" t="n"/>
-      <c r="E46" s="45" t="inlineStr">
+      <c r="D51" s="42" t="n"/>
+      <c r="E51" s="45" t="inlineStr">
         <is>
           <t>검토 (검수자)</t>
         </is>
       </c>
-      <c r="F46" s="42" t="n"/>
-      <c r="G46" s="45" t="inlineStr">
+      <c r="F51" s="42" t="n"/>
+      <c r="G51" s="45" t="inlineStr">
         <is>
           <t>승인 (대표)</t>
         </is>
       </c>
-      <c r="H46" s="42" t="n"/>
-      <c r="I46" s="45" t="inlineStr">
+      <c r="H51" s="42" t="n"/>
+      <c r="I51" s="45" t="inlineStr">
         <is>
           <t>접수 (담당자)</t>
         </is>
       </c>
-      <c r="J46" s="42" t="n"/>
-      <c r="K46" s="45" t="inlineStr">
+      <c r="J51" s="42" t="n"/>
+      <c r="K51" s="45" t="inlineStr">
         <is>
           <t>일자</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="B47" s="45" t="inlineStr">
+    <row r="52" ht="21.75" customHeight="1" s="49">
+      <c r="B52" s="45" t="inlineStr">
         <is>
           <t>서명</t>
         </is>
       </c>
-      <c r="C47" s="47" t="inlineStr">
+      <c r="C52" s="47" t="inlineStr">
         <is>
           <t>서 창 환</t>
         </is>
       </c>
-      <c r="D47" s="42" t="n"/>
-      <c r="E47" s="47" t="inlineStr">
+      <c r="D52" s="42" t="n"/>
+      <c r="E52" s="47" t="inlineStr">
         <is>
           <t>서 창 환</t>
         </is>
       </c>
-      <c r="F47" s="42" t="n"/>
-      <c r="G47" s="47" t="inlineStr">
+      <c r="F52" s="42" t="n"/>
+      <c r="G52" s="47" t="inlineStr">
         <is>
           <t>서 창 환</t>
         </is>
       </c>
-      <c r="H47" s="42" t="n"/>
-      <c r="I47" s="47" t="inlineStr">
+      <c r="H52" s="42" t="n"/>
+      <c r="I52" s="47" t="inlineStr">
         <is>
           <t>황 우 중</t>
         </is>
       </c>
-      <c r="J47" s="42" t="n"/>
-      <c r="K47" s="109" t="inlineStr">
+      <c r="J52" s="42" t="n"/>
+      <c r="K52" s="109" t="inlineStr">
         <is>
           <t>2026-07-20</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="19.5" customHeight="1" s="49"/>
-    <row r="49" ht="21.75" customHeight="1" s="49"/>
-    <row r="50" ht="21.75" customHeight="1" s="49"/>
-    <row r="51" ht="21.75" customHeight="1" s="49"/>
-    <row r="52" ht="21.75" customHeight="1" s="49"/>
     <row r="53" ht="21.75" customHeight="1" s="49"/>
     <row r="54" ht="21.75" customHeight="1" s="49"/>
     <row r="55" ht="21.75" customHeight="1" s="49"/>
@@ -2577,50 +2807,49 @@
     <row r="68" ht="39.75" customHeight="1" s="49"/>
   </sheetData>
   <mergeCells count="39">
+    <mergeCell ref="C47:K47"/>
+    <mergeCell ref="G52:H52"/>
     <mergeCell ref="C10:K10"/>
-    <mergeCell ref="C41:K41"/>
     <mergeCell ref="C15:J15"/>
-    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="C44:K44"/>
     <mergeCell ref="C24:J24"/>
-    <mergeCell ref="C40:K40"/>
     <mergeCell ref="C9:K9"/>
     <mergeCell ref="C14:J14"/>
+    <mergeCell ref="C38:I38"/>
+    <mergeCell ref="E52:F52"/>
     <mergeCell ref="C43:K43"/>
-    <mergeCell ref="B45:K45"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="I47:J47"/>
+    <mergeCell ref="C46:K46"/>
+    <mergeCell ref="E51:F51"/>
+    <mergeCell ref="B50:K50"/>
     <mergeCell ref="C20:J20"/>
     <mergeCell ref="B26:K26"/>
     <mergeCell ref="C16:J16"/>
+    <mergeCell ref="C48:K48"/>
     <mergeCell ref="B7:K7"/>
     <mergeCell ref="C39:K39"/>
+    <mergeCell ref="C22:J22"/>
     <mergeCell ref="C8:K8"/>
-    <mergeCell ref="C22:J22"/>
-    <mergeCell ref="C33:I33"/>
     <mergeCell ref="B14:B21"/>
-    <mergeCell ref="C38:K38"/>
-    <mergeCell ref="C46:D46"/>
     <mergeCell ref="C21:J21"/>
-    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="C51:D51"/>
     <mergeCell ref="B12:K12"/>
+    <mergeCell ref="C52:D52"/>
+    <mergeCell ref="I52:J52"/>
     <mergeCell ref="B2:K2"/>
-    <mergeCell ref="C34:K34"/>
+    <mergeCell ref="B42:K42"/>
     <mergeCell ref="C23:J23"/>
     <mergeCell ref="C17:J17"/>
+    <mergeCell ref="G51:H51"/>
+    <mergeCell ref="I51:J51"/>
     <mergeCell ref="B1:K1"/>
-    <mergeCell ref="G47:H47"/>
-    <mergeCell ref="C42:K42"/>
-    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="C45:K45"/>
+    <mergeCell ref="C13:J13"/>
     <mergeCell ref="C19:J19"/>
-    <mergeCell ref="C13:J13"/>
     <mergeCell ref="C18:J18"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="B37:K37"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I28:I32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I28:I37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"높음,보통,낮음"</formula1>
-      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2634,7 +2863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C1:L47"/>
+  <dimension ref="C1:L52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="19.85546875" customWidth="1" style="49" min="3" max="3"/>
@@ -2715,7 +2944,7 @@
         </is>
       </c>
       <c r="D5" s="26">
-        <f>SUMPRODUCT(F12:F16,H12:H16)</f>
+        <f>SUMPRODUCT(F12:F21,H12:H21)</f>
         <v/>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -2733,7 +2962,7 @@
         </is>
       </c>
       <c r="H5" s="119">
-        <f>SUM('01_업무지시서'!J28:J32)</f>
+        <f>SUM('01_업무지시서'!J28:J37)</f>
         <v/>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -2742,7 +2971,7 @@
         </is>
       </c>
       <c r="J5" s="119">
-        <f>SUM(I12:I16)</f>
+        <f>SUM(I12:I21)</f>
         <v/>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -3024,157 +3253,202 @@
       <c r="K16" s="47" t="n"/>
       <c r="L16" s="47" t="n"/>
     </row>
-    <row r="17" ht="15" customHeight="1" s="49">
-      <c r="C17" s="45" t="inlineStr">
+    <row r="17" ht="27.75" customHeight="1" s="49">
+      <c r="C17" s="17" t="n"/>
+      <c r="D17" s="40">
+        <f>IF('01_업무지시서'!C33="","",'01_업무지시서'!C33)</f>
+        <v/>
+      </c>
+      <c r="E17" s="40">
+        <f>IF('01_업무지시서'!E33="","",'01_업무지시서'!E33)</f>
+        <v/>
+      </c>
+      <c r="F17" s="11">
+        <f>IF('01_업무지시서'!K33="",0,'01_업무지시서'!K33)</f>
+        <v/>
+      </c>
+      <c r="G17" s="47" t="n"/>
+      <c r="H17" s="19" t="n"/>
+      <c r="I17" s="114" t="n"/>
+      <c r="J17" s="47" t="n"/>
+      <c r="K17" s="47" t="n"/>
+      <c r="L17" s="47" t="n"/>
+    </row>
+    <row r="18" ht="27.75" customHeight="1" s="49">
+      <c r="C18" s="17" t="n"/>
+      <c r="D18" s="40">
+        <f>IF('01_업무지시서'!C34="","",'01_업무지시서'!C34)</f>
+        <v/>
+      </c>
+      <c r="E18" s="40">
+        <f>IF('01_업무지시서'!E34="","",'01_업무지시서'!E34)</f>
+        <v/>
+      </c>
+      <c r="F18" s="11">
+        <f>IF('01_업무지시서'!K34="",0,'01_업무지시서'!K34)</f>
+        <v/>
+      </c>
+      <c r="G18" s="47" t="n"/>
+      <c r="H18" s="19" t="n"/>
+      <c r="I18" s="114" t="n"/>
+      <c r="J18" s="47" t="n"/>
+      <c r="K18" s="47" t="n"/>
+      <c r="L18" s="47" t="n"/>
+    </row>
+    <row r="19" ht="27.75" customHeight="1" s="49">
+      <c r="C19" s="17" t="n"/>
+      <c r="D19" s="40">
+        <f>IF('01_업무지시서'!C35="","",'01_업무지시서'!C35)</f>
+        <v/>
+      </c>
+      <c r="E19" s="40">
+        <f>IF('01_업무지시서'!E35="","",'01_업무지시서'!E35)</f>
+        <v/>
+      </c>
+      <c r="F19" s="11">
+        <f>IF('01_업무지시서'!K35="",0,'01_업무지시서'!K35)</f>
+        <v/>
+      </c>
+      <c r="G19" s="47" t="n"/>
+      <c r="H19" s="19" t="n"/>
+      <c r="I19" s="114" t="n"/>
+      <c r="J19" s="47" t="n"/>
+      <c r="K19" s="47" t="n"/>
+      <c r="L19" s="47" t="n"/>
+    </row>
+    <row r="20" ht="27.75" customHeight="1" s="49">
+      <c r="C20" s="17" t="n"/>
+      <c r="D20" s="40">
+        <f>IF('01_업무지시서'!C36="","",'01_업무지시서'!C36)</f>
+        <v/>
+      </c>
+      <c r="E20" s="40">
+        <f>IF('01_업무지시서'!E36="","",'01_업무지시서'!E36)</f>
+        <v/>
+      </c>
+      <c r="F20" s="11">
+        <f>IF('01_업무지시서'!K36="",0,'01_업무지시서'!K36)</f>
+        <v/>
+      </c>
+      <c r="G20" s="47" t="n"/>
+      <c r="H20" s="19" t="n"/>
+      <c r="I20" s="114" t="n"/>
+      <c r="J20" s="47" t="n"/>
+      <c r="K20" s="47" t="n"/>
+      <c r="L20" s="47" t="n"/>
+    </row>
+    <row r="21" ht="27.75" customHeight="1" s="49">
+      <c r="C21" s="17" t="n"/>
+      <c r="D21" s="40">
+        <f>IF('01_업무지시서'!C37="","",'01_업무지시서'!C37)</f>
+        <v/>
+      </c>
+      <c r="E21" s="40">
+        <f>IF('01_업무지시서'!E37="","",'01_업무지시서'!E37)</f>
+        <v/>
+      </c>
+      <c r="F21" s="11">
+        <f>IF('01_업무지시서'!K37="",0,'01_업무지시서'!K37)</f>
+        <v/>
+      </c>
+      <c r="G21" s="47" t="n"/>
+      <c r="H21" s="19" t="n"/>
+      <c r="I21" s="114" t="n"/>
+      <c r="J21" s="47" t="n"/>
+      <c r="K21" s="47" t="n"/>
+      <c r="L21" s="47" t="n"/>
+    </row>
+    <row r="22" ht="15" customHeight="1" s="49">
+      <c r="C22" s="45" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="D17" s="45" t="inlineStr">
+      <c r="D22" s="45" t="inlineStr">
         <is>
           <t>가중 달성률 →</t>
         </is>
       </c>
-      <c r="E17" s="42" t="n"/>
-      <c r="F17" s="21">
-        <f>SUM(F12:F16)</f>
-        <v/>
-      </c>
-      <c r="G17" s="28">
-        <f>SUMPRODUCT(F12:F16,H12:H16)</f>
-        <v/>
-      </c>
-      <c r="H17" s="29">
-        <f>COUNTIF(G12:G16,"완료")</f>
-        <v/>
-      </c>
-      <c r="I17" s="115">
-        <f>SUM(I12:I16)</f>
-        <v/>
-      </c>
-      <c r="J17" s="69">
-        <f>"완료 "&amp;COUNTIF(G12:G16,"완료")&amp;"건 / 진행중 "&amp;COUNTIF(G12:G16,"진행중")&amp;"건 / 미착수 "&amp;COUNTIF(G12:G16,"미착수")&amp;"건"</f>
-        <v/>
-      </c>
-      <c r="K17" s="41" t="n"/>
-      <c r="L17" s="42" t="n"/>
-    </row>
-    <row r="18" ht="24" customHeight="1" s="49">
-      <c r="C18" s="46" t="n"/>
-      <c r="D18" s="46" t="n"/>
-      <c r="I18" s="46" t="n"/>
-      <c r="J18" s="46" t="n"/>
-      <c r="L18" s="46" t="n"/>
-    </row>
-    <row r="19" ht="19.5" customHeight="1" s="49">
-      <c r="C19" s="121" t="inlineStr">
+      <c r="E22" s="42" t="n"/>
+      <c r="F22" s="21">
+        <f>SUM(F12:F21)</f>
+        <v/>
+      </c>
+      <c r="G22" s="28">
+        <f>SUMPRODUCT(F12:F21,H12:H21)</f>
+        <v/>
+      </c>
+      <c r="H22" s="29">
+        <f>COUNTIF(G12:G21,"완료")</f>
+        <v/>
+      </c>
+      <c r="I22" s="115">
+        <f>SUM(I12:I21)</f>
+        <v/>
+      </c>
+      <c r="J22" s="69">
+        <f>"완료 "&amp;COUNTIF(G12:G21,"완료")&amp;"건 / 진행중 "&amp;COUNTIF(G12:G21,"진행중")&amp;"건 / 미착수 "&amp;COUNTIF(G12:G21,"미착수")&amp;"건"</f>
+        <v/>
+      </c>
+      <c r="K22" s="41" t="n"/>
+      <c r="L22" s="42" t="n"/>
+    </row>
+    <row r="23" ht="24" customHeight="1" s="49">
+      <c r="C23" s="46" t="n"/>
+      <c r="D23" s="46" t="n"/>
+      <c r="I23" s="46" t="n"/>
+      <c r="J23" s="46" t="n"/>
+      <c r="L23" s="46" t="n"/>
+    </row>
+    <row r="24" ht="19.5" customHeight="1" s="49">
+      <c r="C24" s="121" t="inlineStr">
         <is>
           <t>2. 자가 검수  —  제출 전 §4 검수기준으로 본인이 먼저 점검</t>
         </is>
       </c>
-      <c r="D19" s="64" t="n"/>
-      <c r="E19" s="64" t="n"/>
-      <c r="F19" s="64" t="n"/>
-      <c r="G19" s="64" t="n"/>
-      <c r="H19" s="64" t="n"/>
-      <c r="I19" s="64" t="n"/>
-      <c r="J19" s="64" t="n"/>
-      <c r="K19" s="64" t="n"/>
-      <c r="L19" s="65" t="n"/>
-    </row>
-    <row r="20" ht="24" customHeight="1" s="49">
-      <c r="C20" s="46" t="inlineStr">
+      <c r="D24" s="64" t="n"/>
+      <c r="E24" s="64" t="n"/>
+      <c r="F24" s="64" t="n"/>
+      <c r="G24" s="64" t="n"/>
+      <c r="H24" s="64" t="n"/>
+      <c r="I24" s="64" t="n"/>
+      <c r="J24" s="64" t="n"/>
+      <c r="K24" s="64" t="n"/>
+      <c r="L24" s="65" t="n"/>
+    </row>
+    <row r="25" ht="24" customHeight="1" s="49">
+      <c r="C25" s="46" t="inlineStr">
         <is>
           <t>검수 항목 (자동)</t>
         </is>
       </c>
-      <c r="D20" s="46" t="inlineStr">
+      <c r="D25" s="46" t="inlineStr">
         <is>
           <t>검수 질문 (자동)</t>
         </is>
       </c>
-      <c r="E20" s="41" t="n"/>
-      <c r="F20" s="41" t="n"/>
-      <c r="G20" s="41" t="n"/>
-      <c r="H20" s="42" t="n"/>
-      <c r="I20" s="46" t="inlineStr">
-        <is>
-          <t>자가
-판정</t>
-        </is>
-      </c>
-      <c r="J20" s="46" t="inlineStr">
-        <is>
-          <t>미충족 사유·보완 계획</t>
-        </is>
-      </c>
-      <c r="K20" s="42" t="n"/>
-      <c r="L20" s="46" t="inlineStr">
-        <is>
-          <t>검수자
-판정</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="24" customHeight="1" s="49">
-      <c r="C21" s="69" t="n"/>
-      <c r="D21" s="55" t="n"/>
-      <c r="E21" s="41" t="n"/>
-      <c r="F21" s="41" t="n"/>
-      <c r="G21" s="41" t="n"/>
-      <c r="H21" s="42" t="n"/>
-      <c r="I21" s="47" t="n"/>
-      <c r="J21" s="44" t="n"/>
-      <c r="K21" s="42" t="n"/>
-      <c r="L21" s="66" t="n"/>
-    </row>
-    <row r="22" ht="24" customHeight="1" s="49">
-      <c r="C22" s="69" t="n"/>
-      <c r="D22" s="55" t="n"/>
-      <c r="E22" s="41" t="n"/>
-      <c r="F22" s="41" t="n"/>
-      <c r="G22" s="41" t="n"/>
-      <c r="H22" s="42" t="n"/>
-      <c r="I22" s="47" t="n"/>
-      <c r="J22" s="44" t="n"/>
-      <c r="K22" s="42" t="n"/>
-      <c r="L22" s="66" t="n"/>
-    </row>
-    <row r="23" ht="24" customHeight="1" s="49">
-      <c r="C23" s="69" t="n"/>
-      <c r="D23" s="55" t="n"/>
-      <c r="E23" s="41" t="n"/>
-      <c r="F23" s="41" t="n"/>
-      <c r="G23" s="41" t="n"/>
-      <c r="H23" s="42" t="n"/>
-      <c r="I23" s="47" t="n"/>
-      <c r="J23" s="44" t="n"/>
-      <c r="K23" s="42" t="n"/>
-      <c r="L23" s="66" t="n"/>
-    </row>
-    <row r="24" ht="24" customHeight="1" s="49">
-      <c r="C24" s="69" t="n"/>
-      <c r="D24" s="55" t="n"/>
-      <c r="E24" s="41" t="n"/>
-      <c r="F24" s="41" t="n"/>
-      <c r="G24" s="41" t="n"/>
-      <c r="H24" s="42" t="n"/>
-      <c r="I24" s="47" t="n"/>
-      <c r="J24" s="44" t="n"/>
-      <c r="K24" s="42" t="n"/>
-      <c r="L24" s="66" t="n"/>
-    </row>
-    <row r="25" ht="24" customHeight="1" s="49">
-      <c r="C25" s="69" t="n"/>
-      <c r="D25" s="55" t="n"/>
       <c r="E25" s="41" t="n"/>
       <c r="F25" s="41" t="n"/>
       <c r="G25" s="41" t="n"/>
       <c r="H25" s="42" t="n"/>
-      <c r="I25" s="47" t="n"/>
-      <c r="J25" s="44" t="n"/>
+      <c r="I25" s="46" t="inlineStr">
+        <is>
+          <t>자가
+판정</t>
+        </is>
+      </c>
+      <c r="J25" s="46" t="inlineStr">
+        <is>
+          <t>미충족 사유·보완 계획</t>
+        </is>
+      </c>
       <c r="K25" s="42" t="n"/>
-      <c r="L25" s="66" t="n"/>
+      <c r="L25" s="46" t="inlineStr">
+        <is>
+          <t>검수자
+판정</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="24" customHeight="1" s="49">
       <c r="C26" s="69" t="n"/>
@@ -3200,410 +3474,470 @@
       <c r="K27" s="42" t="n"/>
       <c r="L27" s="66" t="n"/>
     </row>
-    <row r="28" ht="27.75" customHeight="1" s="49">
-      <c r="C28" s="46" t="n"/>
-      <c r="D28" s="46" t="n"/>
-      <c r="E28" s="46" t="n"/>
-      <c r="F28" s="46" t="n"/>
-      <c r="G28" s="46" t="n"/>
-      <c r="H28" s="46" t="n"/>
-      <c r="I28" s="46" t="n"/>
-      <c r="J28" s="46" t="n"/>
-      <c r="K28" s="46" t="n"/>
-      <c r="L28" s="46" t="n"/>
-    </row>
-    <row r="29" ht="19.5" customHeight="1" s="49">
-      <c r="C29" s="121" t="inlineStr">
+    <row r="28" ht="24" customHeight="1" s="49">
+      <c r="C28" s="69" t="n"/>
+      <c r="D28" s="55" t="n"/>
+      <c r="E28" s="41" t="n"/>
+      <c r="F28" s="41" t="n"/>
+      <c r="G28" s="41" t="n"/>
+      <c r="H28" s="42" t="n"/>
+      <c r="I28" s="47" t="n"/>
+      <c r="J28" s="44" t="n"/>
+      <c r="K28" s="42" t="n"/>
+      <c r="L28" s="66" t="n"/>
+    </row>
+    <row r="29" ht="24" customHeight="1" s="49">
+      <c r="C29" s="69" t="n"/>
+      <c r="D29" s="55" t="n"/>
+      <c r="E29" s="41" t="n"/>
+      <c r="F29" s="41" t="n"/>
+      <c r="G29" s="41" t="n"/>
+      <c r="H29" s="42" t="n"/>
+      <c r="I29" s="47" t="n"/>
+      <c r="J29" s="44" t="n"/>
+      <c r="K29" s="42" t="n"/>
+      <c r="L29" s="66" t="n"/>
+    </row>
+    <row r="30" ht="24" customHeight="1" s="49">
+      <c r="C30" s="69" t="n"/>
+      <c r="D30" s="55" t="n"/>
+      <c r="E30" s="41" t="n"/>
+      <c r="F30" s="41" t="n"/>
+      <c r="G30" s="41" t="n"/>
+      <c r="H30" s="42" t="n"/>
+      <c r="I30" s="47" t="n"/>
+      <c r="J30" s="44" t="n"/>
+      <c r="K30" s="42" t="n"/>
+      <c r="L30" s="66" t="n"/>
+    </row>
+    <row r="31" ht="24" customHeight="1" s="49">
+      <c r="C31" s="69" t="n"/>
+      <c r="D31" s="55" t="n"/>
+      <c r="E31" s="41" t="n"/>
+      <c r="F31" s="41" t="n"/>
+      <c r="G31" s="41" t="n"/>
+      <c r="H31" s="42" t="n"/>
+      <c r="I31" s="47" t="n"/>
+      <c r="J31" s="44" t="n"/>
+      <c r="K31" s="42" t="n"/>
+      <c r="L31" s="66" t="n"/>
+    </row>
+    <row r="32" ht="24" customHeight="1" s="49">
+      <c r="C32" s="69" t="n"/>
+      <c r="D32" s="55" t="n"/>
+      <c r="E32" s="41" t="n"/>
+      <c r="F32" s="41" t="n"/>
+      <c r="G32" s="41" t="n"/>
+      <c r="H32" s="42" t="n"/>
+      <c r="I32" s="47" t="n"/>
+      <c r="J32" s="44" t="n"/>
+      <c r="K32" s="42" t="n"/>
+      <c r="L32" s="66" t="n"/>
+    </row>
+    <row r="33" ht="27.75" customHeight="1" s="49">
+      <c r="C33" s="46" t="n"/>
+      <c r="D33" s="46" t="n"/>
+      <c r="E33" s="46" t="n"/>
+      <c r="F33" s="46" t="n"/>
+      <c r="G33" s="46" t="n"/>
+      <c r="H33" s="46" t="n"/>
+      <c r="I33" s="46" t="n"/>
+      <c r="J33" s="46" t="n"/>
+      <c r="K33" s="46" t="n"/>
+      <c r="L33" s="46" t="n"/>
+    </row>
+    <row r="34" ht="19.5" customHeight="1" s="49">
+      <c r="C34" s="121" t="inlineStr">
         <is>
           <t>3. 이슈 및 지원요청  —  대안 없이 문제만 올리는 보고는 반려</t>
         </is>
       </c>
-      <c r="D29" s="64" t="n"/>
-      <c r="E29" s="64" t="n"/>
-      <c r="F29" s="64" t="n"/>
-      <c r="G29" s="64" t="n"/>
-      <c r="H29" s="64" t="n"/>
-      <c r="I29" s="64" t="n"/>
-      <c r="J29" s="64" t="n"/>
-      <c r="K29" s="64" t="n"/>
-      <c r="L29" s="65" t="n"/>
-    </row>
-    <row r="30" ht="27.75" customHeight="1" s="49">
-      <c r="C30" s="46" t="inlineStr">
+      <c r="D34" s="64" t="n"/>
+      <c r="E34" s="64" t="n"/>
+      <c r="F34" s="64" t="n"/>
+      <c r="G34" s="64" t="n"/>
+      <c r="H34" s="64" t="n"/>
+      <c r="I34" s="64" t="n"/>
+      <c r="J34" s="64" t="n"/>
+      <c r="K34" s="64" t="n"/>
+      <c r="L34" s="65" t="n"/>
+    </row>
+    <row r="35" ht="27.75" customHeight="1" s="49">
+      <c r="C35" s="46" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="D30" s="46" t="inlineStr">
+      <c r="D35" s="46" t="inlineStr">
         <is>
           <t>이슈 내용</t>
         </is>
       </c>
-      <c r="E30" s="46" t="inlineStr">
+      <c r="E35" s="46" t="inlineStr">
         <is>
           <t>영향
 (일정/비용/품질)</t>
         </is>
       </c>
-      <c r="F30" s="46" t="inlineStr">
+      <c r="F35" s="46" t="inlineStr">
         <is>
           <t>근본 원인</t>
         </is>
       </c>
-      <c r="G30" s="46" t="inlineStr">
+      <c r="G35" s="46" t="inlineStr">
         <is>
           <t>대안 1</t>
         </is>
       </c>
-      <c r="H30" s="46" t="inlineStr">
+      <c r="H35" s="46" t="inlineStr">
         <is>
           <t>대안 2</t>
         </is>
       </c>
-      <c r="I30" s="46" t="inlineStr">
+      <c r="I35" s="46" t="inlineStr">
         <is>
           <t>권고안</t>
         </is>
       </c>
-      <c r="J30" s="46" t="inlineStr">
+      <c r="J35" s="46" t="inlineStr">
         <is>
           <t>요청사항</t>
         </is>
       </c>
-      <c r="K30" s="46" t="inlineStr">
+      <c r="K35" s="46" t="inlineStr">
         <is>
           <t>결정기한</t>
         </is>
       </c>
-      <c r="L30" s="46" t="inlineStr">
+      <c r="L35" s="46" t="inlineStr">
         <is>
           <t>대표 결정</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="36" customHeight="1" s="49">
-      <c r="C31" s="6" t="n"/>
-      <c r="D31" s="18" t="n"/>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="18" t="n"/>
-      <c r="G31" s="18" t="n"/>
-      <c r="H31" s="18" t="n"/>
-      <c r="I31" s="18" t="n"/>
-      <c r="J31" s="18" t="n"/>
-      <c r="K31" s="6" t="n"/>
-      <c r="L31" s="66" t="n"/>
-    </row>
-    <row r="32" ht="36" customHeight="1" s="49">
-      <c r="C32" s="6" t="n"/>
-      <c r="D32" s="18" t="n"/>
-      <c r="E32" s="6" t="n"/>
-      <c r="F32" s="18" t="n"/>
-      <c r="G32" s="18" t="n"/>
-      <c r="H32" s="18" t="n"/>
-      <c r="I32" s="18" t="n"/>
-      <c r="J32" s="18" t="n"/>
-      <c r="K32" s="6" t="n"/>
-      <c r="L32" s="66" t="n"/>
-    </row>
-    <row r="33" ht="36" customHeight="1" s="49">
-      <c r="C33" s="6" t="n"/>
-      <c r="D33" s="18" t="n"/>
-      <c r="E33" s="6" t="n"/>
-      <c r="F33" s="18" t="n"/>
-      <c r="G33" s="18" t="n"/>
-      <c r="H33" s="18" t="n"/>
-      <c r="I33" s="18" t="n"/>
-      <c r="J33" s="18" t="n"/>
-      <c r="K33" s="6" t="n"/>
-      <c r="L33" s="66" t="n"/>
-    </row>
-    <row r="34" ht="27.75" customHeight="1" s="49">
-      <c r="C34" s="13" t="n"/>
-      <c r="D34" s="46" t="n"/>
-      <c r="E34" s="46" t="n"/>
-      <c r="F34" s="46" t="n"/>
-      <c r="G34" s="46" t="n"/>
-      <c r="H34" s="46" t="n"/>
-      <c r="I34" s="46" t="n"/>
-      <c r="J34" s="46" t="n"/>
-      <c r="K34" s="46" t="n"/>
-      <c r="L34" s="46" t="n"/>
-    </row>
-    <row r="35" ht="19.5" customHeight="1" s="49">
-      <c r="C35" s="121" t="inlineStr">
+    <row r="36" ht="36" customHeight="1" s="49">
+      <c r="C36" s="6" t="n"/>
+      <c r="D36" s="18" t="n"/>
+      <c r="E36" s="6" t="n"/>
+      <c r="F36" s="18" t="n"/>
+      <c r="G36" s="18" t="n"/>
+      <c r="H36" s="18" t="n"/>
+      <c r="I36" s="18" t="n"/>
+      <c r="J36" s="18" t="n"/>
+      <c r="K36" s="6" t="n"/>
+      <c r="L36" s="66" t="n"/>
+    </row>
+    <row r="37" ht="36" customHeight="1" s="49">
+      <c r="C37" s="6" t="n"/>
+      <c r="D37" s="18" t="n"/>
+      <c r="E37" s="6" t="n"/>
+      <c r="F37" s="18" t="n"/>
+      <c r="G37" s="18" t="n"/>
+      <c r="H37" s="18" t="n"/>
+      <c r="I37" s="18" t="n"/>
+      <c r="J37" s="18" t="n"/>
+      <c r="K37" s="6" t="n"/>
+      <c r="L37" s="66" t="n"/>
+    </row>
+    <row r="38" ht="36" customHeight="1" s="49">
+      <c r="C38" s="6" t="n"/>
+      <c r="D38" s="18" t="n"/>
+      <c r="E38" s="6" t="n"/>
+      <c r="F38" s="18" t="n"/>
+      <c r="G38" s="18" t="n"/>
+      <c r="H38" s="18" t="n"/>
+      <c r="I38" s="18" t="n"/>
+      <c r="J38" s="18" t="n"/>
+      <c r="K38" s="6" t="n"/>
+      <c r="L38" s="66" t="n"/>
+    </row>
+    <row r="39" ht="27.75" customHeight="1" s="49">
+      <c r="C39" s="13" t="n"/>
+      <c r="D39" s="46" t="n"/>
+      <c r="E39" s="46" t="n"/>
+      <c r="F39" s="46" t="n"/>
+      <c r="G39" s="46" t="n"/>
+      <c r="H39" s="46" t="n"/>
+      <c r="I39" s="46" t="n"/>
+      <c r="J39" s="46" t="n"/>
+      <c r="K39" s="46" t="n"/>
+      <c r="L39" s="46" t="n"/>
+    </row>
+    <row r="40" ht="19.5" customHeight="1" s="49">
+      <c r="C40" s="121" t="inlineStr">
         <is>
           <t>4. 다음 주 제안 업무  —  지시를 기다리지 말 것. 본인이 먼저 제안.</t>
         </is>
       </c>
-      <c r="D35" s="64" t="n"/>
-      <c r="E35" s="64" t="n"/>
-      <c r="F35" s="64" t="n"/>
-      <c r="G35" s="64" t="n"/>
-      <c r="H35" s="64" t="n"/>
-      <c r="I35" s="64" t="n"/>
-      <c r="J35" s="64" t="n"/>
-      <c r="K35" s="64" t="n"/>
-      <c r="L35" s="65" t="n"/>
-    </row>
-    <row r="36" ht="27.75" customHeight="1" s="49">
-      <c r="C36" s="13" t="inlineStr">
+      <c r="D40" s="64" t="n"/>
+      <c r="E40" s="64" t="n"/>
+      <c r="F40" s="64" t="n"/>
+      <c r="G40" s="64" t="n"/>
+      <c r="H40" s="64" t="n"/>
+      <c r="I40" s="64" t="n"/>
+      <c r="J40" s="64" t="n"/>
+      <c r="K40" s="64" t="n"/>
+      <c r="L40" s="65" t="n"/>
+    </row>
+    <row r="41" ht="27.75" customHeight="1" s="49">
+      <c r="C41" s="13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D36" s="46" t="inlineStr">
+      <c r="D41" s="46" t="inlineStr">
         <is>
           <t>제안 업무</t>
         </is>
       </c>
-      <c r="E36" s="46" t="inlineStr">
+      <c r="E41" s="46" t="inlineStr">
         <is>
           <t>왜 해야 하는가</t>
         </is>
       </c>
-      <c r="F36" s="46" t="inlineStr">
+      <c r="F41" s="46" t="inlineStr">
         <is>
           <t>완료기준(안)</t>
         </is>
       </c>
-      <c r="G36" s="46" t="inlineStr">
+      <c r="G41" s="46" t="inlineStr">
         <is>
           <t>예상
 소요(h)</t>
         </is>
       </c>
-      <c r="H36" s="46" t="inlineStr">
+      <c r="H41" s="46" t="inlineStr">
         <is>
           <t>우선순위(안)</t>
         </is>
       </c>
-      <c r="I36" s="46" t="inlineStr">
+      <c r="I41" s="46" t="inlineStr">
         <is>
           <t>선행 조건</t>
         </is>
       </c>
-      <c r="J36" s="46" t="inlineStr">
+      <c r="J41" s="46" t="inlineStr">
         <is>
           <t>필요 지원</t>
         </is>
       </c>
-      <c r="K36" s="46" t="inlineStr">
+      <c r="K41" s="46" t="inlineStr">
         <is>
           <t>대표 승인</t>
         </is>
       </c>
-      <c r="L36" s="46" t="inlineStr">
+      <c r="L41" s="46" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="31.5" customHeight="1" s="49">
-      <c r="C37" s="22" t="n">
+    <row r="42" ht="31.5" customHeight="1" s="49">
+      <c r="C42" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="D37" s="18" t="n"/>
-      <c r="E37" s="18" t="n"/>
-      <c r="F37" s="18" t="n"/>
-      <c r="G37" s="114" t="n"/>
-      <c r="H37" s="6" t="n"/>
-      <c r="I37" s="18" t="n"/>
-      <c r="J37" s="18" t="n"/>
-      <c r="K37" s="66" t="n"/>
-      <c r="L37" s="6" t="n"/>
-    </row>
-    <row r="38" ht="31.5" customHeight="1" s="49">
-      <c r="C38" s="22" t="n">
+      <c r="D42" s="18" t="n"/>
+      <c r="E42" s="18" t="n"/>
+      <c r="F42" s="18" t="n"/>
+      <c r="G42" s="114" t="n"/>
+      <c r="H42" s="6" t="n"/>
+      <c r="I42" s="18" t="n"/>
+      <c r="J42" s="18" t="n"/>
+      <c r="K42" s="66" t="n"/>
+      <c r="L42" s="6" t="n"/>
+    </row>
+    <row r="43" ht="31.5" customHeight="1" s="49">
+      <c r="C43" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="D38" s="18" t="n"/>
-      <c r="E38" s="18" t="n"/>
-      <c r="F38" s="18" t="n"/>
-      <c r="G38" s="114" t="n"/>
-      <c r="H38" s="6" t="n"/>
-      <c r="I38" s="18" t="n"/>
-      <c r="J38" s="18" t="n"/>
-      <c r="K38" s="66" t="n"/>
-      <c r="L38" s="6" t="n"/>
-    </row>
-    <row r="39" ht="31.5" customHeight="1" s="49">
-      <c r="C39" s="22" t="n">
+      <c r="D43" s="18" t="n"/>
+      <c r="E43" s="18" t="n"/>
+      <c r="F43" s="18" t="n"/>
+      <c r="G43" s="114" t="n"/>
+      <c r="H43" s="6" t="n"/>
+      <c r="I43" s="18" t="n"/>
+      <c r="J43" s="18" t="n"/>
+      <c r="K43" s="66" t="n"/>
+      <c r="L43" s="6" t="n"/>
+    </row>
+    <row r="44" ht="31.5" customHeight="1" s="49">
+      <c r="C44" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="D39" s="18" t="n"/>
-      <c r="E39" s="18" t="n"/>
-      <c r="F39" s="18" t="n"/>
-      <c r="G39" s="114" t="n"/>
-      <c r="H39" s="6" t="n"/>
-      <c r="I39" s="18" t="n"/>
-      <c r="J39" s="18" t="n"/>
-      <c r="K39" s="66" t="n"/>
-      <c r="L39" s="6" t="n"/>
-    </row>
-    <row r="40" ht="31.5" customHeight="1" s="49">
-      <c r="C40" s="22" t="n">
+      <c r="D44" s="18" t="n"/>
+      <c r="E44" s="18" t="n"/>
+      <c r="F44" s="18" t="n"/>
+      <c r="G44" s="114" t="n"/>
+      <c r="H44" s="6" t="n"/>
+      <c r="I44" s="18" t="n"/>
+      <c r="J44" s="18" t="n"/>
+      <c r="K44" s="66" t="n"/>
+      <c r="L44" s="6" t="n"/>
+    </row>
+    <row r="45" ht="31.5" customHeight="1" s="49">
+      <c r="C45" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="D40" s="18" t="n"/>
-      <c r="E40" s="18" t="n"/>
-      <c r="F40" s="18" t="n"/>
-      <c r="G40" s="114" t="n"/>
-      <c r="H40" s="6" t="n"/>
-      <c r="I40" s="18" t="n"/>
-      <c r="J40" s="18" t="n"/>
-      <c r="K40" s="66" t="n"/>
-      <c r="L40" s="6" t="n"/>
-    </row>
-    <row r="41" ht="25.5" customHeight="1" s="49">
-      <c r="C41" s="45" t="n"/>
-      <c r="D41" s="43" t="n"/>
-      <c r="J41" s="58" t="n"/>
-    </row>
-    <row r="42" ht="19.5" customHeight="1" s="49">
-      <c r="C42" s="48" t="inlineStr">
+      <c r="D45" s="18" t="n"/>
+      <c r="E45" s="18" t="n"/>
+      <c r="F45" s="18" t="n"/>
+      <c r="G45" s="114" t="n"/>
+      <c r="H45" s="6" t="n"/>
+      <c r="I45" s="18" t="n"/>
+      <c r="J45" s="18" t="n"/>
+      <c r="K45" s="66" t="n"/>
+      <c r="L45" s="6" t="n"/>
+    </row>
+    <row r="46" ht="25.5" customHeight="1" s="49">
+      <c r="C46" s="45" t="n"/>
+      <c r="D46" s="43" t="n"/>
+      <c r="J46" s="58" t="n"/>
+    </row>
+    <row r="47" ht="19.5" customHeight="1" s="49">
+      <c r="C47" s="48" t="inlineStr">
         <is>
           <t>5. 자기점검 및 대표 검수</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="25.5" customHeight="1" s="49">
-      <c r="C43" s="45" t="inlineStr">
+    <row r="48" ht="25.5" customHeight="1" s="49">
+      <c r="C48" s="45" t="inlineStr">
         <is>
           <t>이번 주 가장 잘한 것</t>
         </is>
       </c>
-      <c r="D43" s="43" t="inlineStr">
+      <c r="D48" s="43" t="inlineStr">
         <is>
           <t>결과로 증명되는 것 1개만</t>
         </is>
       </c>
-      <c r="E43" s="41" t="n"/>
-      <c r="F43" s="41" t="n"/>
-      <c r="G43" s="41" t="n"/>
-      <c r="H43" s="41" t="n"/>
-      <c r="I43" s="42" t="n"/>
-      <c r="J43" s="58" t="inlineStr">
+      <c r="E48" s="41" t="n"/>
+      <c r="F48" s="41" t="n"/>
+      <c r="G48" s="41" t="n"/>
+      <c r="H48" s="41" t="n"/>
+      <c r="I48" s="42" t="n"/>
+      <c r="J48" s="58" t="inlineStr">
         <is>
           <t>[대표 검수 의견]</t>
         </is>
       </c>
-      <c r="K43" s="59" t="n"/>
-      <c r="L43" s="60" t="n"/>
-    </row>
-    <row r="44" ht="25.5" customHeight="1" s="49">
-      <c r="C44" s="45" t="inlineStr">
+      <c r="K48" s="59" t="n"/>
+      <c r="L48" s="60" t="n"/>
+    </row>
+    <row r="49" ht="25.5" customHeight="1" s="49">
+      <c r="C49" s="45" t="inlineStr">
         <is>
           <t>이번 주 가장 부족한 것</t>
         </is>
       </c>
-      <c r="D44" s="43" t="inlineStr">
+      <c r="D49" s="43" t="inlineStr">
         <is>
           <t>변명 말고 사실만</t>
         </is>
       </c>
-      <c r="E44" s="41" t="n"/>
-      <c r="F44" s="41" t="n"/>
-      <c r="G44" s="41" t="n"/>
-      <c r="H44" s="41" t="n"/>
-      <c r="I44" s="42" t="n"/>
-      <c r="J44" s="61" t="n"/>
-      <c r="L44" s="62" t="n"/>
-    </row>
-    <row r="45" ht="25.5" customHeight="1" s="49">
-      <c r="C45" s="45" t="inlineStr">
+      <c r="E49" s="41" t="n"/>
+      <c r="F49" s="41" t="n"/>
+      <c r="G49" s="41" t="n"/>
+      <c r="H49" s="41" t="n"/>
+      <c r="I49" s="42" t="n"/>
+      <c r="J49" s="61" t="n"/>
+      <c r="L49" s="62" t="n"/>
+    </row>
+    <row r="50" ht="25.5" customHeight="1" s="49">
+      <c r="C50" s="45" t="inlineStr">
         <is>
           <t>다음 주 개선 액션 1개</t>
         </is>
       </c>
-      <c r="D45" s="43" t="inlineStr">
+      <c r="D50" s="43" t="inlineStr">
         <is>
           <t>실행 가능한 행동으로</t>
         </is>
       </c>
-      <c r="E45" s="41" t="n"/>
-      <c r="F45" s="41" t="n"/>
-      <c r="G45" s="41" t="n"/>
-      <c r="H45" s="41" t="n"/>
-      <c r="I45" s="42" t="n"/>
-      <c r="J45" s="63" t="n"/>
-      <c r="K45" s="64" t="n"/>
-      <c r="L45" s="65" t="n"/>
-    </row>
-    <row r="47" ht="33.75" customHeight="1" s="49">
-      <c r="C47" s="45" t="inlineStr">
+      <c r="E50" s="41" t="n"/>
+      <c r="F50" s="41" t="n"/>
+      <c r="G50" s="41" t="n"/>
+      <c r="H50" s="41" t="n"/>
+      <c r="I50" s="42" t="n"/>
+      <c r="J50" s="63" t="n"/>
+      <c r="K50" s="64" t="n"/>
+      <c r="L50" s="65" t="n"/>
+    </row>
+    <row r="52" ht="33.75" customHeight="1" s="49">
+      <c r="C52" s="45" t="inlineStr">
         <is>
           <t>제출자</t>
         </is>
       </c>
-      <c r="D47" s="47" t="n"/>
-      <c r="E47" s="41" t="n"/>
-      <c r="F47" s="42" t="n"/>
-      <c r="G47" s="45" t="inlineStr">
+      <c r="D52" s="47" t="n"/>
+      <c r="E52" s="41" t="n"/>
+      <c r="F52" s="42" t="n"/>
+      <c r="G52" s="45" t="inlineStr">
         <is>
           <t>검수자</t>
         </is>
       </c>
-      <c r="H47" s="66" t="n"/>
-      <c r="I47" s="42" t="n"/>
-      <c r="J47" s="45" t="inlineStr">
+      <c r="H52" s="66" t="n"/>
+      <c r="I52" s="42" t="n"/>
+      <c r="J52" s="45" t="inlineStr">
         <is>
           <t>최종 판정</t>
         </is>
       </c>
-      <c r="K47" s="56" t="n"/>
-      <c r="L47" s="42" t="n"/>
+      <c r="K52" s="56" t="n"/>
+      <c r="L52" s="42" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D47:F47"/>
+    <mergeCell ref="D49:I49"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="D48:I48"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="D31:H31"/>
     <mergeCell ref="D7:L7"/>
-    <mergeCell ref="D43:I43"/>
-    <mergeCell ref="C19:L19"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="K47:L47"/>
-    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J22:L22"/>
     <mergeCell ref="D27:H27"/>
+    <mergeCell ref="C34:L34"/>
     <mergeCell ref="J27:K27"/>
-    <mergeCell ref="C42:L42"/>
-    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="C24:L24"/>
+    <mergeCell ref="H52:I52"/>
     <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="K52:L52"/>
+    <mergeCell ref="J32:K32"/>
     <mergeCell ref="J25:K25"/>
-    <mergeCell ref="C29:L29"/>
-    <mergeCell ref="C35:L35"/>
-    <mergeCell ref="J43:L45"/>
-    <mergeCell ref="J17:L17"/>
-    <mergeCell ref="D44:I44"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="H47:I47"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D50:I50"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="C47:L47"/>
+    <mergeCell ref="J48:L50"/>
     <mergeCell ref="C1:L1"/>
-    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="D30:H30"/>
     <mergeCell ref="D25:H25"/>
+    <mergeCell ref="C40:L40"/>
     <mergeCell ref="C9:L9"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D45:I45"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D52:F52"/>
     <mergeCell ref="C2:L2"/>
     <mergeCell ref="D6:L6"/>
     <mergeCell ref="D26:H26"/>
   </mergeCells>
   <dataValidations count="5">
-    <dataValidation sqref="I21:I27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I26:I32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"충족,미충족"</formula1>
     </dataValidation>
-    <dataValidation sqref="L21:L27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L26:L32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"합격,보완,불합격"</formula1>
     </dataValidation>
-    <dataValidation sqref="K37:K40 L31:L33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K42:K45 L36:L38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"승인,보류,반려"</formula1>
     </dataValidation>
-    <dataValidation sqref="K47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"합격,조건부합격,보완요청,불합격"</formula1>
     </dataValidation>
-    <dataValidation sqref="G12:G16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G12:G21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"완료,진행중,미착수,보류,취소"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Reframe 황우중 W30 as 7 action-oriented work orders
Replace chapter/section-style task titles with imperative work
instructions; consolidate to 7 tasks (5→7 rows) with report sheet,
sums, validations, and approval block re-aligned.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPtt2MinYXH5T7wMFXyfVt
</commit_message>
<xml_diff>
--- a/out/BRING_주간_황우중_2026-W30.xlsx
+++ b/out/BRING_주간_황우중_2026-W30.xlsx
@@ -1544,7 +1544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:K52"/>
+  <dimension ref="B1:K49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="24.7109375" customWidth="1" style="49" min="2" max="2"/>
@@ -1693,9 +1693,8 @@
       </c>
       <c r="C8" s="70" t="inlineStr">
         <is>
-          <t>TRL 1 연구개발보고서에서 대표가 제1장(기술개발 방향·연구개발 목표)을 확정하였다. 제1장의 최상위 기준은 '노후 소형건축물 입구 1개소'를 초기 적용대상으로 하는 Scan-to-Fit 리트로핏 MVP이며, 표준 프레임+맞춤형 공차보정 연결부, 탈부착형 기능 카세트, BIM–BOM–제작도면 연계, 공장 사전제작·현장 건식설치, FM·Building Passport 연계를 핵심 축으로 한다.
-기존 TRL 1 작성 가이드(제2~11장)에는 방 1개·창호 1~2개 중심 MVP와 센서·창호 중심 표현이 다수 남아 있어 제1장 확정 방향과 정합되지 않는다.
-따라서 이번 주에는 후속 작성의 1차로, 제1장 확정 MVP를 최상위 기준으로 제2장(문제 정의 및 기술 개념)을 절 단위로 전면 작성하고, 제3·4장 작성을 위한 연구가설·시스템 모듈·제품구조·필수 산출물 초안을 확보한다.</t>
+          <t>TRL 1 연구개발보고서에서 대표가 제1장(기술개발 방향·연구개발 목표)을 확정하였다. 최상위 기준은 '노후 소형건축물 입구 1개소'를 초기 적용대상으로 하는 Scan-to-Fit 리트로핏 MVP이며, 표준 프레임+맞춤형 공차보정 연결부, 탈부착형 기능 카세트, BIM–BOM–제작도면 연계, 공장 사전제작·현장 건식설치, FM·Building Passport 연계를 핵심 축으로 한다.
+기존 작성 가이드에는 방 1개·창호 1~2개 중심 MVP와 센서·창호 중심 표현이 다수 남아 있어 제1장 확정 방향과 정합되지 않는다. 이번 주에는 후속 작성의 1차로, 제1장 확정 MVP를 기준으로 보고서 본문(문제정의~시스템·제품구조)을 구체화한다.</t>
         </is>
       </c>
       <c r="D8" s="41" t="n"/>
@@ -1716,7 +1715,7 @@
       </c>
       <c r="C9" s="73" t="inlineStr">
         <is>
-          <t>제1장에서 확정된 입구 1개소 중심 Scan-to-Fit 리트로핏 MVP를 최상위 기준으로, TRL 1 보고서 제2장을 절 단위로 전면 작성하고 제3·4장 작성을 위한 연구가설·시스템 모듈·제품구조·산출물 초안을 확정한다.</t>
+          <t>제1장에서 확정된 입구 1개소 중심 Scan-to-Fit 리트로핏 MVP를 기준으로, 연구개발보고서 본문(문제정의·기술개념·연구가설·시스템/제품 구조)을 검증 가능한 연구논리로 구체화한다.</t>
         </is>
       </c>
       <c r="D9" s="41" t="n"/>
@@ -1737,8 +1736,7 @@
       </c>
       <c r="C10" s="73" t="inlineStr">
         <is>
-          <t>제2장 문제정의·기술개념이 입구 MVP 기준으로 정합되지 않으면 이후 전 장이 방·창호 중심 표현과 뒤섞여 연구개발보고서 전체 논리가 흔들린다.
-또한 문제·원인·기술논리·검증계획의 연결이 확보되지 않으면 TRL 2 개념검증 계획과 1:1 목업·시제품 일정이 연쇄적으로 지연되고 후속 장의 재작성 부담이 발생한다.</t>
+          <t>입구 MVP 기준으로 정합되지 않으면 이후 전 장이 방·창호 중심 표현과 뒤섞여 보고서 전체 논리가 흔들린다. 문제·원인·기술논리·검증계획의 연결이 확보되지 않으면 TRL 2 개념검증 계획과 1:1 목업·시제품 일정이 연쇄 지연되고 재작성 부담이 발생한다.</t>
         </is>
       </c>
       <c r="D10" s="41" t="n"/>
@@ -1789,7 +1787,7 @@
       </c>
       <c r="C14" s="111" t="inlineStr">
         <is>
-          <t>제1장 확정 MVP(입구 1개소·Scan-to-Fit·표준 프레임+맞춤 공차보정 연결부·탈부착 기능 카세트·BIM–BOM–제작도면 연계·공장 사전제작·현장 건식설치·FM/Building Passport) 기준 정합</t>
+          <t>제1장 확정 MVP(입구 1개소·Scan-to-Fit·표준 프레임+맞춤 공차보정 연결부·탈부착 기능 카세트·BIM–BOM–제작도면·공장 사전제작·현장 건식설치·FM/Building Passport) 기준 정합</t>
         </is>
       </c>
       <c r="D14" s="41" t="n"/>
@@ -1825,7 +1823,7 @@
       <c r="B16" s="112" t="n"/>
       <c r="C16" s="111" t="inlineStr">
         <is>
-          <t>제2장 5개 절을 절 단위로 각각 전면 작성</t>
+          <t>입구 현장 문제·기존 공정 비효율·기존 기술 한계 분석 및 핵심 문제 정의</t>
         </is>
       </c>
       <c r="D16" s="41" t="n"/>
@@ -1841,7 +1839,7 @@
       <c r="B17" s="112" t="n"/>
       <c r="C17" s="111" t="inlineStr">
         <is>
-          <t>핵심 문제문장 1개 확정 및 하위 문제 분해</t>
+          <t>입구 리트로핏 기술개념·전체 흐름 정립</t>
         </is>
       </c>
       <c r="D17" s="41" t="n"/>
@@ -1857,7 +1855,7 @@
       <c r="B18" s="112" t="n"/>
       <c r="C18" s="111" t="inlineStr">
         <is>
-          <t>제3장 연구가설 목록 및 검증방법 초안 작성</t>
+          <t>연구가설 설정 및 개념검증 논리 수립</t>
         </is>
       </c>
       <c r="D18" s="41" t="n"/>
@@ -1873,7 +1871,7 @@
       <c r="B19" s="112" t="n"/>
       <c r="C19" s="113" t="inlineStr">
         <is>
-          <t>제4장 시스템 모듈(5~6개) 정의·구성방식 비교·제품구조·데이터 흐름 초안 작성</t>
+          <t>시스템·제품 구조 및 데이터 흐름 설계 초안 정립</t>
         </is>
       </c>
       <c r="D19" s="41" t="n"/>
@@ -1889,7 +1887,7 @@
       <c r="B20" s="112" t="n"/>
       <c r="C20" s="111" t="inlineStr">
         <is>
-          <t>제2장 필수 산출물(표·그림) 및 미확인 가정·대표 검토 쟁점·용어/약어 정리</t>
+          <t>필수 산출물·미확인 가정·대표 검토 쟁점·용어 정리</t>
         </is>
       </c>
       <c r="D20" s="41" t="n"/>
@@ -1948,11 +1946,11 @@
       </c>
       <c r="C23" s="105" t="inlineStr">
         <is>
-          <t>· 제1장(대표 확정)의 기술개발 방향·연구개발 목표를 최상위 기준으로 삼는다
-· TRL 1 수준 유지: 문제 관찰·기술원리 정립·시스템 개념 정의·연구가설 설정·적용/제외조건·후보 성능지표·TRL 2 계획까지만 작성
+          <t>· 제1장(대표 확정) 기술개발 방향·연구개발 목표를 최상위 기준으로 삼을 것
+· TRL 1 수준 유지: 문제 관찰·기술원리·시스템 개념·연구가설·적용/제외조건·후보 성능지표·TRL 2 계획까지만 작성
 · '성능 달성·스마트공장 구축·자동설계 완성·원가 절감 완료·센서만으로 원인 확정' 등 달성형 표현 금지
-· 서술은 □핵심주제/○세부주제/•현황·원인·기술필요성·대응방향·TRL1 정립사항 구조로 작성
-· 첨부 작성 가이드는 참고자료이며 입구 MVP와 상충 시 입구 MVP 우선</t>
+· 서술은 □핵심주제 / ○세부주제 / •현황·원인·기술필요성·대응방향·TRL1 정립사항 구조로 작성
+· 첨부 가이드는 참고자료이며 입구 MVP와 상충 시 입구 MVP 우선</t>
         </is>
       </c>
       <c r="D23" s="41" t="n"/>
@@ -1976,7 +1974,7 @@
       </c>
       <c r="C24" s="102" t="inlineStr">
         <is>
-          <t>제1장 확정 MVP와 상충하거나 TRL 1 수준을 넘는 작성이 필요하다고 판단되면 변경 사유·영향을 문서화하여 대표 승인 후 반영한다.</t>
+          <t>제1장 확정 MVP와 상충하거나 TRL 1 수준을 넘는 작성이 필요하면 변경 사유·영향을 문서화하여 대표 승인 후 반영할 것.</t>
         </is>
       </c>
       <c r="D24" s="41" t="n"/>
@@ -2070,25 +2068,25 @@
       </c>
       <c r="C28" s="47" t="inlineStr">
         <is>
-          <t>제1장 확정 MVP 기준 정합 및 가이드 최신화</t>
+          <t>기존 TRL 1 작성 가이드를 입구 1개소 MVP 기준으로 최신화하라</t>
         </is>
       </c>
       <c r="D28" s="47" t="inlineStr">
         <is>
-          <t>기존 TRL 1 작성 가이드의 방·창호·외벽 중심 표현을 입구 1개소 MVP 기준으로 전수 식별·수정하고 초기 MVP와 후속 확장범위를 구분한다.</t>
+          <t>대표가 확정한 입구 1개소 Scan-to-Fit 리트로핏 MVP를 최상위 기준으로, 가이드 전반의 방·창호·외벽 중심 표현을 입구 기준으로 수정하고 적용범위를 확정한다.</t>
         </is>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>① 가이드 내 방·창호·외벽 중심 표현 위치 전수 식별 목록
-② 기존→수정 대조표(입구 1개소 MVP 기준)
-③ 초기 MVP / 후속 확장범위(센서·창호·외벽) 구분표
-④ 기술 중심축 순서(현장·고객조사→입구 3D실측→As-is BIM→문제분석→To-be 기획→Scan-to-Fit→표준/맞춤 분리→BIM–BOM–제작도면→공장 사전제작→현장 건식설치→검증→FM/Building Passport) 흐름도 1개</t>
+          <t>① 가이드 내 방·창호·외벽 중심 표현 위치를 전수 식별한 목록을 작성할 것
+② 기존→수정 대조표를 작성할 것
+③ 초기 MVP / 후속 확장범위(센서·창호·외벽) 구분표를 작성할 것
+④ 기술 중심축(현장·고객조사→입구 3D실측→As-is BIM→문제분석→To-be 기획→Scan-to-Fit→표준/맞춤 분리→BIM–BOM–제작도면→공장 사전제작→현장 건식설치→검증→FM/Building Passport) 흐름도 1개를 확정할 것</t>
         </is>
       </c>
       <c r="F28" s="47" t="inlineStr">
         <is>
-          <t>01_황우중_MVP정합_가이드최신화_W30_v1.xlsx</t>
+          <t>01_황우중_가이드최신화_W30_v1.xlsx</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
@@ -2107,10 +2105,10 @@
         </is>
       </c>
       <c r="J28" s="114" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="29" ht="123" customHeight="1" s="49">
@@ -2119,25 +2117,25 @@
       </c>
       <c r="C29" s="47" t="inlineStr">
         <is>
-          <t>제2장 1절 — 노후건축물 입구·공용부 구조 분석</t>
+          <t>노후건축물 입구 현장의 문제와 기존 공정의 비효율을 분석하라</t>
         </is>
       </c>
       <c r="D29" s="47" t="inlineStr">
         <is>
-          <t>노후 소형건축물 입구·공용부의 구조와 간섭요소를 분석하고, 왜 표준제품을 그대로 적용하기 어려운지를 구조적으로 설명한다.</t>
+          <t>노후 소형건축물 입구·공용부의 구조와 간섭요소를 분석해 표준제품을 그대로 적용하기 어려운 근거를 도출하고, 기존 실측·기획·제작·설치 공정의 비효율을 분석한다.</t>
         </is>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>① 입구 구성요소(벽체·바닥·천장·출입문·계단·캐노피·공용설비) 분류표
-② 벽면 요철·바닥 경사·단차·벽체 기울기 등 시공오차 요인 정리
-③ 배관·배선·계량기·실외기 등 간섭요소 및 구조체 체결 가능 위치 정리
-④ 표준제품 직접 적용이 어려운 근거를 구조적으로 서술 + 운반·반입·조립 영향 조건</t>
+          <t>① 입구 구성요소·간섭요소·구조체 체결 가능 위치 분류표를 작성할 것
+② 벽면 요철·바닥 경사·단차·벽체 기울기 등 시공오차 요인을 정리할 것
+③ 기존 공정 흐름도(현장방문→실측→기획→개별도면→재실측→주문제작→현장 절단·천공·용접→설치→재작업)를 작성할 것
+④ 비효율 8항목 분석표를 작성하고 표준제품 적용 곤란 근거를 서술할 것</t>
         </is>
       </c>
       <c r="F29" s="47" t="inlineStr">
         <is>
-          <t>02_황우중_2장1절_입구구조분석_W30_v1.pdf</t>
+          <t>02_황우중_입구문제_공정분석_W30_v1.pdf</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
@@ -2147,7 +2145,7 @@
       </c>
       <c r="H29" s="107" t="inlineStr">
         <is>
-          <t>07-21(화) 18:00</t>
+          <t>07-22(수) 18:00</t>
         </is>
       </c>
       <c r="I29" s="47" t="inlineStr">
@@ -2156,10 +2154,10 @@
         </is>
       </c>
       <c r="J29" s="114" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>0.1</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="30" ht="84" customHeight="1" s="49">
@@ -2168,24 +2166,25 @@
       </c>
       <c r="C30" s="47" t="inlineStr">
         <is>
-          <t>제2장 2절 — 기존 공간기획·실측·제작·설치 공정 분석</t>
+          <t>기존 기술을 비교하고 브링이 해결할 핵심 문제를 정의하라</t>
         </is>
       </c>
       <c r="D30" s="47" t="inlineStr">
         <is>
-          <t>기존 입구 개선공사 공정의 흐름과 비효율을 분석한다.</t>
+          <t>관련 기존 기술을 비교해 입구 리트로핏 적용 한계와 브링의 보완지점을 도출하고, 보고서 전체의 핵심 문제를 한 문장으로 고정한다.</t>
         </is>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>① 현장방문→실측→공간기획→개별도면→재실측→주문제작→현장 절단·천공·용접→설치→재작업 공정 흐름도
-② 비효율 8항목(기획-제작 분리, 실측 누락·반복, 정보단절, 현장 추가가공, 업체 일정조정, 부품 재제작, 부분교체 곤란, 이력 미관리) 분석표
-③ 정보단절·재작업 발생 지점 표기</t>
+          <t>① 기존 기술 8종(현장 인테리어·리모델링/프리패브·OSC/모듈러 신축/Scan-to-BIM/파라메트릭 설계/3D프린팅/시설관리 앱/BIM·디지털트윈 FM) 비교표(해결문제·강점·입구적용 한계·브링 보완방향)를 작성할 것
+② 핵심 문제문장 1개를 확정할 것
+③ 하위 7개 문제 분해도를 작성할 것
+④ 각 하위문제의 근거를 정리할 것</t>
         </is>
       </c>
       <c r="F30" s="47" t="inlineStr">
         <is>
-          <t>03_황우중_2장2절_공정비효율분석_W30_v1.pdf</t>
+          <t>03_황우중_기술비교_핵심문제_W30_v1.xlsx</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -2204,10 +2203,10 @@
         </is>
       </c>
       <c r="J30" s="114" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>0.1</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="31" ht="90" customHeight="1" s="49">
@@ -2216,23 +2215,24 @@
       </c>
       <c r="C31" s="47" t="inlineStr">
         <is>
-          <t>제2장 3절 — 기존 기술 8종 비교 및 한계</t>
+          <t>입구 리트로핏 기술개념과 전체 흐름을 정립하라</t>
         </is>
       </c>
       <c r="D31" s="47" t="inlineStr">
         <is>
-          <t>관련 기존 기술을 비교하여 입구 리트로핏 적용 시 한계와 브링 기술의 보완지점을 도출한다.</t>
+          <t>입구 조사부터 FM 등록까지의 기술흐름을 개념 수준에서 정의하고 각 단계 입출력을 정리한다.</t>
         </is>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>① 기존 기술 8종(현장 인테리어·리모델링/프리패브·OSC/모듈러 신축/Scan-to-BIM/파라메트릭 설계/3D프린팅/시설관리 앱/BIM·디지털트윈 FM) 비교표
-② 각 기술의 해결문제·강점·노후건축물 입구 적용 한계·브링 보완방향 작성</t>
+          <t>① 기술 개념 흐름도(입구 현장조사→형상·공차 실측→As-is BIM→문제분석→To-be 기획→Scan-to-Fit 설계→표준 프레임 선정→맞춤 연결부 설계→기능 카세트 조합→BOM·제작도면→공장 사전제작·조립→현장 건식설치→품질·탈착 검증→FM/Building Passport 등록)를 작성할 것
+② 각 단계 입력·출력을 정의할 것
+③ 초기 MVP·후속 확장범위 표를 작성할 것</t>
         </is>
       </c>
       <c r="F31" s="47" t="inlineStr">
         <is>
-          <t>04_황우중_2장3절_기존기술비교_W30_v1.xlsx</t>
+          <t>04_황우중_기술개념_흐름정립_W30_v1.pdf</t>
         </is>
       </c>
       <c r="G31" s="108" t="inlineStr">
@@ -2242,7 +2242,7 @@
       </c>
       <c r="H31" s="107" t="inlineStr">
         <is>
-          <t>07-22(수) 18:00</t>
+          <t>07-23(목) 18:00</t>
         </is>
       </c>
       <c r="I31" s="47" t="inlineStr">
@@ -2251,10 +2251,10 @@
         </is>
       </c>
       <c r="J31" s="114" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K31" s="19" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="32" ht="69" customHeight="1" s="49">
@@ -2263,24 +2263,25 @@
       </c>
       <c r="C32" s="47" t="inlineStr">
         <is>
-          <t>제2장 4절 — 핵심 문제 정의 및 분해</t>
+          <t>연구가설을 설정하고 개념검증 논리를 수립하라</t>
         </is>
       </c>
       <c r="D32" s="47" t="inlineStr">
         <is>
-          <t>보고서 전체의 핵심 문제를 한 문장으로 고정하고 하위 문제로 분해한다.</t>
+          <t>각 기술요소의 필요성을 인과관계로 설명하고 검증 가능한 연구가설로 전환한다.</t>
         </is>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>① 핵심 문제문장 1개 확정(형상 상이·시공오차·정보 분리·현장 맞춤가공·재작업 반복)
-② 하위 7개 문제(형상정보 부족/기획-제작 단절/현장 공차 대응 부족/표준·맞춤 구분 부재/공장 사전제작률 부족/탈부착·부분교체 부족/설치 후 이력관리 부족) 분해도
-③ 각 하위문제의 근거</t>
+          <t>① 연구가설 6개 이상(디지털 실측/BIM 기반 기획-제작 연계/표준·맞춤 분리 반복성/공장 사전조립 작업·재작업 절감/탈부착 카세트 부분교체·기능추가/Building Passport 이력관리)을 설정할 것
+② 가설별 표(연구가설/논리적 근거/확인할 데이터/TRL 2 검증방법/예상 산출물)를 작성할 것
+③ 완전주문제작·완전표준화·혼합생산 비교표를 작성할 것
+④ 기술요소별 필요성 표를 작성할 것</t>
         </is>
       </c>
       <c r="F32" s="47" t="inlineStr">
         <is>
-          <t>05_황우중_2장4절_핵심문제정의_W30_v1.pdf</t>
+          <t>05_황우중_연구가설_검증논리_W30_v1.xlsx</t>
         </is>
       </c>
       <c r="G32" s="108" t="inlineStr">
@@ -2290,7 +2291,7 @@
       </c>
       <c r="H32" s="107" t="inlineStr">
         <is>
-          <t>07-22(수) 18:00</t>
+          <t>07-23(목) 18:00</t>
         </is>
       </c>
       <c r="I32" s="47" t="inlineStr">
@@ -2299,34 +2300,35 @@
         </is>
       </c>
       <c r="J32" s="114" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>0.1</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="33" ht="90" customHeight="1" s="49">
       <c r="B33" s="17" t="n"/>
       <c r="C33" s="47" t="inlineStr">
         <is>
-          <t>제2장 5절 — 기술 개념 정의 및 흐름도</t>
+          <t>시스템·제품 구조와 데이터 흐름을 설계 초안으로 정립하라</t>
         </is>
       </c>
       <c r="D33" s="47" t="inlineStr">
         <is>
-          <t>입구 리트로핏 기술흐름을 개념 수준에서 정의한다.</t>
+          <t>TRL 1 수준에서 시스템을 5~6개 모듈로 정리하고 혼합생산형 입구 리트로핏 구조를 개념안으로 도출한다.</t>
         </is>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>① 기술 개념 흐름도(입구 현장조사→형상·공차 실측→As-is BIM→공간·성능 문제 분석→To-be 공간기획→Scan-to-Fit 설계→표준 프레임 선정→맞춤 연결부 설계→기능 카세트 조합→BOM·제작도면→공장 사전제작·조립→현장 건식설치→품질·탈착 검증→FM/Building Passport 등록)
-② 각 단계 입력·출력 정의
-③ 초기 MVP·후속 확장범위 표</t>
+          <t>① 모듈 5~6개 정의표(역할/입력/처리/출력/HW/SW/수행주체/초기MVP 포함여부/후속확장)를 작성할 것
+② 구성방식 6후보 비교표(현장적합성·제작난이도·원가·표준화·운송·설치·탈착·확장성·스마트공장 연계)를 작성할 것
+③ 최적 구조 선정 근거표(혼합생산형 입구 리트로핏 — TRL 2에서 변경 가능한 개념안)를 작성할 것
+④ 전체 시스템 구성도·제품 분해구조도(표준 프레임–맞춤 연결부–기능 카세트)·데이터 흐름도(BIM–BOM–제작도면–부품ID–FM)를 작성할 것</t>
         </is>
       </c>
       <c r="F33" s="47" t="inlineStr">
         <is>
-          <t>06_황우중_2장5절_기술개념흐름_W30_v1.pdf</t>
+          <t>06_황우중_시스템제품구조_초안_W30_v1.pdf</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
@@ -2336,7 +2338,7 @@
       </c>
       <c r="H33" s="107" t="inlineStr">
         <is>
-          <t>07-23(목) 18:00</t>
+          <t>07-24(금) 15:00</t>
         </is>
       </c>
       <c r="I33" s="47" t="inlineStr">
@@ -2345,35 +2347,35 @@
         </is>
       </c>
       <c r="J33" s="114" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K33" s="19" t="n">
-        <v>0.1</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="34" ht="90" customHeight="1" s="49">
       <c r="B34" s="17" t="n"/>
       <c r="C34" s="47" t="inlineStr">
         <is>
-          <t>제3장 — 연구가설 및 개념검증 논리 초안</t>
+          <t>필수 산출물을 완비하고 미확인 가정·검토 쟁점·용어를 정리하여 제출하라</t>
         </is>
       </c>
       <c r="D34" s="47" t="inlineStr">
         <is>
-          <t>각 기술요소가 왜 필요한지 인과관계로 설명하고 검증 가능한 연구가설로 전환한다.</t>
+          <t>제2장 필수 산출물을 완비하고 TRL 1 단계에서 확정되지 않은 가정과 대표 검토가 필요한 쟁점을 분리 정리한다.</t>
         </is>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>① 최소 6개 연구가설(디지털 실측/BIM 기반 기획-제작 연계/표준·맞춤 분리 반복성/공장 사전조립 작업·재작업 절감/탈부착 카세트 부분교체·기능추가/Building Passport 이력관리)
-② 가설별 표: 연구가설 / 논리적 근거 / 확인해야 할 데이터 / TRL 2 검증방법 / 예상 산출물
-③ 완전주문제작·완전표준화·혼합생산 비교표
-④ 기술요소별 필요성 표</t>
+          <t>① 필수 산출물 6종(입구 구조 분류표/기존 공정 비효율표/기존 기술 비교표/핵심 문제 분해도/기술개념 흐름도/초기 MVP·후속확장 표)을 완비할 것
+② 확인되지 않은 가정 목록을 작성할 것
+③ 대표 검토가 필요한 쟁점 목록을 작성할 것
+④ 용어정의·약어목록·참고문헌 초안을 제출할 것</t>
         </is>
       </c>
       <c r="F34" s="47" t="inlineStr">
         <is>
-          <t>07_황우중_3장_연구가설_검증초안_W30_v1.xlsx</t>
+          <t>07_황우중_산출물_쟁점_용어정리_W30_v1.pdf</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
@@ -2383,234 +2385,143 @@
       </c>
       <c r="H34" s="107" t="inlineStr">
         <is>
-          <t>07-23(목) 18:00</t>
+          <t>07-24(금) 17:00</t>
         </is>
       </c>
       <c r="I34" s="47" t="inlineStr">
         <is>
-          <t>높음</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="J34" s="114" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K34" s="19" t="n">
-        <v>0.12</v>
-      </c>
-    </row>
-    <row r="35" ht="90" customHeight="1" s="49">
-      <c r="B35" s="17" t="n"/>
-      <c r="C35" s="47" t="inlineStr">
-        <is>
-          <t>제4장 — 시스템 구조·구성방식·최적구조 초안</t>
-        </is>
-      </c>
-      <c r="D35" s="47" t="inlineStr">
-        <is>
-          <t>TRL 1 수준에서 시스템을 5~6개 모듈로 정리하고 혼합생산형 입구 리트로핏 구조를 개념안으로 도출한다.</t>
-        </is>
-      </c>
-      <c r="E35" s="1" t="inlineStr">
-        <is>
-          <t>① 모듈 5~6개 정의표(역할/입력/처리/출력/HW/SW/수행주체/초기MVP 포함여부/후속확장)
-② 구성방식 6후보 비교표(현장적합성·제작난이도·원가·표준화·운송·설치·탈착·확장성·스마트공장 연계)
-③ 최적 구조 선정 근거표(혼합생산형 입구 리트로핏 — TRL 2에서 변경 가능한 개념안으로 표기)
-④ 전체 시스템 구성도</t>
-        </is>
-      </c>
-      <c r="F35" s="47" t="inlineStr">
-        <is>
-          <t>08_황우중_4장_시스템구조_초안_W30_v1.pdf</t>
-        </is>
-      </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>브링 구글 드라이브</t>
-        </is>
-      </c>
-      <c r="H35" s="107" t="inlineStr">
-        <is>
-          <t>07-24(금) 12:00</t>
-        </is>
-      </c>
-      <c r="I35" s="47" t="inlineStr">
-        <is>
-          <t>높음</t>
-        </is>
-      </c>
-      <c r="J35" s="114" t="n">
-        <v>6</v>
-      </c>
-      <c r="K35" s="19" t="n">
-        <v>0.12</v>
-      </c>
-    </row>
-    <row r="36" ht="90" customHeight="1" s="49">
-      <c r="B36" s="17" t="n"/>
-      <c r="C36" s="47" t="inlineStr">
-        <is>
-          <t>제4장 — 제품구조·데이터 흐름 + 제2장 필수 산출물 패키지</t>
-        </is>
-      </c>
-      <c r="D36" s="47" t="inlineStr">
-        <is>
-          <t>제품 분해구조와 데이터 흐름을 초안화하고 제2장 필수 산출물을 완비한다.</t>
-        </is>
-      </c>
-      <c r="E36" s="1" t="inlineStr">
-        <is>
-          <t>① 제품 분해구조도(표준 프레임–맞춤 공차보정 연결부–탈부착 기능 카세트)
-② 데이터 흐름도(BIM–BOM–제작도면–부품 ID–품질검사–FM/Passport)
-③ 제2장 필수 산출물 6종 완비(입구 구조 분류표/기존 공정 비효율표/기존 기술 비교표/핵심 문제 분해도/기술개념 흐름도/초기 MVP·후속확장 표)</t>
-        </is>
-      </c>
-      <c r="F36" s="47" t="inlineStr">
-        <is>
-          <t>09_황우중_4장제품구조_2장산출물_W30_v1.pdf</t>
-        </is>
-      </c>
-      <c r="G36" s="6" t="inlineStr">
-        <is>
-          <t>브링 구글 드라이브</t>
-        </is>
-      </c>
-      <c r="H36" s="107" t="inlineStr">
-        <is>
-          <t>07-24(금) 15:00</t>
-        </is>
-      </c>
-      <c r="I36" s="47" t="inlineStr">
-        <is>
-          <t>높음</t>
-        </is>
-      </c>
-      <c r="J36" s="114" t="n">
-        <v>5</v>
-      </c>
-      <c r="K36" s="19" t="n">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="37" ht="90" customHeight="1" s="49">
-      <c r="B37" s="17" t="n"/>
-      <c r="C37" s="47" t="inlineStr">
-        <is>
-          <t>미확인 가정·대표 검토 쟁점·용어/약어 정리</t>
-        </is>
-      </c>
-      <c r="D37" s="47" t="inlineStr">
-        <is>
-          <t>TRL 1 단계에서 확정되지 않은 가정과 대표 검토가 필요한 쟁점을 분리하고 부속자료를 정리한다.</t>
-        </is>
-      </c>
-      <c r="E37" s="1" t="inlineStr">
-        <is>
-          <t>① 확인되지 않은 가정 목록
-② 대표 검토가 필요한 쟁점 목록
-③ 용어정의·약어목록 초안
-④ 참고문헌·근거자료 출처 목록</t>
-        </is>
-      </c>
-      <c r="F37" s="47" t="inlineStr">
-        <is>
-          <t>10_황우중_가정_쟁점_용어정리_W30_v1.pdf</t>
-        </is>
-      </c>
-      <c r="G37" s="6" t="inlineStr">
-        <is>
-          <t>브링 구글 드라이브</t>
-        </is>
-      </c>
-      <c r="H37" s="107" t="inlineStr">
-        <is>
-          <t>07-24(금) 17:00</t>
-        </is>
-      </c>
-      <c r="I37" s="47" t="inlineStr">
-        <is>
-          <t>보통</t>
-        </is>
-      </c>
-      <c r="J37" s="114" t="n">
-        <v>3</v>
-      </c>
-      <c r="K37" s="19" t="n">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="38" ht="69" customHeight="1" s="49">
-      <c r="B38" s="45" t="inlineStr">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="35" ht="69" customHeight="1" s="49">
+      <c r="B35" s="45" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="C38" s="51" t="n"/>
-      <c r="D38" s="41" t="n"/>
-      <c r="E38" s="41" t="n"/>
-      <c r="F38" s="41" t="n"/>
-      <c r="G38" s="41" t="n"/>
-      <c r="H38" s="41" t="n"/>
-      <c r="I38" s="42" t="n"/>
-      <c r="J38" s="115">
-        <f>SUM(J28:J37)</f>
-        <v/>
-      </c>
-      <c r="K38" s="21">
-        <f>SUM(K28:K37)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" ht="24" customHeight="1" s="49">
-      <c r="B39" s="45" t="inlineStr">
+      <c r="C35" s="51" t="n"/>
+      <c r="D35" s="41" t="n"/>
+      <c r="E35" s="41" t="n"/>
+      <c r="F35" s="41" t="n"/>
+      <c r="G35" s="41" t="n"/>
+      <c r="H35" s="41" t="n"/>
+      <c r="I35" s="42" t="n"/>
+      <c r="J35" s="115">
+        <f>SUM(J28:J34)</f>
+        <v/>
+      </c>
+      <c r="K35" s="21">
+        <f>SUM(K28:K34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1" s="49">
+      <c r="B36" s="45" t="inlineStr">
         <is>
           <t>발행 검증</t>
         </is>
       </c>
-      <c r="C39" s="116">
-        <f>IF(COUNTA(C28:C37)=0,"업무 미입력",IF(COUNTA(E28:E37)&lt;COUNTA(C28:C37),"발행 불가 — 완료기준 누락 업무 있음",IF(COUNTA(F28:F37)&lt;COUNTA(C28:C37),"발행 불가 — 산출물 누락 업무 있음",IF(SUM(K28:K37)&lt;&gt;1,"발행 불가 — 가중치 합계 "&amp;TEXT(SUM(K28:K37),"0%")&amp;" (100% 필요)","발행 가능 — 완료기준·산출물·가중치 충족"))))</f>
-        <v/>
-      </c>
-      <c r="D39" s="41" t="n"/>
-      <c r="E39" s="41" t="n"/>
-      <c r="F39" s="41" t="n"/>
-      <c r="G39" s="41" t="n"/>
-      <c r="H39" s="41" t="n"/>
-      <c r="I39" s="41" t="n"/>
-      <c r="J39" s="41" t="n"/>
-      <c r="K39" s="42" t="n"/>
-    </row>
-    <row r="40" ht="24" customHeight="1" s="49">
-      <c r="B40" s="45" t="n"/>
-      <c r="C40" s="43" t="n"/>
-    </row>
-    <row r="41" ht="24" customHeight="1" s="49">
-      <c r="B41" s="45" t="n"/>
-      <c r="C41" s="43" t="n"/>
-    </row>
-    <row r="42" ht="18" customHeight="1" s="49">
-      <c r="B42" s="89" t="inlineStr">
+      <c r="C36" s="116">
+        <f>IF(COUNTA(C28:C34)=0,"업무 미입력",IF(COUNTA(E28:E34)&lt;COUNTA(C28:C34),"발행 불가 — 완료기준 누락 업무 있음",IF(COUNTA(F28:F34)&lt;COUNTA(C28:C34),"발행 불가 — 산출물 누락 업무 있음",IF(SUM(K28:K34)&lt;&gt;1,"발행 불가 — 가중치 합계 "&amp;TEXT(SUM(K28:K34),"0%")&amp;" (100% 필요)","발행 가능 — 완료기준·산출물·가중치 충족"))))</f>
+        <v/>
+      </c>
+      <c r="D36" s="41" t="n"/>
+      <c r="E36" s="41" t="n"/>
+      <c r="F36" s="41" t="n"/>
+      <c r="G36" s="41" t="n"/>
+      <c r="H36" s="41" t="n"/>
+      <c r="I36" s="41" t="n"/>
+      <c r="J36" s="41" t="n"/>
+      <c r="K36" s="42" t="n"/>
+    </row>
+    <row r="37" ht="24" customHeight="1" s="49">
+      <c r="B37" s="89" t="n"/>
+    </row>
+    <row r="38" ht="24" customHeight="1" s="49">
+      <c r="B38" s="45" t="n"/>
+      <c r="C38" s="117" t="n"/>
+    </row>
+    <row r="39" ht="18" customHeight="1" s="49">
+      <c r="B39" s="89" t="inlineStr">
         <is>
           <t>담당자 접수확인  —  월요일 12:00까지 담당자 직접 작성 (미작성 = 업무 미이해로 간주, 재지시)</t>
         </is>
       </c>
-      <c r="C42" s="64" t="n"/>
-      <c r="D42" s="64" t="n"/>
-      <c r="E42" s="64" t="n"/>
-      <c r="F42" s="64" t="n"/>
-      <c r="G42" s="64" t="n"/>
-      <c r="H42" s="64" t="n"/>
-      <c r="I42" s="64" t="n"/>
-      <c r="J42" s="64" t="n"/>
-      <c r="K42" s="64" t="n"/>
-    </row>
-    <row r="43" ht="36" customHeight="1" s="49">
-      <c r="B43" s="45" t="inlineStr">
+      <c r="C39" s="64" t="n"/>
+      <c r="D39" s="64" t="n"/>
+      <c r="E39" s="64" t="n"/>
+      <c r="F39" s="64" t="n"/>
+      <c r="G39" s="64" t="n"/>
+      <c r="H39" s="64" t="n"/>
+      <c r="I39" s="64" t="n"/>
+      <c r="J39" s="64" t="n"/>
+      <c r="K39" s="64" t="n"/>
+    </row>
+    <row r="40" ht="36" customHeight="1" s="49">
+      <c r="B40" s="45" t="inlineStr">
         <is>
           <t>내가 이해한 업무
 (본인 언어로 재작성)</t>
         </is>
       </c>
-      <c r="C43" s="117" t="n"/>
+      <c r="C40" s="117" t="n"/>
+      <c r="D40" s="41" t="n"/>
+      <c r="E40" s="41" t="n"/>
+      <c r="F40" s="41" t="n"/>
+      <c r="G40" s="41" t="n"/>
+      <c r="H40" s="41" t="n"/>
+      <c r="I40" s="41" t="n"/>
+      <c r="J40" s="41" t="n"/>
+      <c r="K40" s="42" t="n"/>
+    </row>
+    <row r="41" ht="19.5" customHeight="1" s="49">
+      <c r="B41" s="45" t="inlineStr">
+        <is>
+          <t>완료기준 재확인
+(무엇이 되면 끝인가)</t>
+        </is>
+      </c>
+      <c r="C41" s="118" t="n"/>
+      <c r="D41" s="41" t="n"/>
+      <c r="E41" s="41" t="n"/>
+      <c r="F41" s="41" t="n"/>
+      <c r="G41" s="41" t="n"/>
+      <c r="H41" s="41" t="n"/>
+      <c r="I41" s="41" t="n"/>
+      <c r="J41" s="41" t="n"/>
+      <c r="K41" s="42" t="n"/>
+    </row>
+    <row r="42" ht="24" customHeight="1" s="49">
+      <c r="B42" s="45" t="inlineStr">
+        <is>
+          <t>예상 리스크
+(막힐 것 같은 지점)</t>
+        </is>
+      </c>
+      <c r="C42" s="43" t="n"/>
+      <c r="D42" s="41" t="n"/>
+      <c r="E42" s="41" t="n"/>
+      <c r="F42" s="41" t="n"/>
+      <c r="G42" s="41" t="n"/>
+      <c r="H42" s="41" t="n"/>
+      <c r="I42" s="41" t="n"/>
+      <c r="J42" s="41" t="n"/>
+      <c r="K42" s="42" t="n"/>
+    </row>
+    <row r="43" ht="24" customHeight="1" s="49">
+      <c r="B43" s="45" t="inlineStr">
+        <is>
+          <t>필요한 지원·의사결정</t>
+        </is>
+      </c>
+      <c r="C43" s="43" t="n"/>
       <c r="D43" s="41" t="n"/>
       <c r="E43" s="41" t="n"/>
       <c r="F43" s="41" t="n"/>
@@ -2620,14 +2531,13 @@
       <c r="J43" s="41" t="n"/>
       <c r="K43" s="42" t="n"/>
     </row>
-    <row r="44" ht="19.5" customHeight="1" s="49">
+    <row r="44" ht="24" customHeight="1" s="49">
       <c r="B44" s="45" t="inlineStr">
         <is>
-          <t>완료기준 재확인
-(무엇이 되면 끝인가)</t>
-        </is>
-      </c>
-      <c r="C44" s="118" t="n"/>
+          <t>실행 계획 (요일 배분)</t>
+        </is>
+      </c>
+      <c r="C44" s="43" t="n"/>
       <c r="D44" s="41" t="n"/>
       <c r="E44" s="41" t="n"/>
       <c r="F44" s="41" t="n"/>
@@ -2640,11 +2550,10 @@
     <row r="45" ht="24" customHeight="1" s="49">
       <c r="B45" s="45" t="inlineStr">
         <is>
-          <t>예상 리스크
-(막힐 것 같은 지점)</t>
-        </is>
-      </c>
-      <c r="C45" s="43" t="n"/>
+          <t>접수 확인 일시 / 서명</t>
+        </is>
+      </c>
+      <c r="C45" s="47" t="n"/>
       <c r="D45" s="41" t="n"/>
       <c r="E45" s="41" t="n"/>
       <c r="F45" s="41" t="n"/>
@@ -2655,28 +2564,20 @@
       <c r="K45" s="42" t="n"/>
     </row>
     <row r="46" ht="24" customHeight="1" s="49">
-      <c r="B46" s="45" t="inlineStr">
-        <is>
-          <t>필요한 지원·의사결정</t>
-        </is>
-      </c>
-      <c r="C46" s="43" t="n"/>
-      <c r="D46" s="41" t="n"/>
-      <c r="E46" s="41" t="n"/>
-      <c r="F46" s="41" t="n"/>
-      <c r="G46" s="41" t="n"/>
-      <c r="H46" s="41" t="n"/>
-      <c r="I46" s="41" t="n"/>
-      <c r="J46" s="41" t="n"/>
-      <c r="K46" s="42" t="n"/>
+      <c r="B46" s="45" t="n"/>
+      <c r="C46" s="45" t="n"/>
+      <c r="E46" s="45" t="n"/>
+      <c r="G46" s="45" t="n"/>
+      <c r="I46" s="45" t="n"/>
+      <c r="K46" s="45" t="n"/>
     </row>
     <row r="47" ht="24" customHeight="1" s="49">
-      <c r="B47" s="45" t="inlineStr">
-        <is>
-          <t>실행 계획 (요일 배분)</t>
-        </is>
-      </c>
-      <c r="C47" s="43" t="n"/>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>결   재</t>
+        </is>
+      </c>
+      <c r="C47" s="41" t="n"/>
       <c r="D47" s="41" t="n"/>
       <c r="E47" s="41" t="n"/>
       <c r="F47" s="41" t="n"/>
@@ -2689,108 +2590,78 @@
     <row r="48" ht="24" customHeight="1" s="49">
       <c r="B48" s="45" t="inlineStr">
         <is>
-          <t>접수 확인 일시 / 서명</t>
-        </is>
-      </c>
-      <c r="C48" s="47" t="n"/>
-      <c r="D48" s="41" t="n"/>
-      <c r="E48" s="41" t="n"/>
-      <c r="F48" s="41" t="n"/>
-      <c r="G48" s="41" t="n"/>
-      <c r="H48" s="41" t="n"/>
-      <c r="I48" s="41" t="n"/>
-      <c r="J48" s="41" t="n"/>
-      <c r="K48" s="42" t="n"/>
-    </row>
-    <row r="49" ht="24" customHeight="1" s="49"/>
-    <row r="50" ht="24" customHeight="1" s="49">
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>결   재</t>
-        </is>
-      </c>
-      <c r="C50" s="41" t="n"/>
-      <c r="D50" s="41" t="n"/>
-      <c r="E50" s="41" t="n"/>
-      <c r="F50" s="41" t="n"/>
-      <c r="G50" s="41" t="n"/>
-      <c r="H50" s="41" t="n"/>
-      <c r="I50" s="41" t="n"/>
-      <c r="J50" s="41" t="n"/>
-      <c r="K50" s="42" t="n"/>
-    </row>
-    <row r="51" ht="24" customHeight="1" s="49">
-      <c r="B51" s="45" t="inlineStr">
-        <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="C51" s="45" t="inlineStr">
+      <c r="C48" s="45" t="inlineStr">
         <is>
           <t>작성 (지시자)</t>
         </is>
       </c>
-      <c r="D51" s="42" t="n"/>
-      <c r="E51" s="45" t="inlineStr">
+      <c r="D48" s="42" t="n"/>
+      <c r="E48" s="45" t="inlineStr">
         <is>
           <t>검토 (검수자)</t>
         </is>
       </c>
-      <c r="F51" s="42" t="n"/>
-      <c r="G51" s="45" t="inlineStr">
+      <c r="F48" s="42" t="n"/>
+      <c r="G48" s="45" t="inlineStr">
         <is>
           <t>승인 (대표)</t>
         </is>
       </c>
-      <c r="H51" s="42" t="n"/>
-      <c r="I51" s="45" t="inlineStr">
+      <c r="H48" s="42" t="n"/>
+      <c r="I48" s="45" t="inlineStr">
         <is>
           <t>접수 (담당자)</t>
         </is>
       </c>
-      <c r="J51" s="42" t="n"/>
-      <c r="K51" s="45" t="inlineStr">
+      <c r="J48" s="42" t="n"/>
+      <c r="K48" s="45" t="inlineStr">
         <is>
           <t>일자</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="21.75" customHeight="1" s="49">
-      <c r="B52" s="45" t="inlineStr">
+    <row r="49" ht="21.75" customHeight="1" s="49">
+      <c r="B49" s="45" t="inlineStr">
         <is>
           <t>서명</t>
         </is>
       </c>
-      <c r="C52" s="47" t="inlineStr">
+      <c r="C49" s="47" t="inlineStr">
         <is>
           <t>서 창 환</t>
         </is>
       </c>
-      <c r="D52" s="42" t="n"/>
-      <c r="E52" s="47" t="inlineStr">
+      <c r="D49" s="42" t="n"/>
+      <c r="E49" s="47" t="inlineStr">
         <is>
           <t>서 창 환</t>
         </is>
       </c>
-      <c r="F52" s="42" t="n"/>
-      <c r="G52" s="47" t="inlineStr">
+      <c r="F49" s="42" t="n"/>
+      <c r="G49" s="47" t="inlineStr">
         <is>
           <t>서 창 환</t>
         </is>
       </c>
-      <c r="H52" s="42" t="n"/>
-      <c r="I52" s="47" t="inlineStr">
+      <c r="H49" s="42" t="n"/>
+      <c r="I49" s="47" t="inlineStr">
         <is>
           <t>황 우 중</t>
         </is>
       </c>
-      <c r="J52" s="42" t="n"/>
-      <c r="K52" s="109" t="inlineStr">
+      <c r="J49" s="42" t="n"/>
+      <c r="K49" s="109" t="inlineStr">
         <is>
           <t>2026-07-20</t>
         </is>
       </c>
     </row>
+    <row r="50" ht="21.75" customHeight="1" s="49"/>
+    <row r="51" ht="21.75" customHeight="1" s="49"/>
+    <row r="52" ht="21.75" customHeight="1" s="49"/>
     <row r="53" ht="21.75" customHeight="1" s="49"/>
     <row r="54" ht="21.75" customHeight="1" s="49"/>
     <row r="55" ht="21.75" customHeight="1" s="49"/>
@@ -2807,48 +2678,48 @@
     <row r="68" ht="39.75" customHeight="1" s="49"/>
   </sheetData>
   <mergeCells count="39">
-    <mergeCell ref="C47:K47"/>
-    <mergeCell ref="G52:H52"/>
+    <mergeCell ref="C41:K41"/>
     <mergeCell ref="C10:K10"/>
     <mergeCell ref="C15:J15"/>
     <mergeCell ref="C44:K44"/>
     <mergeCell ref="C24:J24"/>
+    <mergeCell ref="I49:J49"/>
     <mergeCell ref="C9:K9"/>
+    <mergeCell ref="C40:K40"/>
     <mergeCell ref="C14:J14"/>
-    <mergeCell ref="C38:I38"/>
-    <mergeCell ref="E52:F52"/>
+    <mergeCell ref="E48:F48"/>
     <mergeCell ref="C43:K43"/>
-    <mergeCell ref="C46:K46"/>
-    <mergeCell ref="E51:F51"/>
-    <mergeCell ref="B50:K50"/>
+    <mergeCell ref="G48:H48"/>
     <mergeCell ref="C20:J20"/>
     <mergeCell ref="B26:K26"/>
+    <mergeCell ref="C36:K36"/>
     <mergeCell ref="C16:J16"/>
-    <mergeCell ref="C48:K48"/>
     <mergeCell ref="B7:K7"/>
-    <mergeCell ref="C39:K39"/>
     <mergeCell ref="C22:J22"/>
     <mergeCell ref="C8:K8"/>
+    <mergeCell ref="B47:K47"/>
     <mergeCell ref="B14:B21"/>
+    <mergeCell ref="G49:H49"/>
     <mergeCell ref="C21:J21"/>
-    <mergeCell ref="C51:D51"/>
+    <mergeCell ref="C35:I35"/>
+    <mergeCell ref="E49:F49"/>
     <mergeCell ref="B12:K12"/>
-    <mergeCell ref="C52:D52"/>
-    <mergeCell ref="I52:J52"/>
+    <mergeCell ref="B39:K39"/>
     <mergeCell ref="B2:K2"/>
-    <mergeCell ref="B42:K42"/>
+    <mergeCell ref="C48:D48"/>
+    <mergeCell ref="I48:J48"/>
     <mergeCell ref="C23:J23"/>
     <mergeCell ref="C17:J17"/>
-    <mergeCell ref="G51:H51"/>
-    <mergeCell ref="I51:J51"/>
     <mergeCell ref="B1:K1"/>
+    <mergeCell ref="C42:K42"/>
     <mergeCell ref="C45:K45"/>
     <mergeCell ref="C13:J13"/>
     <mergeCell ref="C19:J19"/>
+    <mergeCell ref="C49:D49"/>
     <mergeCell ref="C18:J18"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I28:I37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I28:I34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"높음,보통,낮음"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2863,7 +2734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C1:L52"/>
+  <dimension ref="C1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="19.85546875" customWidth="1" style="49" min="3" max="3"/>
@@ -2944,7 +2815,7 @@
         </is>
       </c>
       <c r="D5" s="26">
-        <f>SUMPRODUCT(F12:F21,H12:H21)</f>
+        <f>SUMPRODUCT(F12:F18,H12:H18)</f>
         <v/>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -2962,7 +2833,7 @@
         </is>
       </c>
       <c r="H5" s="119">
-        <f>SUM('01_업무지시서'!J28:J37)</f>
+        <f>SUM('01_업무지시서'!J28:J34)</f>
         <v/>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -2971,7 +2842,7 @@
         </is>
       </c>
       <c r="J5" s="119">
-        <f>SUM(I12:I21)</f>
+        <f>SUM(I12:I18)</f>
         <v/>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -3295,160 +3166,133 @@
       <c r="K18" s="47" t="n"/>
       <c r="L18" s="47" t="n"/>
     </row>
-    <row r="19" ht="27.75" customHeight="1" s="49">
-      <c r="C19" s="17" t="n"/>
-      <c r="D19" s="40">
-        <f>IF('01_업무지시서'!C35="","",'01_업무지시서'!C35)</f>
-        <v/>
-      </c>
-      <c r="E19" s="40">
-        <f>IF('01_업무지시서'!E35="","",'01_업무지시서'!E35)</f>
-        <v/>
-      </c>
-      <c r="F19" s="11">
-        <f>IF('01_업무지시서'!K35="",0,'01_업무지시서'!K35)</f>
-        <v/>
-      </c>
-      <c r="G19" s="47" t="n"/>
-      <c r="H19" s="19" t="n"/>
-      <c r="I19" s="114" t="n"/>
-      <c r="J19" s="47" t="n"/>
-      <c r="K19" s="47" t="n"/>
-      <c r="L19" s="47" t="n"/>
-    </row>
-    <row r="20" ht="27.75" customHeight="1" s="49">
-      <c r="C20" s="17" t="n"/>
-      <c r="D20" s="40">
-        <f>IF('01_업무지시서'!C36="","",'01_업무지시서'!C36)</f>
-        <v/>
-      </c>
-      <c r="E20" s="40">
-        <f>IF('01_업무지시서'!E36="","",'01_업무지시서'!E36)</f>
-        <v/>
-      </c>
-      <c r="F20" s="11">
-        <f>IF('01_업무지시서'!K36="",0,'01_업무지시서'!K36)</f>
-        <v/>
-      </c>
-      <c r="G20" s="47" t="n"/>
-      <c r="H20" s="19" t="n"/>
-      <c r="I20" s="114" t="n"/>
-      <c r="J20" s="47" t="n"/>
-      <c r="K20" s="47" t="n"/>
-      <c r="L20" s="47" t="n"/>
-    </row>
-    <row r="21" ht="27.75" customHeight="1" s="49">
-      <c r="C21" s="17" t="n"/>
-      <c r="D21" s="40">
-        <f>IF('01_업무지시서'!C37="","",'01_업무지시서'!C37)</f>
-        <v/>
-      </c>
-      <c r="E21" s="40">
-        <f>IF('01_업무지시서'!E37="","",'01_업무지시서'!E37)</f>
-        <v/>
-      </c>
-      <c r="F21" s="11">
-        <f>IF('01_업무지시서'!K37="",0,'01_업무지시서'!K37)</f>
-        <v/>
-      </c>
-      <c r="G21" s="47" t="n"/>
-      <c r="H21" s="19" t="n"/>
-      <c r="I21" s="114" t="n"/>
-      <c r="J21" s="47" t="n"/>
-      <c r="K21" s="47" t="n"/>
-      <c r="L21" s="47" t="n"/>
-    </row>
-    <row r="22" ht="15" customHeight="1" s="49">
-      <c r="C22" s="45" t="inlineStr">
+    <row r="19" ht="15" customHeight="1" s="49">
+      <c r="C19" s="45" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="D22" s="45" t="inlineStr">
+      <c r="D19" s="45" t="inlineStr">
         <is>
           <t>가중 달성률 →</t>
         </is>
       </c>
-      <c r="E22" s="42" t="n"/>
-      <c r="F22" s="21">
-        <f>SUM(F12:F21)</f>
-        <v/>
-      </c>
-      <c r="G22" s="28">
-        <f>SUMPRODUCT(F12:F21,H12:H21)</f>
-        <v/>
-      </c>
-      <c r="H22" s="29">
-        <f>COUNTIF(G12:G21,"완료")</f>
-        <v/>
-      </c>
-      <c r="I22" s="115">
-        <f>SUM(I12:I21)</f>
-        <v/>
-      </c>
-      <c r="J22" s="69">
-        <f>"완료 "&amp;COUNTIF(G12:G21,"완료")&amp;"건 / 진행중 "&amp;COUNTIF(G12:G21,"진행중")&amp;"건 / 미착수 "&amp;COUNTIF(G12:G21,"미착수")&amp;"건"</f>
-        <v/>
-      </c>
-      <c r="K22" s="41" t="n"/>
-      <c r="L22" s="42" t="n"/>
+      <c r="E19" s="42" t="n"/>
+      <c r="F19" s="21">
+        <f>SUM(F12:F18)</f>
+        <v/>
+      </c>
+      <c r="G19" s="28">
+        <f>SUMPRODUCT(F12:F18,H12:H18)</f>
+        <v/>
+      </c>
+      <c r="H19" s="29">
+        <f>COUNTIF(G12:G18,"완료")</f>
+        <v/>
+      </c>
+      <c r="I19" s="115">
+        <f>SUM(I12:I18)</f>
+        <v/>
+      </c>
+      <c r="J19" s="69">
+        <f>"완료 "&amp;COUNTIF(G12:G18,"완료")&amp;"건 / 진행중 "&amp;COUNTIF(G12:G18,"진행중")&amp;"건 / 미착수 "&amp;COUNTIF(G12:G18,"미착수")&amp;"건"</f>
+        <v/>
+      </c>
+      <c r="K19" s="41" t="n"/>
+      <c r="L19" s="42" t="n"/>
+    </row>
+    <row r="20" ht="24" customHeight="1" s="49">
+      <c r="C20" s="46" t="n"/>
+      <c r="D20" s="46" t="n"/>
+      <c r="I20" s="46" t="n"/>
+      <c r="J20" s="46" t="n"/>
+      <c r="L20" s="46" t="n"/>
+    </row>
+    <row r="21" ht="19.5" customHeight="1" s="49">
+      <c r="C21" s="121" t="inlineStr">
+        <is>
+          <t>2. 자가 검수  —  제출 전 §4 검수기준으로 본인이 먼저 점검</t>
+        </is>
+      </c>
+      <c r="D21" s="64" t="n"/>
+      <c r="E21" s="64" t="n"/>
+      <c r="F21" s="64" t="n"/>
+      <c r="G21" s="64" t="n"/>
+      <c r="H21" s="64" t="n"/>
+      <c r="I21" s="64" t="n"/>
+      <c r="J21" s="64" t="n"/>
+      <c r="K21" s="64" t="n"/>
+      <c r="L21" s="65" t="n"/>
+    </row>
+    <row r="22" ht="24" customHeight="1" s="49">
+      <c r="C22" s="46" t="inlineStr">
+        <is>
+          <t>검수 항목 (자동)</t>
+        </is>
+      </c>
+      <c r="D22" s="46" t="inlineStr">
+        <is>
+          <t>검수 질문 (자동)</t>
+        </is>
+      </c>
+      <c r="E22" s="41" t="n"/>
+      <c r="F22" s="41" t="n"/>
+      <c r="G22" s="41" t="n"/>
+      <c r="H22" s="42" t="n"/>
+      <c r="I22" s="46" t="inlineStr">
+        <is>
+          <t>자가
+판정</t>
+        </is>
+      </c>
+      <c r="J22" s="46" t="inlineStr">
+        <is>
+          <t>미충족 사유·보완 계획</t>
+        </is>
+      </c>
+      <c r="K22" s="42" t="n"/>
+      <c r="L22" s="46" t="inlineStr">
+        <is>
+          <t>검수자
+판정</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="24" customHeight="1" s="49">
-      <c r="C23" s="46" t="n"/>
-      <c r="D23" s="46" t="n"/>
-      <c r="I23" s="46" t="n"/>
-      <c r="J23" s="46" t="n"/>
-      <c r="L23" s="46" t="n"/>
-    </row>
-    <row r="24" ht="19.5" customHeight="1" s="49">
-      <c r="C24" s="121" t="inlineStr">
-        <is>
-          <t>2. 자가 검수  —  제출 전 §4 검수기준으로 본인이 먼저 점검</t>
-        </is>
-      </c>
-      <c r="D24" s="64" t="n"/>
-      <c r="E24" s="64" t="n"/>
-      <c r="F24" s="64" t="n"/>
-      <c r="G24" s="64" t="n"/>
-      <c r="H24" s="64" t="n"/>
-      <c r="I24" s="64" t="n"/>
-      <c r="J24" s="64" t="n"/>
-      <c r="K24" s="64" t="n"/>
-      <c r="L24" s="65" t="n"/>
+      <c r="C23" s="69" t="n"/>
+      <c r="D23" s="55" t="n"/>
+      <c r="E23" s="41" t="n"/>
+      <c r="F23" s="41" t="n"/>
+      <c r="G23" s="41" t="n"/>
+      <c r="H23" s="42" t="n"/>
+      <c r="I23" s="47" t="n"/>
+      <c r="J23" s="44" t="n"/>
+      <c r="K23" s="42" t="n"/>
+      <c r="L23" s="66" t="n"/>
+    </row>
+    <row r="24" ht="24" customHeight="1" s="49">
+      <c r="C24" s="69" t="n"/>
+      <c r="D24" s="55" t="n"/>
+      <c r="E24" s="41" t="n"/>
+      <c r="F24" s="41" t="n"/>
+      <c r="G24" s="41" t="n"/>
+      <c r="H24" s="42" t="n"/>
+      <c r="I24" s="47" t="n"/>
+      <c r="J24" s="44" t="n"/>
+      <c r="K24" s="42" t="n"/>
+      <c r="L24" s="66" t="n"/>
     </row>
     <row r="25" ht="24" customHeight="1" s="49">
-      <c r="C25" s="46" t="inlineStr">
-        <is>
-          <t>검수 항목 (자동)</t>
-        </is>
-      </c>
-      <c r="D25" s="46" t="inlineStr">
-        <is>
-          <t>검수 질문 (자동)</t>
-        </is>
-      </c>
+      <c r="C25" s="69" t="n"/>
+      <c r="D25" s="55" t="n"/>
       <c r="E25" s="41" t="n"/>
       <c r="F25" s="41" t="n"/>
       <c r="G25" s="41" t="n"/>
       <c r="H25" s="42" t="n"/>
-      <c r="I25" s="46" t="inlineStr">
-        <is>
-          <t>자가
-판정</t>
-        </is>
-      </c>
-      <c r="J25" s="46" t="inlineStr">
-        <is>
-          <t>미충족 사유·보완 계획</t>
-        </is>
-      </c>
+      <c r="I25" s="47" t="n"/>
+      <c r="J25" s="44" t="n"/>
       <c r="K25" s="42" t="n"/>
-      <c r="L25" s="46" t="inlineStr">
-        <is>
-          <t>검수자
-판정</t>
-        </is>
-      </c>
+      <c r="L25" s="66" t="n"/>
     </row>
     <row r="26" ht="24" customHeight="1" s="49">
       <c r="C26" s="69" t="n"/>
@@ -3498,243 +3342,249 @@
       <c r="K29" s="42" t="n"/>
       <c r="L29" s="66" t="n"/>
     </row>
-    <row r="30" ht="24" customHeight="1" s="49">
-      <c r="C30" s="69" t="n"/>
-      <c r="D30" s="55" t="n"/>
-      <c r="E30" s="41" t="n"/>
-      <c r="F30" s="41" t="n"/>
-      <c r="G30" s="41" t="n"/>
-      <c r="H30" s="42" t="n"/>
-      <c r="I30" s="47" t="n"/>
-      <c r="J30" s="44" t="n"/>
-      <c r="K30" s="42" t="n"/>
-      <c r="L30" s="66" t="n"/>
-    </row>
-    <row r="31" ht="24" customHeight="1" s="49">
-      <c r="C31" s="69" t="n"/>
-      <c r="D31" s="55" t="n"/>
-      <c r="E31" s="41" t="n"/>
-      <c r="F31" s="41" t="n"/>
-      <c r="G31" s="41" t="n"/>
-      <c r="H31" s="42" t="n"/>
-      <c r="I31" s="47" t="n"/>
-      <c r="J31" s="44" t="n"/>
-      <c r="K31" s="42" t="n"/>
-      <c r="L31" s="66" t="n"/>
-    </row>
-    <row r="32" ht="24" customHeight="1" s="49">
-      <c r="C32" s="69" t="n"/>
-      <c r="D32" s="55" t="n"/>
-      <c r="E32" s="41" t="n"/>
-      <c r="F32" s="41" t="n"/>
-      <c r="G32" s="41" t="n"/>
-      <c r="H32" s="42" t="n"/>
-      <c r="I32" s="47" t="n"/>
-      <c r="J32" s="44" t="n"/>
-      <c r="K32" s="42" t="n"/>
-      <c r="L32" s="66" t="n"/>
-    </row>
-    <row r="33" ht="27.75" customHeight="1" s="49">
-      <c r="C33" s="46" t="n"/>
-      <c r="D33" s="46" t="n"/>
-      <c r="E33" s="46" t="n"/>
-      <c r="F33" s="46" t="n"/>
-      <c r="G33" s="46" t="n"/>
-      <c r="H33" s="46" t="n"/>
-      <c r="I33" s="46" t="n"/>
-      <c r="J33" s="46" t="n"/>
-      <c r="K33" s="46" t="n"/>
-      <c r="L33" s="46" t="n"/>
-    </row>
-    <row r="34" ht="19.5" customHeight="1" s="49">
-      <c r="C34" s="121" t="inlineStr">
+    <row r="30" ht="27.75" customHeight="1" s="49">
+      <c r="C30" s="46" t="n"/>
+      <c r="D30" s="46" t="n"/>
+      <c r="E30" s="46" t="n"/>
+      <c r="F30" s="46" t="n"/>
+      <c r="G30" s="46" t="n"/>
+      <c r="H30" s="46" t="n"/>
+      <c r="I30" s="46" t="n"/>
+      <c r="J30" s="46" t="n"/>
+      <c r="K30" s="46" t="n"/>
+      <c r="L30" s="46" t="n"/>
+    </row>
+    <row r="31" ht="19.5" customHeight="1" s="49">
+      <c r="C31" s="121" t="inlineStr">
         <is>
           <t>3. 이슈 및 지원요청  —  대안 없이 문제만 올리는 보고는 반려</t>
         </is>
       </c>
-      <c r="D34" s="64" t="n"/>
-      <c r="E34" s="64" t="n"/>
-      <c r="F34" s="64" t="n"/>
-      <c r="G34" s="64" t="n"/>
-      <c r="H34" s="64" t="n"/>
-      <c r="I34" s="64" t="n"/>
-      <c r="J34" s="64" t="n"/>
-      <c r="K34" s="64" t="n"/>
-      <c r="L34" s="65" t="n"/>
-    </row>
-    <row r="35" ht="27.75" customHeight="1" s="49">
-      <c r="C35" s="46" t="inlineStr">
+      <c r="D31" s="64" t="n"/>
+      <c r="E31" s="64" t="n"/>
+      <c r="F31" s="64" t="n"/>
+      <c r="G31" s="64" t="n"/>
+      <c r="H31" s="64" t="n"/>
+      <c r="I31" s="64" t="n"/>
+      <c r="J31" s="64" t="n"/>
+      <c r="K31" s="64" t="n"/>
+      <c r="L31" s="65" t="n"/>
+    </row>
+    <row r="32" ht="27.75" customHeight="1" s="49">
+      <c r="C32" s="46" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="D35" s="46" t="inlineStr">
+      <c r="D32" s="46" t="inlineStr">
         <is>
           <t>이슈 내용</t>
         </is>
       </c>
-      <c r="E35" s="46" t="inlineStr">
+      <c r="E32" s="46" t="inlineStr">
         <is>
           <t>영향
 (일정/비용/품질)</t>
         </is>
       </c>
-      <c r="F35" s="46" t="inlineStr">
+      <c r="F32" s="46" t="inlineStr">
         <is>
           <t>근본 원인</t>
         </is>
       </c>
-      <c r="G35" s="46" t="inlineStr">
+      <c r="G32" s="46" t="inlineStr">
         <is>
           <t>대안 1</t>
         </is>
       </c>
-      <c r="H35" s="46" t="inlineStr">
+      <c r="H32" s="46" t="inlineStr">
         <is>
           <t>대안 2</t>
         </is>
       </c>
-      <c r="I35" s="46" t="inlineStr">
+      <c r="I32" s="46" t="inlineStr">
         <is>
           <t>권고안</t>
         </is>
       </c>
-      <c r="J35" s="46" t="inlineStr">
+      <c r="J32" s="46" t="inlineStr">
         <is>
           <t>요청사항</t>
         </is>
       </c>
-      <c r="K35" s="46" t="inlineStr">
+      <c r="K32" s="46" t="inlineStr">
         <is>
           <t>결정기한</t>
         </is>
       </c>
-      <c r="L35" s="46" t="inlineStr">
+      <c r="L32" s="46" t="inlineStr">
         <is>
           <t>대표 결정</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="36" customHeight="1" s="49">
-      <c r="C36" s="6" t="n"/>
-      <c r="D36" s="18" t="n"/>
-      <c r="E36" s="6" t="n"/>
-      <c r="F36" s="18" t="n"/>
-      <c r="G36" s="18" t="n"/>
-      <c r="H36" s="18" t="n"/>
-      <c r="I36" s="18" t="n"/>
-      <c r="J36" s="18" t="n"/>
-      <c r="K36" s="6" t="n"/>
-      <c r="L36" s="66" t="n"/>
-    </row>
-    <row r="37" ht="36" customHeight="1" s="49">
-      <c r="C37" s="6" t="n"/>
-      <c r="D37" s="18" t="n"/>
-      <c r="E37" s="6" t="n"/>
-      <c r="F37" s="18" t="n"/>
-      <c r="G37" s="18" t="n"/>
-      <c r="H37" s="18" t="n"/>
-      <c r="I37" s="18" t="n"/>
-      <c r="J37" s="18" t="n"/>
-      <c r="K37" s="6" t="n"/>
-      <c r="L37" s="66" t="n"/>
-    </row>
-    <row r="38" ht="36" customHeight="1" s="49">
-      <c r="C38" s="6" t="n"/>
-      <c r="D38" s="18" t="n"/>
-      <c r="E38" s="6" t="n"/>
-      <c r="F38" s="18" t="n"/>
-      <c r="G38" s="18" t="n"/>
-      <c r="H38" s="18" t="n"/>
-      <c r="I38" s="18" t="n"/>
-      <c r="J38" s="18" t="n"/>
-      <c r="K38" s="6" t="n"/>
-      <c r="L38" s="66" t="n"/>
-    </row>
-    <row r="39" ht="27.75" customHeight="1" s="49">
-      <c r="C39" s="13" t="n"/>
-      <c r="D39" s="46" t="n"/>
-      <c r="E39" s="46" t="n"/>
-      <c r="F39" s="46" t="n"/>
-      <c r="G39" s="46" t="n"/>
-      <c r="H39" s="46" t="n"/>
-      <c r="I39" s="46" t="n"/>
-      <c r="J39" s="46" t="n"/>
-      <c r="K39" s="46" t="n"/>
-      <c r="L39" s="46" t="n"/>
-    </row>
-    <row r="40" ht="19.5" customHeight="1" s="49">
-      <c r="C40" s="121" t="inlineStr">
+    <row r="33" ht="36" customHeight="1" s="49">
+      <c r="C33" s="6" t="n"/>
+      <c r="D33" s="18" t="n"/>
+      <c r="E33" s="6" t="n"/>
+      <c r="F33" s="18" t="n"/>
+      <c r="G33" s="18" t="n"/>
+      <c r="H33" s="18" t="n"/>
+      <c r="I33" s="18" t="n"/>
+      <c r="J33" s="18" t="n"/>
+      <c r="K33" s="6" t="n"/>
+      <c r="L33" s="66" t="n"/>
+    </row>
+    <row r="34" ht="36" customHeight="1" s="49">
+      <c r="C34" s="6" t="n"/>
+      <c r="D34" s="18" t="n"/>
+      <c r="E34" s="6" t="n"/>
+      <c r="F34" s="18" t="n"/>
+      <c r="G34" s="18" t="n"/>
+      <c r="H34" s="18" t="n"/>
+      <c r="I34" s="18" t="n"/>
+      <c r="J34" s="18" t="n"/>
+      <c r="K34" s="6" t="n"/>
+      <c r="L34" s="66" t="n"/>
+    </row>
+    <row r="35" ht="36" customHeight="1" s="49">
+      <c r="C35" s="6" t="n"/>
+      <c r="D35" s="18" t="n"/>
+      <c r="E35" s="6" t="n"/>
+      <c r="F35" s="18" t="n"/>
+      <c r="G35" s="18" t="n"/>
+      <c r="H35" s="18" t="n"/>
+      <c r="I35" s="18" t="n"/>
+      <c r="J35" s="18" t="n"/>
+      <c r="K35" s="6" t="n"/>
+      <c r="L35" s="66" t="n"/>
+    </row>
+    <row r="36" ht="27.75" customHeight="1" s="49">
+      <c r="C36" s="13" t="n"/>
+      <c r="D36" s="46" t="n"/>
+      <c r="E36" s="46" t="n"/>
+      <c r="F36" s="46" t="n"/>
+      <c r="G36" s="46" t="n"/>
+      <c r="H36" s="46" t="n"/>
+      <c r="I36" s="46" t="n"/>
+      <c r="J36" s="46" t="n"/>
+      <c r="K36" s="46" t="n"/>
+      <c r="L36" s="46" t="n"/>
+    </row>
+    <row r="37" ht="19.5" customHeight="1" s="49">
+      <c r="C37" s="121" t="inlineStr">
         <is>
           <t>4. 다음 주 제안 업무  —  지시를 기다리지 말 것. 본인이 먼저 제안.</t>
         </is>
       </c>
-      <c r="D40" s="64" t="n"/>
-      <c r="E40" s="64" t="n"/>
-      <c r="F40" s="64" t="n"/>
-      <c r="G40" s="64" t="n"/>
-      <c r="H40" s="64" t="n"/>
-      <c r="I40" s="64" t="n"/>
-      <c r="J40" s="64" t="n"/>
-      <c r="K40" s="64" t="n"/>
-      <c r="L40" s="65" t="n"/>
-    </row>
-    <row r="41" ht="27.75" customHeight="1" s="49">
-      <c r="C41" s="13" t="inlineStr">
+      <c r="D37" s="64" t="n"/>
+      <c r="E37" s="64" t="n"/>
+      <c r="F37" s="64" t="n"/>
+      <c r="G37" s="64" t="n"/>
+      <c r="H37" s="64" t="n"/>
+      <c r="I37" s="64" t="n"/>
+      <c r="J37" s="64" t="n"/>
+      <c r="K37" s="64" t="n"/>
+      <c r="L37" s="65" t="n"/>
+    </row>
+    <row r="38" ht="27.75" customHeight="1" s="49">
+      <c r="C38" s="13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D41" s="46" t="inlineStr">
+      <c r="D38" s="46" t="inlineStr">
         <is>
           <t>제안 업무</t>
         </is>
       </c>
-      <c r="E41" s="46" t="inlineStr">
+      <c r="E38" s="46" t="inlineStr">
         <is>
           <t>왜 해야 하는가</t>
         </is>
       </c>
-      <c r="F41" s="46" t="inlineStr">
+      <c r="F38" s="46" t="inlineStr">
         <is>
           <t>완료기준(안)</t>
         </is>
       </c>
-      <c r="G41" s="46" t="inlineStr">
+      <c r="G38" s="46" t="inlineStr">
         <is>
           <t>예상
 소요(h)</t>
         </is>
       </c>
-      <c r="H41" s="46" t="inlineStr">
+      <c r="H38" s="46" t="inlineStr">
         <is>
           <t>우선순위(안)</t>
         </is>
       </c>
-      <c r="I41" s="46" t="inlineStr">
+      <c r="I38" s="46" t="inlineStr">
         <is>
           <t>선행 조건</t>
         </is>
       </c>
-      <c r="J41" s="46" t="inlineStr">
+      <c r="J38" s="46" t="inlineStr">
         <is>
           <t>필요 지원</t>
         </is>
       </c>
-      <c r="K41" s="46" t="inlineStr">
+      <c r="K38" s="46" t="inlineStr">
         <is>
           <t>대표 승인</t>
         </is>
       </c>
-      <c r="L41" s="46" t="inlineStr">
+      <c r="L38" s="46" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
+    </row>
+    <row r="39" ht="31.5" customHeight="1" s="49">
+      <c r="C39" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="18" t="n"/>
+      <c r="E39" s="18" t="n"/>
+      <c r="F39" s="18" t="n"/>
+      <c r="G39" s="114" t="n"/>
+      <c r="H39" s="6" t="n"/>
+      <c r="I39" s="18" t="n"/>
+      <c r="J39" s="18" t="n"/>
+      <c r="K39" s="66" t="n"/>
+      <c r="L39" s="6" t="n"/>
+    </row>
+    <row r="40" ht="31.5" customHeight="1" s="49">
+      <c r="C40" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" s="18" t="n"/>
+      <c r="E40" s="18" t="n"/>
+      <c r="F40" s="18" t="n"/>
+      <c r="G40" s="114" t="n"/>
+      <c r="H40" s="6" t="n"/>
+      <c r="I40" s="18" t="n"/>
+      <c r="J40" s="18" t="n"/>
+      <c r="K40" s="66" t="n"/>
+      <c r="L40" s="6" t="n"/>
+    </row>
+    <row r="41" ht="31.5" customHeight="1" s="49">
+      <c r="C41" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" s="18" t="n"/>
+      <c r="E41" s="18" t="n"/>
+      <c r="F41" s="18" t="n"/>
+      <c r="G41" s="114" t="n"/>
+      <c r="H41" s="6" t="n"/>
+      <c r="I41" s="18" t="n"/>
+      <c r="J41" s="18" t="n"/>
+      <c r="K41" s="66" t="n"/>
+      <c r="L41" s="6" t="n"/>
     </row>
     <row r="42" ht="31.5" customHeight="1" s="49">
       <c r="C42" s="22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D42" s="18" t="n"/>
       <c r="E42" s="18" t="n"/>
@@ -3746,198 +3596,156 @@
       <c r="K42" s="66" t="n"/>
       <c r="L42" s="6" t="n"/>
     </row>
-    <row r="43" ht="31.5" customHeight="1" s="49">
-      <c r="C43" s="22" t="n">
-        <v>2</v>
-      </c>
-      <c r="D43" s="18" t="n"/>
-      <c r="E43" s="18" t="n"/>
-      <c r="F43" s="18" t="n"/>
-      <c r="G43" s="114" t="n"/>
-      <c r="H43" s="6" t="n"/>
-      <c r="I43" s="18" t="n"/>
-      <c r="J43" s="18" t="n"/>
-      <c r="K43" s="66" t="n"/>
-      <c r="L43" s="6" t="n"/>
-    </row>
-    <row r="44" ht="31.5" customHeight="1" s="49">
-      <c r="C44" s="22" t="n">
-        <v>3</v>
-      </c>
-      <c r="D44" s="18" t="n"/>
-      <c r="E44" s="18" t="n"/>
-      <c r="F44" s="18" t="n"/>
-      <c r="G44" s="114" t="n"/>
-      <c r="H44" s="6" t="n"/>
-      <c r="I44" s="18" t="n"/>
-      <c r="J44" s="18" t="n"/>
-      <c r="K44" s="66" t="n"/>
-      <c r="L44" s="6" t="n"/>
-    </row>
-    <row r="45" ht="31.5" customHeight="1" s="49">
-      <c r="C45" s="22" t="n">
-        <v>4</v>
-      </c>
-      <c r="D45" s="18" t="n"/>
-      <c r="E45" s="18" t="n"/>
-      <c r="F45" s="18" t="n"/>
-      <c r="G45" s="114" t="n"/>
-      <c r="H45" s="6" t="n"/>
-      <c r="I45" s="18" t="n"/>
-      <c r="J45" s="18" t="n"/>
-      <c r="K45" s="66" t="n"/>
-      <c r="L45" s="6" t="n"/>
+    <row r="43" ht="25.5" customHeight="1" s="49">
+      <c r="C43" s="45" t="n"/>
+      <c r="D43" s="43" t="n"/>
+      <c r="J43" s="58" t="n"/>
+    </row>
+    <row r="44" ht="19.5" customHeight="1" s="49">
+      <c r="C44" s="48" t="inlineStr">
+        <is>
+          <t>5. 자기점검 및 대표 검수</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="25.5" customHeight="1" s="49">
+      <c r="C45" s="45" t="inlineStr">
+        <is>
+          <t>이번 주 가장 잘한 것</t>
+        </is>
+      </c>
+      <c r="D45" s="43" t="inlineStr">
+        <is>
+          <t>결과로 증명되는 것 1개만</t>
+        </is>
+      </c>
+      <c r="E45" s="41" t="n"/>
+      <c r="F45" s="41" t="n"/>
+      <c r="G45" s="41" t="n"/>
+      <c r="H45" s="41" t="n"/>
+      <c r="I45" s="42" t="n"/>
+      <c r="J45" s="58" t="inlineStr">
+        <is>
+          <t>[대표 검수 의견]</t>
+        </is>
+      </c>
+      <c r="K45" s="59" t="n"/>
+      <c r="L45" s="60" t="n"/>
     </row>
     <row r="46" ht="25.5" customHeight="1" s="49">
-      <c r="C46" s="45" t="n"/>
-      <c r="D46" s="43" t="n"/>
-      <c r="J46" s="58" t="n"/>
-    </row>
-    <row r="47" ht="19.5" customHeight="1" s="49">
-      <c r="C47" s="48" t="inlineStr">
-        <is>
-          <t>5. 자기점검 및 대표 검수</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="25.5" customHeight="1" s="49">
-      <c r="C48" s="45" t="inlineStr">
-        <is>
-          <t>이번 주 가장 잘한 것</t>
-        </is>
-      </c>
-      <c r="D48" s="43" t="inlineStr">
-        <is>
-          <t>결과로 증명되는 것 1개만</t>
-        </is>
-      </c>
-      <c r="E48" s="41" t="n"/>
-      <c r="F48" s="41" t="n"/>
-      <c r="G48" s="41" t="n"/>
-      <c r="H48" s="41" t="n"/>
-      <c r="I48" s="42" t="n"/>
-      <c r="J48" s="58" t="inlineStr">
-        <is>
-          <t>[대표 검수 의견]</t>
-        </is>
-      </c>
-      <c r="K48" s="59" t="n"/>
-      <c r="L48" s="60" t="n"/>
-    </row>
-    <row r="49" ht="25.5" customHeight="1" s="49">
+      <c r="C46" s="45" t="inlineStr">
+        <is>
+          <t>이번 주 가장 부족한 것</t>
+        </is>
+      </c>
+      <c r="D46" s="43" t="inlineStr">
+        <is>
+          <t>변명 말고 사실만</t>
+        </is>
+      </c>
+      <c r="E46" s="41" t="n"/>
+      <c r="F46" s="41" t="n"/>
+      <c r="G46" s="41" t="n"/>
+      <c r="H46" s="41" t="n"/>
+      <c r="I46" s="42" t="n"/>
+      <c r="J46" s="61" t="n"/>
+      <c r="L46" s="62" t="n"/>
+    </row>
+    <row r="47" ht="25.5" customHeight="1" s="49">
+      <c r="C47" s="45" t="inlineStr">
+        <is>
+          <t>다음 주 개선 액션 1개</t>
+        </is>
+      </c>
+      <c r="D47" s="43" t="inlineStr">
+        <is>
+          <t>실행 가능한 행동으로</t>
+        </is>
+      </c>
+      <c r="E47" s="41" t="n"/>
+      <c r="F47" s="41" t="n"/>
+      <c r="G47" s="41" t="n"/>
+      <c r="H47" s="41" t="n"/>
+      <c r="I47" s="42" t="n"/>
+      <c r="J47" s="63" t="n"/>
+      <c r="K47" s="64" t="n"/>
+      <c r="L47" s="65" t="n"/>
+    </row>
+    <row r="49" ht="33.75" customHeight="1" s="49">
       <c r="C49" s="45" t="inlineStr">
         <is>
-          <t>이번 주 가장 부족한 것</t>
-        </is>
-      </c>
-      <c r="D49" s="43" t="inlineStr">
-        <is>
-          <t>변명 말고 사실만</t>
-        </is>
-      </c>
+          <t>제출자</t>
+        </is>
+      </c>
+      <c r="D49" s="47" t="n"/>
       <c r="E49" s="41" t="n"/>
-      <c r="F49" s="41" t="n"/>
-      <c r="G49" s="41" t="n"/>
-      <c r="H49" s="41" t="n"/>
+      <c r="F49" s="42" t="n"/>
+      <c r="G49" s="45" t="inlineStr">
+        <is>
+          <t>검수자</t>
+        </is>
+      </c>
+      <c r="H49" s="66" t="n"/>
       <c r="I49" s="42" t="n"/>
-      <c r="J49" s="61" t="n"/>
-      <c r="L49" s="62" t="n"/>
-    </row>
-    <row r="50" ht="25.5" customHeight="1" s="49">
-      <c r="C50" s="45" t="inlineStr">
-        <is>
-          <t>다음 주 개선 액션 1개</t>
-        </is>
-      </c>
-      <c r="D50" s="43" t="inlineStr">
-        <is>
-          <t>실행 가능한 행동으로</t>
-        </is>
-      </c>
-      <c r="E50" s="41" t="n"/>
-      <c r="F50" s="41" t="n"/>
-      <c r="G50" s="41" t="n"/>
-      <c r="H50" s="41" t="n"/>
-      <c r="I50" s="42" t="n"/>
-      <c r="J50" s="63" t="n"/>
-      <c r="K50" s="64" t="n"/>
-      <c r="L50" s="65" t="n"/>
-    </row>
-    <row r="52" ht="33.75" customHeight="1" s="49">
-      <c r="C52" s="45" t="inlineStr">
-        <is>
-          <t>제출자</t>
-        </is>
-      </c>
-      <c r="D52" s="47" t="n"/>
-      <c r="E52" s="41" t="n"/>
-      <c r="F52" s="42" t="n"/>
-      <c r="G52" s="45" t="inlineStr">
-        <is>
-          <t>검수자</t>
-        </is>
-      </c>
-      <c r="H52" s="66" t="n"/>
-      <c r="I52" s="42" t="n"/>
-      <c r="J52" s="45" t="inlineStr">
+      <c r="J49" s="45" t="inlineStr">
         <is>
           <t>최종 판정</t>
         </is>
       </c>
-      <c r="K52" s="56" t="n"/>
-      <c r="L52" s="42" t="n"/>
+      <c r="K49" s="56" t="n"/>
+      <c r="L49" s="42" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="D49:I49"/>
+    <mergeCell ref="K49:L49"/>
     <mergeCell ref="J29:K29"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="D48:I48"/>
+    <mergeCell ref="D19:E19"/>
     <mergeCell ref="J28:K28"/>
-    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="D47:I47"/>
     <mergeCell ref="D7:L7"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="J22:L22"/>
+    <mergeCell ref="C37:L37"/>
+    <mergeCell ref="J45:L47"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="H49:I49"/>
     <mergeCell ref="D27:H27"/>
-    <mergeCell ref="C34:L34"/>
     <mergeCell ref="J27:K27"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="C24:L24"/>
-    <mergeCell ref="H52:I52"/>
     <mergeCell ref="J26:K26"/>
-    <mergeCell ref="K52:L52"/>
-    <mergeCell ref="J32:K32"/>
     <mergeCell ref="J25:K25"/>
     <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D50:I50"/>
-    <mergeCell ref="J31:K31"/>
-    <mergeCell ref="C47:L47"/>
-    <mergeCell ref="J48:L50"/>
+    <mergeCell ref="J22:K22"/>
     <mergeCell ref="C1:L1"/>
-    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="C44:L44"/>
     <mergeCell ref="D25:H25"/>
-    <mergeCell ref="C40:L40"/>
+    <mergeCell ref="C31:L31"/>
+    <mergeCell ref="D46:I46"/>
     <mergeCell ref="C9:L9"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="J19:L19"/>
     <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D52:F52"/>
+    <mergeCell ref="C21:L21"/>
+    <mergeCell ref="D45:I45"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="J23:K23"/>
     <mergeCell ref="C2:L2"/>
     <mergeCell ref="D6:L6"/>
+    <mergeCell ref="D49:F49"/>
     <mergeCell ref="D26:H26"/>
   </mergeCells>
   <dataValidations count="5">
-    <dataValidation sqref="I26:I32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I23:I29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"충족,미충족"</formula1>
     </dataValidation>
-    <dataValidation sqref="L26:L32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L23:L29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"합격,보완,불합격"</formula1>
     </dataValidation>
-    <dataValidation sqref="K42:K45 L36:L38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K39:K42 L33:L35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"승인,보류,반려"</formula1>
     </dataValidation>
-    <dataValidation sqref="K52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"합격,조건부합격,보완요청,불합격"</formula1>
     </dataValidation>
-    <dataValidation sqref="G12:G21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G12:G18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"완료,진행중,미착수,보류,취소"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Rework 황우중 W30 as report-first plan (안 A), cooperative tone
Report-body draft as top-priority task (weight 38%); fold guide
reconciliation into task 1 with plain-language wording; tables/figures
deliverable switched to PPT; imperative phrasing changed to
cooperative-request tone; add '최우선' to priority dropdown.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPtt2MinYXH5T7wMFXyfVt
</commit_message>
<xml_diff>
--- a/out/BRING_주간_황우중_2026-W30.xlsx
+++ b/out/BRING_주간_황우중_2026-W30.xlsx
@@ -1544,7 +1544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:K49"/>
+  <dimension ref="B1:K47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="24.7109375" customWidth="1" style="49" min="2" max="2"/>
@@ -1693,8 +1693,9 @@
       </c>
       <c r="C8" s="70" t="inlineStr">
         <is>
-          <t>TRL 1 연구개발보고서에서 대표가 제1장(기술개발 방향·연구개발 목표)을 확정하였다. 최상위 기준은 '노후 소형건축물 입구 1개소'를 초기 적용대상으로 하는 Scan-to-Fit 리트로핏 MVP이며, 표준 프레임+맞춤형 공차보정 연결부, 탈부착형 기능 카세트, BIM–BOM–제작도면 연계, 공장 사전제작·현장 건식설치, FM·Building Passport 연계를 핵심 축으로 한다.
-기존 작성 가이드에는 방 1개·창호 1~2개 중심 MVP와 센서·창호 중심 표현이 다수 남아 있어 제1장 확정 방향과 정합되지 않는다. 이번 주에는 후속 작성의 1차로, 제1장 확정 MVP를 기준으로 보고서 본문(문제정의~시스템·제품구조)을 구체화한다.</t>
+          <t>대표가 제1장에서 회사의 기술개발 방향을 확정하였습니다. 확정된 방향은 '노후 소형건축물의 입구 1개소'를 처음 적용 대상으로 하여, 현장을 3D로 실측하고 그 형상에 맞춰 표준 프레임과 맞춤형 연결부, 탈부착이 가능한 기능 카세트를 공장에서 미리 만들어 현장에 조립·설치하는 리트로핏(개선) 기술입니다.
+다만 예전에 만들어 둔 TRL1 보고서 작성 가이드는 '방 1개·창문 1~2개'와 센서 중심으로 쓰여 있어, 지금 확정된 '건물 입구' 방향과 맞지 않는 부분이 많습니다. 이 상태로 본문을 쓰면 옛 방향(방·창문)이 그대로 섞여 나옵니다.
+따라서 이번 주에는 이 보고서의 본문을 실제로 쓰는 일을 최우선으로 하고, 거기서 나온 내용이 나머지 산출물(표·그림·연구가설·위험요소 등)로 이어지도록 진행합니다.</t>
         </is>
       </c>
       <c r="D8" s="41" t="n"/>
@@ -1715,7 +1716,7 @@
       </c>
       <c r="C9" s="73" t="inlineStr">
         <is>
-          <t>제1장에서 확정된 입구 1개소 중심 Scan-to-Fit 리트로핏 MVP를 기준으로, 연구개발보고서 본문(문제정의·기술개념·연구가설·시스템/제품 구조)을 검증 가능한 연구논리로 구체화한다.</t>
+          <t>제1장에서 확정된 '건물 입구 1개소' 중심 리트로핏 방향을 기준으로 TRL1 연구개발보고서의 본문을 작성하고, 그 내용을 뒷받침하는 표·그림·연구가설·위험요소를 함께 정리하는 것입니다.</t>
         </is>
       </c>
       <c r="D9" s="41" t="n"/>
@@ -1736,7 +1737,7 @@
       </c>
       <c r="C10" s="73" t="inlineStr">
         <is>
-          <t>입구 MVP 기준으로 정합되지 않으면 이후 전 장이 방·창호 중심 표현과 뒤섞여 보고서 전체 논리가 흔들린다. 문제·원인·기술논리·검증계획의 연결이 확보되지 않으면 TRL 2 개념검증 계획과 1:1 목업·시제품 일정이 연쇄 지연되고 재작성 부담이 발생한다.</t>
+          <t>보고서가 옛 방향(방·창문)과 섞이면, 이후 모든 장의 논리가 흔들리고 다시 써야 합니다. 또한 문제→기술→구조→검증으로 이어지는 논리가 정리되지 않으면, 다음 단계(TRL2)의 개념검증·시제품 일정이 함께 미뤄지고 재작업 부담이 커집니다.</t>
         </is>
       </c>
       <c r="D10" s="41" t="n"/>
@@ -1787,7 +1788,7 @@
       </c>
       <c r="C14" s="111" t="inlineStr">
         <is>
-          <t>제1장 확정 MVP(입구 1개소·Scan-to-Fit·표준 프레임+맞춤 공차보정 연결부·탈부착 기능 카세트·BIM–BOM–제작도면·공장 사전제작·현장 건식설치·FM/Building Passport) 기준 정합</t>
+          <t>제1장에서 확정된 '건물 입구 1개소' 중심 방향을 최상위 기준으로 삼아 진행</t>
         </is>
       </c>
       <c r="D14" s="41" t="n"/>
@@ -1807,7 +1808,7 @@
       <c r="B15" s="112" t="n"/>
       <c r="C15" s="111" t="inlineStr">
         <is>
-          <t>기존 가이드의 방·창호·외벽 중심 표현을 입구 1개소 MVP 기준으로 최신화</t>
+          <t>예전 작성 가이드의 '방·창문·외벽' 중심 표현을 '건물 입구' 기준으로 고쳐 맞춘 뒤 본문 작성</t>
         </is>
       </c>
       <c r="D15" s="41" t="n"/>
@@ -1823,7 +1824,7 @@
       <c r="B16" s="112" t="n"/>
       <c r="C16" s="111" t="inlineStr">
         <is>
-          <t>입구 현장 문제·기존 공정 비효율·기존 기술 한계 분석 및 핵심 문제 정의</t>
+          <t>TRL1 연구개발보고서 본문(문제 정의 → 기술 개념 → 시스템·제품 구조) 초안 작성</t>
         </is>
       </c>
       <c r="D16" s="41" t="n"/>
@@ -1839,7 +1840,7 @@
       <c r="B17" s="112" t="n"/>
       <c r="C17" s="111" t="inlineStr">
         <is>
-          <t>입구 리트로핏 기술개념·전체 흐름 정립</t>
+          <t>본문을 뒷받침하는 핵심 표·그림을 발표용 슬라이드(PPT)로 제작</t>
         </is>
       </c>
       <c r="D17" s="41" t="n"/>
@@ -1855,7 +1856,7 @@
       <c r="B18" s="112" t="n"/>
       <c r="C18" s="111" t="inlineStr">
         <is>
-          <t>연구가설 설정 및 개념검증 논리 수립</t>
+          <t>연구가설과 다음 단계 검증계획 정리</t>
         </is>
       </c>
       <c r="D18" s="41" t="n"/>
@@ -1871,7 +1872,7 @@
       <c r="B19" s="112" t="n"/>
       <c r="C19" s="113" t="inlineStr">
         <is>
-          <t>시스템·제품 구조 및 데이터 흐름 설계 초안 정립</t>
+          <t>위험요소와 나중에 측정할 성능지표 후보 정리</t>
         </is>
       </c>
       <c r="D19" s="41" t="n"/>
@@ -1887,7 +1888,7 @@
       <c r="B20" s="112" t="n"/>
       <c r="C20" s="111" t="inlineStr">
         <is>
-          <t>필수 산출물·미확인 가정·대표 검토 쟁점·용어 정리</t>
+          <t>확인되지 않은 가정·대표 검토가 필요한 쟁점·용어 정리</t>
         </is>
       </c>
       <c r="D20" s="41" t="n"/>
@@ -1919,10 +1920,10 @@
       </c>
       <c r="C22" s="105" t="inlineStr">
         <is>
-          <t>· 센서·창호·외벽 중심 상세 설계 (후속 확장범위로만 구분 표기)
-· 제10장 시장·사업화, 제11장 경제성의 단독 확정 (기술자료·초안 지원까지만)
-· 모듈러주택 전체 구조체
-· 성능 달성값·정량 절감률 확정 (TRL 2 후보지표로만 제시)</t>
+          <t>· 센서·창문·외벽 중심의 상세 설계 (지금은 '후속 확장범위'로만 표기)
+· 시장·사업화 전략, 수익·가격 산정의 단독 확정 (기술 자료·초안 지원까지만)
+· 모듈러주택 전체 구조
+· 성능 달성값·구체 절감률의 확정 (다음 단계에서 측정할 '후보 지표'로만 제시)</t>
         </is>
       </c>
       <c r="D22" s="41" t="n"/>
@@ -1946,11 +1947,11 @@
       </c>
       <c r="C23" s="105" t="inlineStr">
         <is>
-          <t>· 제1장(대표 확정) 기술개발 방향·연구개발 목표를 최상위 기준으로 삼을 것
-· TRL 1 수준 유지: 문제 관찰·기술원리·시스템 개념·연구가설·적용/제외조건·후보 성능지표·TRL 2 계획까지만 작성
-· '성능 달성·스마트공장 구축·자동설계 완성·원가 절감 완료·센서만으로 원인 확정' 등 달성형 표현 금지
-· 서술은 □핵심주제 / ○세부주제 / •현황·원인·기술필요성·대응방향·TRL1 정립사항 구조로 작성
-· 첨부 가이드는 참고자료이며 입구 MVP와 상충 시 입구 MVP 우선</t>
+          <t>· 제1장(대표 확정)의 방향과 목표를 최상위 기준으로 삼습니다
+· TRL1 단계에 맞춰, 문제 관찰·기술 원리·개념 정의·연구가설·적용/제외 조건·후보 성능지표·다음 단계 계획까지만 작성합니다
+· '이미 성능을 달성했다 / 스마트공장을 지금 구축한다 / 자동설계가 완성됐다 / 원가를 이미 절감했다'와 같은 완성형 표현은 지양해 주시기 바랍니다
+· 서술은 □ 큰 주제 / ○ 세부 주제 / • 현황·원인·필요성·대응방향·이번 단계 정립사항 순서로 정리해 주시면 읽기 쉽습니다
+· 첨부된 예전 가이드는 참고자료이며, 입구 방향과 다를 경우 입구 방향을 우선합니다</t>
         </is>
       </c>
       <c r="D23" s="41" t="n"/>
@@ -1974,7 +1975,7 @@
       </c>
       <c r="C24" s="102" t="inlineStr">
         <is>
-          <t>제1장 확정 MVP와 상충하거나 TRL 1 수준을 넘는 작성이 필요하면 변경 사유·영향을 문서화하여 대표 승인 후 반영할 것.</t>
+          <t>작성 중 제1장 방향과 맞지 않거나 TRL1 범위를 넘는 판단이 필요하면, 사유와 영향을 간단히 적어 대표와 상의 후 진행해 주시기 바랍니다.</t>
         </is>
       </c>
       <c r="D24" s="41" t="n"/>
@@ -2068,25 +2069,25 @@
       </c>
       <c r="C28" s="47" t="inlineStr">
         <is>
-          <t>기존 TRL 1 작성 가이드를 입구 1개소 MVP 기준으로 최신화하라</t>
+          <t>TRL1 보고서 본문 초안 작성  (이번 주 최우선)</t>
         </is>
       </c>
       <c r="D28" s="47" t="inlineStr">
         <is>
-          <t>대표가 확정한 입구 1개소 Scan-to-Fit 리트로핏 MVP를 최상위 기준으로, 가이드 전반의 방·창호·외벽 중심 표현을 입구 기준으로 수정하고 적용범위를 확정한다.</t>
+          <t>보고서를 쓰기 전에, 예전 작성 가이드에서 '방·창문·외벽' 기준으로 된 부분을 지금 확정된 '건물 입구' 기준으로 먼저 고쳐 맞춘 뒤, 핵심 문제와 연구가설을 정하고 본문을 하나의 논리로 작성해 주시면 됩니다.</t>
         </is>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>① 가이드 내 방·창호·외벽 중심 표현 위치를 전수 식별한 목록을 작성할 것
-② 기존→수정 대조표를 작성할 것
-③ 초기 MVP / 후속 확장범위(센서·창호·외벽) 구분표를 작성할 것
-④ 기술 중심축(현장·고객조사→입구 3D실측→As-is BIM→문제분석→To-be 기획→Scan-to-Fit→표준/맞춤 분리→BIM–BOM–제작도면→공장 사전제작→현장 건식설치→검증→FM/Building Passport) 흐름도 1개를 확정할 것</t>
+          <t>① 예전 가이드에서 '방·창문·외벽'으로 된 표현을 찾아 '건물 입구' 기준으로 어떻게 바꿀지 대조표(위치 / 기존 표현 / 수정 표현 / 초기적용·후속확장 구분)로 먼저 정리해 주시면 됩니다.
+② 보고서 전체가 답할 '핵심 문제 한 문장'과 그 아래 세부 문제들을 먼저 확정해 주시면 됩니다.
+③ 이어서 본문 초안을 (가)문제 정의 (나)기술 개념·전체 흐름 (다)시스템·제품 구조 순서로, 서로 연결되게 작성해 주시면 됩니다.
+④ 아직 확인되지 않은 성능·효과는 '이미 달성'이 아니라 '다음 단계(TRL2)에서 확인할 항목'으로 적어 주시면 됩니다.</t>
         </is>
       </c>
       <c r="F28" s="47" t="inlineStr">
         <is>
-          <t>01_황우중_가이드최신화_W30_v1.xlsx</t>
+          <t>01_황우중_TRL1보고서_본문초안_W30_v1.docx</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
@@ -2096,19 +2097,19 @@
       </c>
       <c r="H28" s="107" t="inlineStr">
         <is>
-          <t>07-21(화) 12:00</t>
+          <t>07-24(금) 12:00</t>
         </is>
       </c>
       <c r="I28" s="47" t="inlineStr">
         <is>
-          <t>높음</t>
+          <t>최우선</t>
         </is>
       </c>
       <c r="J28" s="114" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>0.12</v>
+        <v>0.38</v>
       </c>
     </row>
     <row r="29" ht="123" customHeight="1" s="49">
@@ -2117,25 +2118,24 @@
       </c>
       <c r="C29" s="47" t="inlineStr">
         <is>
-          <t>노후건축물 입구 현장의 문제와 기존 공정의 비효율을 분석하라</t>
+          <t>연구가설·다음 단계 검증계획 정리</t>
         </is>
       </c>
       <c r="D29" s="47" t="inlineStr">
         <is>
-          <t>노후 소형건축물 입구·공용부의 구조와 간섭요소를 분석해 표준제품을 그대로 적용하기 어려운 근거를 도출하고, 기존 실측·기획·제작·설치 공정의 비효율을 분석한다.</t>
+          <t>본문에서 세운 '이렇게 하면 이런 효과가 있을 것이다'라는 가정(연구가설)을, 나중에 어떻게 확인할지(검증방법)와 짝지어 표로 정리해 주시면 됩니다. 지금은 증명이 아니라 '무엇을 어떻게 확인할지 계획'까지만 정리하면 됩니다.</t>
         </is>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>① 입구 구성요소·간섭요소·구조체 체결 가능 위치 분류표를 작성할 것
-② 벽면 요철·바닥 경사·단차·벽체 기울기 등 시공오차 요인을 정리할 것
-③ 기존 공정 흐름도(현장방문→실측→기획→개별도면→재실측→주문제작→현장 절단·천공·용접→설치→재작업)를 작성할 것
-④ 비효율 8항목 분석표를 작성하고 표준제품 적용 곤란 근거를 서술할 것</t>
+          <t>① 연구가설을 6개 이상 정리해 주시면 됩니다 (예: 디지털 실측으로 재방문·치수 누락을 줄일 수 있다 / 표준부품과 맞춤부품을 나누면 반복 제작이 쉬워진다 등).
+② 가설마다 [가설 / 그렇게 보는 근거 / 확인할 데이터 / 다음 단계 확인방법 / 예상 산출물]을 한 줄로 정리해 주시면 됩니다.
+③ '전부 맞춤제작 / 전부 표준화 / 섞어서(혼합)' 세 방식을 비교한 표를 함께 넣어 주시면 됩니다.</t>
         </is>
       </c>
       <c r="F29" s="47" t="inlineStr">
         <is>
-          <t>02_황우중_입구문제_공정분석_W30_v1.pdf</t>
+          <t>02_황우중_연구가설_검증계획_W30_v1.xlsx</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="H29" s="107" t="inlineStr">
         <is>
-          <t>07-22(수) 18:00</t>
+          <t>07-24(금) 15:00</t>
         </is>
       </c>
       <c r="I29" s="47" t="inlineStr">
@@ -2166,25 +2166,24 @@
       </c>
       <c r="C30" s="47" t="inlineStr">
         <is>
-          <t>기존 기술을 비교하고 브링이 해결할 핵심 문제를 정의하라</t>
+          <t>핵심 표·그림 패키지 제작 (발표용 PPT)</t>
         </is>
       </c>
       <c r="D30" s="47" t="inlineStr">
         <is>
-          <t>관련 기존 기술을 비교해 입구 리트로핏 적용 한계와 브링의 보완지점을 도출하고, 보고서 전체의 핵심 문제를 한 문장으로 고정한다.</t>
+          <t>보고서 본문의 근거가 되는 핵심 표와 그림을, 회의·발표에서 바로 쓸 수 있도록 PPT 슬라이드로 만들어 주시면 됩니다. 글은 최소로 하고 표·그림 위주로 한 장에 한 가지 메시지가 보이게 해 주시면 됩니다.</t>
         </is>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>① 기존 기술 8종(현장 인테리어·리모델링/프리패브·OSC/모듈러 신축/Scan-to-BIM/파라메트릭 설계/3D프린팅/시설관리 앱/BIM·디지털트윈 FM) 비교표(해결문제·강점·입구적용 한계·브링 보완방향)를 작성할 것
-② 핵심 문제문장 1개를 확정할 것
-③ 하위 7개 문제 분해도를 작성할 것
-④ 각 하위문제의 근거를 정리할 것</t>
+          <t>① 다음 6종을 각각 슬라이드로 만들어 주시면 됩니다: 입구 구조 분류 / 기존 공정의 비효율 / 기존 기술 비교 / 핵심 문제 구조 / 기술 개념 흐름도 / 초기 적용범위와 후속 확장범위.
+② 한 장에 하나의 메시지가 보이도록 정리해 주시면 됩니다.
+③ 각 장에 제목·범례·출처를 표기해 주시면 됩니다.</t>
         </is>
       </c>
       <c r="F30" s="47" t="inlineStr">
         <is>
-          <t>03_황우중_기술비교_핵심문제_W30_v1.xlsx</t>
+          <t>03_황우중_핵심표그림_발표자료_W30_v1.pptx</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -2194,7 +2193,7 @@
       </c>
       <c r="H30" s="107" t="inlineStr">
         <is>
-          <t>07-22(수) 18:00</t>
+          <t>07-24(금) 15:00</t>
         </is>
       </c>
       <c r="I30" s="47" t="inlineStr">
@@ -2203,10 +2202,10 @@
         </is>
       </c>
       <c r="J30" s="114" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="31" ht="90" customHeight="1" s="49">
@@ -2215,24 +2214,24 @@
       </c>
       <c r="C31" s="47" t="inlineStr">
         <is>
-          <t>입구 리트로핏 기술개념과 전체 흐름을 정립하라</t>
+          <t>위험요소·후보 성능지표 정리</t>
         </is>
       </c>
       <c r="D31" s="47" t="inlineStr">
         <is>
-          <t>입구 조사부터 FM 등록까지의 기술흐름을 개념 수준에서 정의하고 각 단계 입출력을 정리한다.</t>
+          <t>이 기술을 실제로 만들 때 생길 수 있는 위험과, 나중에 성능을 어떤 숫자로 확인할지 후보 지표를 정리해 주시면 됩니다. 지금은 목표 숫자를 확정하는 게 아니라 '무엇을 측정할지'만 정하면 됩니다.</t>
         </is>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>① 기술 개념 흐름도(입구 현장조사→형상·공차 실측→As-is BIM→문제분석→To-be 기획→Scan-to-Fit 설계→표준 프레임 선정→맞춤 연결부 설계→기능 카세트 조합→BOM·제작도면→공장 사전제작·조립→현장 건식설치→품질·탈착 검증→FM/Building Passport 등록)를 작성할 것
-② 각 단계 입력·출력을 정의할 것
-③ 초기 MVP·후속 확장범위 표를 작성할 것</t>
+          <t>① 위험요소를 4개 분야(기술 / 제조 / 현장·운영 / 사업 확장)로 나눠 [위험 / 원인 / 영향 / 예방·대응]으로 정리해 주시면 됩니다.
+② 나중에 측정할 성능지표 후보 목록을 정리해 주시면 됩니다 (예: 실측 시간·오차, 설치 시간, 현장 추가가공 횟수, 부품 교체 가능 여부 등).
+③ 각 지표는 '목표값 확정'이 아니라 '다음 단계에서 측정'으로 표기해 주시면 됩니다.</t>
         </is>
       </c>
       <c r="F31" s="47" t="inlineStr">
         <is>
-          <t>04_황우중_기술개념_흐름정립_W30_v1.pdf</t>
+          <t>04_황우중_위험요소_성능지표_W30_v1.pdf</t>
         </is>
       </c>
       <c r="G31" s="108" t="inlineStr">
@@ -2242,19 +2241,19 @@
       </c>
       <c r="H31" s="107" t="inlineStr">
         <is>
-          <t>07-23(목) 18:00</t>
+          <t>07-24(금) 17:00</t>
         </is>
       </c>
       <c r="I31" s="47" t="inlineStr">
         <is>
-          <t>높음</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="J31" s="114" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K31" s="19" t="n">
-        <v>0.12</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="32" ht="69" customHeight="1" s="49">
@@ -2263,25 +2262,24 @@
       </c>
       <c r="C32" s="47" t="inlineStr">
         <is>
-          <t>연구가설을 설정하고 개념검증 논리를 수립하라</t>
+          <t>미확인 가정·대표 검토 쟁점·용어 정리</t>
         </is>
       </c>
       <c r="D32" s="47" t="inlineStr">
         <is>
-          <t>각 기술요소의 필요성을 인과관계로 설명하고 검증 가능한 연구가설로 전환한다.</t>
+          <t>아직 확실하지 않아 대표 판단이 필요한 부분과, 혼자 정하면 안 되는 쟁점을 따로 모아 주시고, 보고서에 쓰인 용어·약어도 정리해 주시면 됩니다.</t>
         </is>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>① 연구가설 6개 이상(디지털 실측/BIM 기반 기획-제작 연계/표준·맞춤 분리 반복성/공장 사전조립 작업·재작업 절감/탈부착 카세트 부분교체·기능추가/Building Passport 이력관리)을 설정할 것
-② 가설별 표(연구가설/논리적 근거/확인할 데이터/TRL 2 검증방법/예상 산출물)를 작성할 것
-③ 완전주문제작·완전표준화·혼합생산 비교표를 작성할 것
-④ 기술요소별 필요성 표를 작성할 것</t>
+          <t>① 아직 확인되지 않은 가정 목록을 정리해 주시면 됩니다.
+② 대표 검토·결정이 필요한 쟁점 목록을 정리해 주시면 됩니다.
+③ 용어 정의·약어 목록과 참고자료 출처를 정리해 주시면 됩니다.</t>
         </is>
       </c>
       <c r="F32" s="47" t="inlineStr">
         <is>
-          <t>05_황우중_연구가설_검증논리_W30_v1.xlsx</t>
+          <t>05_황우중_가정_쟁점_용어정리_W30_v1.pdf</t>
         </is>
       </c>
       <c r="G32" s="108" t="inlineStr">
@@ -2291,187 +2289,122 @@
       </c>
       <c r="H32" s="107" t="inlineStr">
         <is>
-          <t>07-23(목) 18:00</t>
+          <t>07-24(금) 17:00</t>
         </is>
       </c>
       <c r="I32" s="47" t="inlineStr">
         <is>
-          <t>높음</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="J32" s="114" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>0.16</v>
-      </c>
-    </row>
-    <row r="33" ht="90" customHeight="1" s="49">
-      <c r="B33" s="17" t="n"/>
-      <c r="C33" s="47" t="inlineStr">
-        <is>
-          <t>시스템·제품 구조와 데이터 흐름을 설계 초안으로 정립하라</t>
-        </is>
-      </c>
-      <c r="D33" s="47" t="inlineStr">
-        <is>
-          <t>TRL 1 수준에서 시스템을 5~6개 모듈로 정리하고 혼합생산형 입구 리트로핏 구조를 개념안으로 도출한다.</t>
-        </is>
-      </c>
-      <c r="E33" s="1" t="inlineStr">
-        <is>
-          <t>① 모듈 5~6개 정의표(역할/입력/처리/출력/HW/SW/수행주체/초기MVP 포함여부/후속확장)를 작성할 것
-② 구성방식 6후보 비교표(현장적합성·제작난이도·원가·표준화·운송·설치·탈착·확장성·스마트공장 연계)를 작성할 것
-③ 최적 구조 선정 근거표(혼합생산형 입구 리트로핏 — TRL 2에서 변경 가능한 개념안)를 작성할 것
-④ 전체 시스템 구성도·제품 분해구조도(표준 프레임–맞춤 연결부–기능 카세트)·데이터 흐름도(BIM–BOM–제작도면–부품ID–FM)를 작성할 것</t>
-        </is>
-      </c>
-      <c r="F33" s="47" t="inlineStr">
-        <is>
-          <t>06_황우중_시스템제품구조_초안_W30_v1.pdf</t>
-        </is>
-      </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>브링 구글 드라이브</t>
-        </is>
-      </c>
-      <c r="H33" s="107" t="inlineStr">
-        <is>
-          <t>07-24(금) 15:00</t>
-        </is>
-      </c>
-      <c r="I33" s="47" t="inlineStr">
-        <is>
-          <t>높음</t>
-        </is>
-      </c>
-      <c r="J33" s="114" t="n">
-        <v>7</v>
-      </c>
-      <c r="K33" s="19" t="n">
-        <v>0.16</v>
-      </c>
-    </row>
-    <row r="34" ht="90" customHeight="1" s="49">
-      <c r="B34" s="17" t="n"/>
-      <c r="C34" s="47" t="inlineStr">
-        <is>
-          <t>필수 산출물을 완비하고 미확인 가정·검토 쟁점·용어를 정리하여 제출하라</t>
-        </is>
-      </c>
-      <c r="D34" s="47" t="inlineStr">
-        <is>
-          <t>제2장 필수 산출물을 완비하고 TRL 1 단계에서 확정되지 않은 가정과 대표 검토가 필요한 쟁점을 분리 정리한다.</t>
-        </is>
-      </c>
-      <c r="E34" s="1" t="inlineStr">
-        <is>
-          <t>① 필수 산출물 6종(입구 구조 분류표/기존 공정 비효율표/기존 기술 비교표/핵심 문제 분해도/기술개념 흐름도/초기 MVP·후속확장 표)을 완비할 것
-② 확인되지 않은 가정 목록을 작성할 것
-③ 대표 검토가 필요한 쟁점 목록을 작성할 것
-④ 용어정의·약어목록·참고문헌 초안을 제출할 것</t>
-        </is>
-      </c>
-      <c r="F34" s="47" t="inlineStr">
-        <is>
-          <t>07_황우중_산출물_쟁점_용어정리_W30_v1.pdf</t>
-        </is>
-      </c>
-      <c r="G34" s="6" t="inlineStr">
-        <is>
-          <t>브링 구글 드라이브</t>
-        </is>
-      </c>
-      <c r="H34" s="107" t="inlineStr">
-        <is>
-          <t>07-24(금) 17:00</t>
-        </is>
-      </c>
-      <c r="I34" s="47" t="inlineStr">
-        <is>
-          <t>보통</t>
-        </is>
-      </c>
-      <c r="J34" s="114" t="n">
-        <v>4</v>
-      </c>
-      <c r="K34" s="19" t="n">
         <v>0.14</v>
       </c>
     </row>
-    <row r="35" ht="69" customHeight="1" s="49">
-      <c r="B35" s="45" t="inlineStr">
+    <row r="33" ht="69" customHeight="1" s="49">
+      <c r="B33" s="45" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="C35" s="51" t="n"/>
-      <c r="D35" s="41" t="n"/>
-      <c r="E35" s="41" t="n"/>
-      <c r="F35" s="41" t="n"/>
-      <c r="G35" s="41" t="n"/>
-      <c r="H35" s="41" t="n"/>
-      <c r="I35" s="42" t="n"/>
-      <c r="J35" s="115">
-        <f>SUM(J28:J34)</f>
-        <v/>
-      </c>
-      <c r="K35" s="21">
-        <f>SUM(K28:K34)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="24" customHeight="1" s="49">
-      <c r="B36" s="45" t="inlineStr">
+      <c r="C33" s="51" t="n"/>
+      <c r="D33" s="41" t="n"/>
+      <c r="E33" s="41" t="n"/>
+      <c r="F33" s="41" t="n"/>
+      <c r="G33" s="41" t="n"/>
+      <c r="H33" s="41" t="n"/>
+      <c r="I33" s="42" t="n"/>
+      <c r="J33" s="115">
+        <f>SUM(J28:J32)</f>
+        <v/>
+      </c>
+      <c r="K33" s="21">
+        <f>SUM(K28:K32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="24" customHeight="1" s="49">
+      <c r="B34" s="45" t="inlineStr">
         <is>
           <t>발행 검증</t>
         </is>
       </c>
-      <c r="C36" s="116">
-        <f>IF(COUNTA(C28:C34)=0,"업무 미입력",IF(COUNTA(E28:E34)&lt;COUNTA(C28:C34),"발행 불가 — 완료기준 누락 업무 있음",IF(COUNTA(F28:F34)&lt;COUNTA(C28:C34),"발행 불가 — 산출물 누락 업무 있음",IF(SUM(K28:K34)&lt;&gt;1,"발행 불가 — 가중치 합계 "&amp;TEXT(SUM(K28:K34),"0%")&amp;" (100% 필요)","발행 가능 — 완료기준·산출물·가중치 충족"))))</f>
-        <v/>
-      </c>
-      <c r="D36" s="41" t="n"/>
-      <c r="E36" s="41" t="n"/>
-      <c r="F36" s="41" t="n"/>
-      <c r="G36" s="41" t="n"/>
-      <c r="H36" s="41" t="n"/>
-      <c r="I36" s="41" t="n"/>
-      <c r="J36" s="41" t="n"/>
-      <c r="K36" s="42" t="n"/>
-    </row>
-    <row r="37" ht="24" customHeight="1" s="49">
-      <c r="B37" s="89" t="n"/>
-    </row>
-    <row r="38" ht="24" customHeight="1" s="49">
-      <c r="B38" s="45" t="n"/>
-      <c r="C38" s="117" t="n"/>
-    </row>
-    <row r="39" ht="18" customHeight="1" s="49">
-      <c r="B39" s="89" t="inlineStr">
+      <c r="C34" s="116">
+        <f>IF(COUNTA(C28:C32)=0,"업무 미입력",IF(COUNTA(E28:E32)&lt;COUNTA(C28:C32),"발행 불가 — 완료기준 누락 업무 있음",IF(COUNTA(F28:F32)&lt;COUNTA(C28:C32),"발행 불가 — 산출물 누락 업무 있음",IF(SUM(K28:K32)&lt;&gt;1,"발행 불가 — 가중치 합계 "&amp;TEXT(SUM(K28:K32),"0%")&amp;" (100% 필요)","발행 가능 — 완료기준·산출물·가중치 충족"))))</f>
+        <v/>
+      </c>
+      <c r="D34" s="41" t="n"/>
+      <c r="E34" s="41" t="n"/>
+      <c r="F34" s="41" t="n"/>
+      <c r="G34" s="41" t="n"/>
+      <c r="H34" s="41" t="n"/>
+      <c r="I34" s="41" t="n"/>
+      <c r="J34" s="41" t="n"/>
+      <c r="K34" s="42" t="n"/>
+    </row>
+    <row r="35" ht="24" customHeight="1" s="49"/>
+    <row r="36" ht="24" customHeight="1" s="49"/>
+    <row r="37" ht="18" customHeight="1" s="49">
+      <c r="B37" s="89" t="inlineStr">
         <is>
           <t>담당자 접수확인  —  월요일 12:00까지 담당자 직접 작성 (미작성 = 업무 미이해로 간주, 재지시)</t>
         </is>
       </c>
-      <c r="C39" s="64" t="n"/>
-      <c r="D39" s="64" t="n"/>
-      <c r="E39" s="64" t="n"/>
-      <c r="F39" s="64" t="n"/>
-      <c r="G39" s="64" t="n"/>
-      <c r="H39" s="64" t="n"/>
-      <c r="I39" s="64" t="n"/>
-      <c r="J39" s="64" t="n"/>
-      <c r="K39" s="64" t="n"/>
-    </row>
-    <row r="40" ht="36" customHeight="1" s="49">
-      <c r="B40" s="45" t="inlineStr">
+      <c r="C37" s="64" t="n"/>
+      <c r="D37" s="64" t="n"/>
+      <c r="E37" s="64" t="n"/>
+      <c r="F37" s="64" t="n"/>
+      <c r="G37" s="64" t="n"/>
+      <c r="H37" s="64" t="n"/>
+      <c r="I37" s="64" t="n"/>
+      <c r="J37" s="64" t="n"/>
+      <c r="K37" s="64" t="n"/>
+    </row>
+    <row r="38" ht="36" customHeight="1" s="49">
+      <c r="B38" s="45" t="inlineStr">
         <is>
           <t>내가 이해한 업무
 (본인 언어로 재작성)</t>
         </is>
       </c>
-      <c r="C40" s="117" t="n"/>
+      <c r="C38" s="117" t="n"/>
+      <c r="D38" s="41" t="n"/>
+      <c r="E38" s="41" t="n"/>
+      <c r="F38" s="41" t="n"/>
+      <c r="G38" s="41" t="n"/>
+      <c r="H38" s="41" t="n"/>
+      <c r="I38" s="41" t="n"/>
+      <c r="J38" s="41" t="n"/>
+      <c r="K38" s="42" t="n"/>
+    </row>
+    <row r="39" ht="19.5" customHeight="1" s="49">
+      <c r="B39" s="45" t="inlineStr">
+        <is>
+          <t>완료기준 재확인
+(무엇이 되면 끝인가)</t>
+        </is>
+      </c>
+      <c r="C39" s="118" t="n"/>
+      <c r="D39" s="41" t="n"/>
+      <c r="E39" s="41" t="n"/>
+      <c r="F39" s="41" t="n"/>
+      <c r="G39" s="41" t="n"/>
+      <c r="H39" s="41" t="n"/>
+      <c r="I39" s="41" t="n"/>
+      <c r="J39" s="41" t="n"/>
+      <c r="K39" s="42" t="n"/>
+    </row>
+    <row r="40" ht="24" customHeight="1" s="49">
+      <c r="B40" s="45" t="inlineStr">
+        <is>
+          <t>예상 리스크
+(막힐 것 같은 지점)</t>
+        </is>
+      </c>
+      <c r="C40" s="43" t="n"/>
       <c r="D40" s="41" t="n"/>
       <c r="E40" s="41" t="n"/>
       <c r="F40" s="41" t="n"/>
@@ -2481,14 +2414,13 @@
       <c r="J40" s="41" t="n"/>
       <c r="K40" s="42" t="n"/>
     </row>
-    <row r="41" ht="19.5" customHeight="1" s="49">
+    <row r="41" ht="24" customHeight="1" s="49">
       <c r="B41" s="45" t="inlineStr">
         <is>
-          <t>완료기준 재확인
-(무엇이 되면 끝인가)</t>
-        </is>
-      </c>
-      <c r="C41" s="118" t="n"/>
+          <t>필요한 지원·의사결정</t>
+        </is>
+      </c>
+      <c r="C41" s="43" t="n"/>
       <c r="D41" s="41" t="n"/>
       <c r="E41" s="41" t="n"/>
       <c r="F41" s="41" t="n"/>
@@ -2501,8 +2433,7 @@
     <row r="42" ht="24" customHeight="1" s="49">
       <c r="B42" s="45" t="inlineStr">
         <is>
-          <t>예상 리스크
-(막힐 것 같은 지점)</t>
+          <t>실행 계획 (요일 배분)</t>
         </is>
       </c>
       <c r="C42" s="43" t="n"/>
@@ -2518,10 +2449,10 @@
     <row r="43" ht="24" customHeight="1" s="49">
       <c r="B43" s="45" t="inlineStr">
         <is>
-          <t>필요한 지원·의사결정</t>
-        </is>
-      </c>
-      <c r="C43" s="43" t="n"/>
+          <t>접수 확인 일시 / 서명</t>
+        </is>
+      </c>
+      <c r="C43" s="47" t="n"/>
       <c r="D43" s="41" t="n"/>
       <c r="E43" s="41" t="n"/>
       <c r="F43" s="41" t="n"/>
@@ -2531,29 +2462,14 @@
       <c r="J43" s="41" t="n"/>
       <c r="K43" s="42" t="n"/>
     </row>
-    <row r="44" ht="24" customHeight="1" s="49">
-      <c r="B44" s="45" t="inlineStr">
-        <is>
-          <t>실행 계획 (요일 배분)</t>
-        </is>
-      </c>
-      <c r="C44" s="43" t="n"/>
-      <c r="D44" s="41" t="n"/>
-      <c r="E44" s="41" t="n"/>
-      <c r="F44" s="41" t="n"/>
-      <c r="G44" s="41" t="n"/>
-      <c r="H44" s="41" t="n"/>
-      <c r="I44" s="41" t="n"/>
-      <c r="J44" s="41" t="n"/>
-      <c r="K44" s="42" t="n"/>
-    </row>
+    <row r="44" ht="24" customHeight="1" s="49"/>
     <row r="45" ht="24" customHeight="1" s="49">
-      <c r="B45" s="45" t="inlineStr">
-        <is>
-          <t>접수 확인 일시 / 서명</t>
-        </is>
-      </c>
-      <c r="C45" s="47" t="n"/>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>결   재</t>
+        </is>
+      </c>
+      <c r="C45" s="41" t="n"/>
       <c r="D45" s="41" t="n"/>
       <c r="E45" s="41" t="n"/>
       <c r="F45" s="41" t="n"/>
@@ -2564,101 +2480,79 @@
       <c r="K45" s="42" t="n"/>
     </row>
     <row r="46" ht="24" customHeight="1" s="49">
-      <c r="B46" s="45" t="n"/>
-      <c r="C46" s="45" t="n"/>
-      <c r="E46" s="45" t="n"/>
-      <c r="G46" s="45" t="n"/>
-      <c r="I46" s="45" t="n"/>
-      <c r="K46" s="45" t="n"/>
-    </row>
-    <row r="47" ht="24" customHeight="1" s="49">
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>결   재</t>
-        </is>
-      </c>
-      <c r="C47" s="41" t="n"/>
-      <c r="D47" s="41" t="n"/>
-      <c r="E47" s="41" t="n"/>
-      <c r="F47" s="41" t="n"/>
-      <c r="G47" s="41" t="n"/>
-      <c r="H47" s="41" t="n"/>
-      <c r="I47" s="41" t="n"/>
-      <c r="J47" s="41" t="n"/>
-      <c r="K47" s="42" t="n"/>
-    </row>
-    <row r="48" ht="24" customHeight="1" s="49">
-      <c r="B48" s="45" t="inlineStr">
+      <c r="B46" s="45" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="C48" s="45" t="inlineStr">
+      <c r="C46" s="45" t="inlineStr">
         <is>
           <t>작성 (지시자)</t>
         </is>
       </c>
-      <c r="D48" s="42" t="n"/>
-      <c r="E48" s="45" t="inlineStr">
+      <c r="D46" s="42" t="n"/>
+      <c r="E46" s="45" t="inlineStr">
         <is>
           <t>검토 (검수자)</t>
         </is>
       </c>
-      <c r="F48" s="42" t="n"/>
-      <c r="G48" s="45" t="inlineStr">
+      <c r="F46" s="42" t="n"/>
+      <c r="G46" s="45" t="inlineStr">
         <is>
           <t>승인 (대표)</t>
         </is>
       </c>
-      <c r="H48" s="42" t="n"/>
-      <c r="I48" s="45" t="inlineStr">
+      <c r="H46" s="42" t="n"/>
+      <c r="I46" s="45" t="inlineStr">
         <is>
           <t>접수 (담당자)</t>
         </is>
       </c>
-      <c r="J48" s="42" t="n"/>
-      <c r="K48" s="45" t="inlineStr">
+      <c r="J46" s="42" t="n"/>
+      <c r="K46" s="45" t="inlineStr">
         <is>
           <t>일자</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="21.75" customHeight="1" s="49">
-      <c r="B49" s="45" t="inlineStr">
+    <row r="47">
+      <c r="B47" s="45" t="inlineStr">
         <is>
           <t>서명</t>
         </is>
       </c>
-      <c r="C49" s="47" t="inlineStr">
+      <c r="C47" s="47" t="inlineStr">
         <is>
           <t>서 창 환</t>
         </is>
       </c>
-      <c r="D49" s="42" t="n"/>
-      <c r="E49" s="47" t="inlineStr">
+      <c r="D47" s="42" t="n"/>
+      <c r="E47" s="47" t="inlineStr">
         <is>
           <t>서 창 환</t>
         </is>
       </c>
-      <c r="F49" s="42" t="n"/>
-      <c r="G49" s="47" t="inlineStr">
+      <c r="F47" s="42" t="n"/>
+      <c r="G47" s="47" t="inlineStr">
         <is>
           <t>서 창 환</t>
         </is>
       </c>
-      <c r="H49" s="42" t="n"/>
-      <c r="I49" s="47" t="inlineStr">
+      <c r="H47" s="42" t="n"/>
+      <c r="I47" s="47" t="inlineStr">
         <is>
           <t>황 우 중</t>
         </is>
       </c>
-      <c r="J49" s="42" t="n"/>
-      <c r="K49" s="109" t="inlineStr">
+      <c r="J47" s="42" t="n"/>
+      <c r="K47" s="109" t="inlineStr">
         <is>
           <t>2026-07-20</t>
         </is>
       </c>
     </row>
+    <row r="48" ht="19.5" customHeight="1" s="49"/>
+    <row r="49" ht="21.75" customHeight="1" s="49"/>
     <row r="50" ht="21.75" customHeight="1" s="49"/>
     <row r="51" ht="21.75" customHeight="1" s="49"/>
     <row r="52" ht="21.75" customHeight="1" s="49"/>
@@ -2678,49 +2572,49 @@
     <row r="68" ht="39.75" customHeight="1" s="49"/>
   </sheetData>
   <mergeCells count="39">
+    <mergeCell ref="C10:K10"/>
     <mergeCell ref="C41:K41"/>
-    <mergeCell ref="C10:K10"/>
     <mergeCell ref="C15:J15"/>
-    <mergeCell ref="C44:K44"/>
+    <mergeCell ref="I46:J46"/>
     <mergeCell ref="C24:J24"/>
-    <mergeCell ref="I49:J49"/>
+    <mergeCell ref="C40:K40"/>
     <mergeCell ref="C9:K9"/>
-    <mergeCell ref="C40:K40"/>
     <mergeCell ref="C14:J14"/>
-    <mergeCell ref="E48:F48"/>
     <mergeCell ref="C43:K43"/>
-    <mergeCell ref="G48:H48"/>
+    <mergeCell ref="B45:K45"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="I47:J47"/>
     <mergeCell ref="C20:J20"/>
     <mergeCell ref="B26:K26"/>
-    <mergeCell ref="C36:K36"/>
     <mergeCell ref="C16:J16"/>
     <mergeCell ref="B7:K7"/>
+    <mergeCell ref="C39:K39"/>
+    <mergeCell ref="C8:K8"/>
     <mergeCell ref="C22:J22"/>
-    <mergeCell ref="C8:K8"/>
-    <mergeCell ref="B47:K47"/>
+    <mergeCell ref="C33:I33"/>
     <mergeCell ref="B14:B21"/>
-    <mergeCell ref="G49:H49"/>
+    <mergeCell ref="C38:K38"/>
+    <mergeCell ref="C46:D46"/>
     <mergeCell ref="C21:J21"/>
-    <mergeCell ref="C35:I35"/>
-    <mergeCell ref="E49:F49"/>
+    <mergeCell ref="E46:F46"/>
     <mergeCell ref="B12:K12"/>
-    <mergeCell ref="B39:K39"/>
     <mergeCell ref="B2:K2"/>
-    <mergeCell ref="C48:D48"/>
-    <mergeCell ref="I48:J48"/>
+    <mergeCell ref="C34:K34"/>
     <mergeCell ref="C23:J23"/>
     <mergeCell ref="C17:J17"/>
     <mergeCell ref="B1:K1"/>
+    <mergeCell ref="G47:H47"/>
     <mergeCell ref="C42:K42"/>
-    <mergeCell ref="C45:K45"/>
+    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="C19:J19"/>
     <mergeCell ref="C13:J13"/>
-    <mergeCell ref="C19:J19"/>
-    <mergeCell ref="C49:D49"/>
     <mergeCell ref="C18:J18"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="B37:K37"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I28:I34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"높음,보통,낮음"</formula1>
+    <dataValidation sqref="I28:I32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"최우선,높음,보통,낮음"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2734,7 +2628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C1:L49"/>
+  <dimension ref="C1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="19.85546875" customWidth="1" style="49" min="3" max="3"/>
@@ -2815,7 +2709,7 @@
         </is>
       </c>
       <c r="D5" s="26">
-        <f>SUMPRODUCT(F12:F18,H12:H18)</f>
+        <f>SUMPRODUCT(F12:F16,H12:H16)</f>
         <v/>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -2833,7 +2727,7 @@
         </is>
       </c>
       <c r="H5" s="119">
-        <f>SUM('01_업무지시서'!J28:J34)</f>
+        <f>SUM('01_업무지시서'!J28:J32)</f>
         <v/>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -2842,7 +2736,7 @@
         </is>
       </c>
       <c r="J5" s="119">
-        <f>SUM(I12:I18)</f>
+        <f>SUM(I12:I16)</f>
         <v/>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -3124,139 +3018,121 @@
       <c r="K16" s="47" t="n"/>
       <c r="L16" s="47" t="n"/>
     </row>
-    <row r="17" ht="27.75" customHeight="1" s="49">
-      <c r="C17" s="17" t="n"/>
-      <c r="D17" s="40">
-        <f>IF('01_업무지시서'!C33="","",'01_업무지시서'!C33)</f>
-        <v/>
-      </c>
-      <c r="E17" s="40">
-        <f>IF('01_업무지시서'!E33="","",'01_업무지시서'!E33)</f>
-        <v/>
-      </c>
-      <c r="F17" s="11">
-        <f>IF('01_업무지시서'!K33="",0,'01_업무지시서'!K33)</f>
-        <v/>
-      </c>
-      <c r="G17" s="47" t="n"/>
-      <c r="H17" s="19" t="n"/>
-      <c r="I17" s="114" t="n"/>
-      <c r="J17" s="47" t="n"/>
-      <c r="K17" s="47" t="n"/>
-      <c r="L17" s="47" t="n"/>
-    </row>
-    <row r="18" ht="27.75" customHeight="1" s="49">
-      <c r="C18" s="17" t="n"/>
-      <c r="D18" s="40">
-        <f>IF('01_업무지시서'!C34="","",'01_업무지시서'!C34)</f>
-        <v/>
-      </c>
-      <c r="E18" s="40">
-        <f>IF('01_업무지시서'!E34="","",'01_업무지시서'!E34)</f>
-        <v/>
-      </c>
-      <c r="F18" s="11">
-        <f>IF('01_업무지시서'!K34="",0,'01_업무지시서'!K34)</f>
-        <v/>
-      </c>
-      <c r="G18" s="47" t="n"/>
-      <c r="H18" s="19" t="n"/>
-      <c r="I18" s="114" t="n"/>
-      <c r="J18" s="47" t="n"/>
-      <c r="K18" s="47" t="n"/>
-      <c r="L18" s="47" t="n"/>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="49">
-      <c r="C19" s="45" t="inlineStr">
+    <row r="17" ht="15" customHeight="1" s="49">
+      <c r="C17" s="45" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="D19" s="45" t="inlineStr">
+      <c r="D17" s="45" t="inlineStr">
         <is>
           <t>가중 달성률 →</t>
         </is>
       </c>
-      <c r="E19" s="42" t="n"/>
-      <c r="F19" s="21">
-        <f>SUM(F12:F18)</f>
-        <v/>
-      </c>
-      <c r="G19" s="28">
-        <f>SUMPRODUCT(F12:F18,H12:H18)</f>
-        <v/>
-      </c>
-      <c r="H19" s="29">
-        <f>COUNTIF(G12:G18,"완료")</f>
-        <v/>
-      </c>
-      <c r="I19" s="115">
-        <f>SUM(I12:I18)</f>
-        <v/>
-      </c>
-      <c r="J19" s="69">
-        <f>"완료 "&amp;COUNTIF(G12:G18,"완료")&amp;"건 / 진행중 "&amp;COUNTIF(G12:G18,"진행중")&amp;"건 / 미착수 "&amp;COUNTIF(G12:G18,"미착수")&amp;"건"</f>
-        <v/>
-      </c>
-      <c r="K19" s="41" t="n"/>
-      <c r="L19" s="42" t="n"/>
+      <c r="E17" s="42" t="n"/>
+      <c r="F17" s="21">
+        <f>SUM(F12:F16)</f>
+        <v/>
+      </c>
+      <c r="G17" s="28">
+        <f>SUMPRODUCT(F12:F16,H12:H16)</f>
+        <v/>
+      </c>
+      <c r="H17" s="29">
+        <f>COUNTIF(G12:G16,"완료")</f>
+        <v/>
+      </c>
+      <c r="I17" s="115">
+        <f>SUM(I12:I16)</f>
+        <v/>
+      </c>
+      <c r="J17" s="69">
+        <f>"완료 "&amp;COUNTIF(G12:G16,"완료")&amp;"건 / 진행중 "&amp;COUNTIF(G12:G16,"진행중")&amp;"건 / 미착수 "&amp;COUNTIF(G12:G16,"미착수")&amp;"건"</f>
+        <v/>
+      </c>
+      <c r="K17" s="41" t="n"/>
+      <c r="L17" s="42" t="n"/>
+    </row>
+    <row r="18" ht="24" customHeight="1" s="49">
+      <c r="C18" s="46" t="n"/>
+      <c r="D18" s="46" t="n"/>
+      <c r="I18" s="46" t="n"/>
+      <c r="J18" s="46" t="n"/>
+      <c r="L18" s="46" t="n"/>
+    </row>
+    <row r="19" ht="19.5" customHeight="1" s="49">
+      <c r="C19" s="121" t="inlineStr">
+        <is>
+          <t>2. 자가 검수  —  제출 전 §4 검수기준으로 본인이 먼저 점검</t>
+        </is>
+      </c>
+      <c r="D19" s="64" t="n"/>
+      <c r="E19" s="64" t="n"/>
+      <c r="F19" s="64" t="n"/>
+      <c r="G19" s="64" t="n"/>
+      <c r="H19" s="64" t="n"/>
+      <c r="I19" s="64" t="n"/>
+      <c r="J19" s="64" t="n"/>
+      <c r="K19" s="64" t="n"/>
+      <c r="L19" s="65" t="n"/>
     </row>
     <row r="20" ht="24" customHeight="1" s="49">
-      <c r="C20" s="46" t="n"/>
-      <c r="D20" s="46" t="n"/>
-      <c r="I20" s="46" t="n"/>
-      <c r="J20" s="46" t="n"/>
-      <c r="L20" s="46" t="n"/>
-    </row>
-    <row r="21" ht="19.5" customHeight="1" s="49">
-      <c r="C21" s="121" t="inlineStr">
-        <is>
-          <t>2. 자가 검수  —  제출 전 §4 검수기준으로 본인이 먼저 점검</t>
-        </is>
-      </c>
-      <c r="D21" s="64" t="n"/>
-      <c r="E21" s="64" t="n"/>
-      <c r="F21" s="64" t="n"/>
-      <c r="G21" s="64" t="n"/>
-      <c r="H21" s="64" t="n"/>
-      <c r="I21" s="64" t="n"/>
-      <c r="J21" s="64" t="n"/>
-      <c r="K21" s="64" t="n"/>
-      <c r="L21" s="65" t="n"/>
+      <c r="C20" s="46" t="inlineStr">
+        <is>
+          <t>검수 항목 (자동)</t>
+        </is>
+      </c>
+      <c r="D20" s="46" t="inlineStr">
+        <is>
+          <t>검수 질문 (자동)</t>
+        </is>
+      </c>
+      <c r="E20" s="41" t="n"/>
+      <c r="F20" s="41" t="n"/>
+      <c r="G20" s="41" t="n"/>
+      <c r="H20" s="42" t="n"/>
+      <c r="I20" s="46" t="inlineStr">
+        <is>
+          <t>자가
+판정</t>
+        </is>
+      </c>
+      <c r="J20" s="46" t="inlineStr">
+        <is>
+          <t>미충족 사유·보완 계획</t>
+        </is>
+      </c>
+      <c r="K20" s="42" t="n"/>
+      <c r="L20" s="46" t="inlineStr">
+        <is>
+          <t>검수자
+판정</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1" s="49">
+      <c r="C21" s="69" t="n"/>
+      <c r="D21" s="55" t="n"/>
+      <c r="E21" s="41" t="n"/>
+      <c r="F21" s="41" t="n"/>
+      <c r="G21" s="41" t="n"/>
+      <c r="H21" s="42" t="n"/>
+      <c r="I21" s="47" t="n"/>
+      <c r="J21" s="44" t="n"/>
+      <c r="K21" s="42" t="n"/>
+      <c r="L21" s="66" t="n"/>
     </row>
     <row r="22" ht="24" customHeight="1" s="49">
-      <c r="C22" s="46" t="inlineStr">
-        <is>
-          <t>검수 항목 (자동)</t>
-        </is>
-      </c>
-      <c r="D22" s="46" t="inlineStr">
-        <is>
-          <t>검수 질문 (자동)</t>
-        </is>
-      </c>
+      <c r="C22" s="69" t="n"/>
+      <c r="D22" s="55" t="n"/>
       <c r="E22" s="41" t="n"/>
       <c r="F22" s="41" t="n"/>
       <c r="G22" s="41" t="n"/>
       <c r="H22" s="42" t="n"/>
-      <c r="I22" s="46" t="inlineStr">
-        <is>
-          <t>자가
-판정</t>
-        </is>
-      </c>
-      <c r="J22" s="46" t="inlineStr">
-        <is>
-          <t>미충족 사유·보완 계획</t>
-        </is>
-      </c>
+      <c r="I22" s="47" t="n"/>
+      <c r="J22" s="44" t="n"/>
       <c r="K22" s="42" t="n"/>
-      <c r="L22" s="46" t="inlineStr">
-        <is>
-          <t>검수자
-판정</t>
-        </is>
-      </c>
+      <c r="L22" s="66" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1" s="49">
       <c r="C23" s="69" t="n"/>
@@ -3318,110 +3194,110 @@
       <c r="K27" s="42" t="n"/>
       <c r="L27" s="66" t="n"/>
     </row>
-    <row r="28" ht="24" customHeight="1" s="49">
-      <c r="C28" s="69" t="n"/>
-      <c r="D28" s="55" t="n"/>
-      <c r="E28" s="41" t="n"/>
-      <c r="F28" s="41" t="n"/>
-      <c r="G28" s="41" t="n"/>
-      <c r="H28" s="42" t="n"/>
-      <c r="I28" s="47" t="n"/>
-      <c r="J28" s="44" t="n"/>
-      <c r="K28" s="42" t="n"/>
-      <c r="L28" s="66" t="n"/>
-    </row>
-    <row r="29" ht="24" customHeight="1" s="49">
-      <c r="C29" s="69" t="n"/>
-      <c r="D29" s="55" t="n"/>
-      <c r="E29" s="41" t="n"/>
-      <c r="F29" s="41" t="n"/>
-      <c r="G29" s="41" t="n"/>
-      <c r="H29" s="42" t="n"/>
-      <c r="I29" s="47" t="n"/>
-      <c r="J29" s="44" t="n"/>
-      <c r="K29" s="42" t="n"/>
-      <c r="L29" s="66" t="n"/>
+    <row r="28" ht="27.75" customHeight="1" s="49">
+      <c r="C28" s="46" t="n"/>
+      <c r="D28" s="46" t="n"/>
+      <c r="E28" s="46" t="n"/>
+      <c r="F28" s="46" t="n"/>
+      <c r="G28" s="46" t="n"/>
+      <c r="H28" s="46" t="n"/>
+      <c r="I28" s="46" t="n"/>
+      <c r="J28" s="46" t="n"/>
+      <c r="K28" s="46" t="n"/>
+      <c r="L28" s="46" t="n"/>
+    </row>
+    <row r="29" ht="19.5" customHeight="1" s="49">
+      <c r="C29" s="121" t="inlineStr">
+        <is>
+          <t>3. 이슈 및 지원요청  —  대안 없이 문제만 올리는 보고는 반려</t>
+        </is>
+      </c>
+      <c r="D29" s="64" t="n"/>
+      <c r="E29" s="64" t="n"/>
+      <c r="F29" s="64" t="n"/>
+      <c r="G29" s="64" t="n"/>
+      <c r="H29" s="64" t="n"/>
+      <c r="I29" s="64" t="n"/>
+      <c r="J29" s="64" t="n"/>
+      <c r="K29" s="64" t="n"/>
+      <c r="L29" s="65" t="n"/>
     </row>
     <row r="30" ht="27.75" customHeight="1" s="49">
-      <c r="C30" s="46" t="n"/>
-      <c r="D30" s="46" t="n"/>
-      <c r="E30" s="46" t="n"/>
-      <c r="F30" s="46" t="n"/>
-      <c r="G30" s="46" t="n"/>
-      <c r="H30" s="46" t="n"/>
-      <c r="I30" s="46" t="n"/>
-      <c r="J30" s="46" t="n"/>
-      <c r="K30" s="46" t="n"/>
-      <c r="L30" s="46" t="n"/>
-    </row>
-    <row r="31" ht="19.5" customHeight="1" s="49">
-      <c r="C31" s="121" t="inlineStr">
-        <is>
-          <t>3. 이슈 및 지원요청  —  대안 없이 문제만 올리는 보고는 반려</t>
-        </is>
-      </c>
-      <c r="D31" s="64" t="n"/>
-      <c r="E31" s="64" t="n"/>
-      <c r="F31" s="64" t="n"/>
-      <c r="G31" s="64" t="n"/>
-      <c r="H31" s="64" t="n"/>
-      <c r="I31" s="64" t="n"/>
-      <c r="J31" s="64" t="n"/>
-      <c r="K31" s="64" t="n"/>
-      <c r="L31" s="65" t="n"/>
-    </row>
-    <row r="32" ht="27.75" customHeight="1" s="49">
-      <c r="C32" s="46" t="inlineStr">
+      <c r="C30" s="46" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="D32" s="46" t="inlineStr">
+      <c r="D30" s="46" t="inlineStr">
         <is>
           <t>이슈 내용</t>
         </is>
       </c>
-      <c r="E32" s="46" t="inlineStr">
+      <c r="E30" s="46" t="inlineStr">
         <is>
           <t>영향
 (일정/비용/품질)</t>
         </is>
       </c>
-      <c r="F32" s="46" t="inlineStr">
+      <c r="F30" s="46" t="inlineStr">
         <is>
           <t>근본 원인</t>
         </is>
       </c>
-      <c r="G32" s="46" t="inlineStr">
+      <c r="G30" s="46" t="inlineStr">
         <is>
           <t>대안 1</t>
         </is>
       </c>
-      <c r="H32" s="46" t="inlineStr">
+      <c r="H30" s="46" t="inlineStr">
         <is>
           <t>대안 2</t>
         </is>
       </c>
-      <c r="I32" s="46" t="inlineStr">
+      <c r="I30" s="46" t="inlineStr">
         <is>
           <t>권고안</t>
         </is>
       </c>
-      <c r="J32" s="46" t="inlineStr">
+      <c r="J30" s="46" t="inlineStr">
         <is>
           <t>요청사항</t>
         </is>
       </c>
-      <c r="K32" s="46" t="inlineStr">
+      <c r="K30" s="46" t="inlineStr">
         <is>
           <t>결정기한</t>
         </is>
       </c>
-      <c r="L32" s="46" t="inlineStr">
+      <c r="L30" s="46" t="inlineStr">
         <is>
           <t>대표 결정</t>
         </is>
       </c>
+    </row>
+    <row r="31" ht="36" customHeight="1" s="49">
+      <c r="C31" s="6" t="n"/>
+      <c r="D31" s="18" t="n"/>
+      <c r="E31" s="6" t="n"/>
+      <c r="F31" s="18" t="n"/>
+      <c r="G31" s="18" t="n"/>
+      <c r="H31" s="18" t="n"/>
+      <c r="I31" s="18" t="n"/>
+      <c r="J31" s="18" t="n"/>
+      <c r="K31" s="6" t="n"/>
+      <c r="L31" s="66" t="n"/>
+    </row>
+    <row r="32" ht="36" customHeight="1" s="49">
+      <c r="C32" s="6" t="n"/>
+      <c r="D32" s="18" t="n"/>
+      <c r="E32" s="6" t="n"/>
+      <c r="F32" s="18" t="n"/>
+      <c r="G32" s="18" t="n"/>
+      <c r="H32" s="18" t="n"/>
+      <c r="I32" s="18" t="n"/>
+      <c r="J32" s="18" t="n"/>
+      <c r="K32" s="6" t="n"/>
+      <c r="L32" s="66" t="n"/>
     </row>
     <row r="33" ht="36" customHeight="1" s="49">
       <c r="C33" s="6" t="n"/>
@@ -3435,114 +3311,118 @@
       <c r="K33" s="6" t="n"/>
       <c r="L33" s="66" t="n"/>
     </row>
-    <row r="34" ht="36" customHeight="1" s="49">
-      <c r="C34" s="6" t="n"/>
-      <c r="D34" s="18" t="n"/>
-      <c r="E34" s="6" t="n"/>
-      <c r="F34" s="18" t="n"/>
-      <c r="G34" s="18" t="n"/>
-      <c r="H34" s="18" t="n"/>
-      <c r="I34" s="18" t="n"/>
-      <c r="J34" s="18" t="n"/>
-      <c r="K34" s="6" t="n"/>
-      <c r="L34" s="66" t="n"/>
-    </row>
-    <row r="35" ht="36" customHeight="1" s="49">
-      <c r="C35" s="6" t="n"/>
-      <c r="D35" s="18" t="n"/>
-      <c r="E35" s="6" t="n"/>
-      <c r="F35" s="18" t="n"/>
-      <c r="G35" s="18" t="n"/>
-      <c r="H35" s="18" t="n"/>
-      <c r="I35" s="18" t="n"/>
-      <c r="J35" s="18" t="n"/>
-      <c r="K35" s="6" t="n"/>
-      <c r="L35" s="66" t="n"/>
+    <row r="34" ht="27.75" customHeight="1" s="49">
+      <c r="C34" s="13" t="n"/>
+      <c r="D34" s="46" t="n"/>
+      <c r="E34" s="46" t="n"/>
+      <c r="F34" s="46" t="n"/>
+      <c r="G34" s="46" t="n"/>
+      <c r="H34" s="46" t="n"/>
+      <c r="I34" s="46" t="n"/>
+      <c r="J34" s="46" t="n"/>
+      <c r="K34" s="46" t="n"/>
+      <c r="L34" s="46" t="n"/>
+    </row>
+    <row r="35" ht="19.5" customHeight="1" s="49">
+      <c r="C35" s="121" t="inlineStr">
+        <is>
+          <t>4. 다음 주 제안 업무  —  지시를 기다리지 말 것. 본인이 먼저 제안.</t>
+        </is>
+      </c>
+      <c r="D35" s="64" t="n"/>
+      <c r="E35" s="64" t="n"/>
+      <c r="F35" s="64" t="n"/>
+      <c r="G35" s="64" t="n"/>
+      <c r="H35" s="64" t="n"/>
+      <c r="I35" s="64" t="n"/>
+      <c r="J35" s="64" t="n"/>
+      <c r="K35" s="64" t="n"/>
+      <c r="L35" s="65" t="n"/>
     </row>
     <row r="36" ht="27.75" customHeight="1" s="49">
-      <c r="C36" s="13" t="n"/>
-      <c r="D36" s="46" t="n"/>
-      <c r="E36" s="46" t="n"/>
-      <c r="F36" s="46" t="n"/>
-      <c r="G36" s="46" t="n"/>
-      <c r="H36" s="46" t="n"/>
-      <c r="I36" s="46" t="n"/>
-      <c r="J36" s="46" t="n"/>
-      <c r="K36" s="46" t="n"/>
-      <c r="L36" s="46" t="n"/>
-    </row>
-    <row r="37" ht="19.5" customHeight="1" s="49">
-      <c r="C37" s="121" t="inlineStr">
-        <is>
-          <t>4. 다음 주 제안 업무  —  지시를 기다리지 말 것. 본인이 먼저 제안.</t>
-        </is>
-      </c>
-      <c r="D37" s="64" t="n"/>
-      <c r="E37" s="64" t="n"/>
-      <c r="F37" s="64" t="n"/>
-      <c r="G37" s="64" t="n"/>
-      <c r="H37" s="64" t="n"/>
-      <c r="I37" s="64" t="n"/>
-      <c r="J37" s="64" t="n"/>
-      <c r="K37" s="64" t="n"/>
-      <c r="L37" s="65" t="n"/>
-    </row>
-    <row r="38" ht="27.75" customHeight="1" s="49">
-      <c r="C38" s="13" t="inlineStr">
+      <c r="C36" s="13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D38" s="46" t="inlineStr">
+      <c r="D36" s="46" t="inlineStr">
         <is>
           <t>제안 업무</t>
         </is>
       </c>
-      <c r="E38" s="46" t="inlineStr">
+      <c r="E36" s="46" t="inlineStr">
         <is>
           <t>왜 해야 하는가</t>
         </is>
       </c>
-      <c r="F38" s="46" t="inlineStr">
+      <c r="F36" s="46" t="inlineStr">
         <is>
           <t>완료기준(안)</t>
         </is>
       </c>
-      <c r="G38" s="46" t="inlineStr">
+      <c r="G36" s="46" t="inlineStr">
         <is>
           <t>예상
 소요(h)</t>
         </is>
       </c>
-      <c r="H38" s="46" t="inlineStr">
+      <c r="H36" s="46" t="inlineStr">
         <is>
           <t>우선순위(안)</t>
         </is>
       </c>
-      <c r="I38" s="46" t="inlineStr">
+      <c r="I36" s="46" t="inlineStr">
         <is>
           <t>선행 조건</t>
         </is>
       </c>
-      <c r="J38" s="46" t="inlineStr">
+      <c r="J36" s="46" t="inlineStr">
         <is>
           <t>필요 지원</t>
         </is>
       </c>
-      <c r="K38" s="46" t="inlineStr">
+      <c r="K36" s="46" t="inlineStr">
         <is>
           <t>대표 승인</t>
         </is>
       </c>
-      <c r="L38" s="46" t="inlineStr">
+      <c r="L36" s="46" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
+    </row>
+    <row r="37" ht="31.5" customHeight="1" s="49">
+      <c r="C37" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="18" t="n"/>
+      <c r="E37" s="18" t="n"/>
+      <c r="F37" s="18" t="n"/>
+      <c r="G37" s="114" t="n"/>
+      <c r="H37" s="6" t="n"/>
+      <c r="I37" s="18" t="n"/>
+      <c r="J37" s="18" t="n"/>
+      <c r="K37" s="66" t="n"/>
+      <c r="L37" s="6" t="n"/>
+    </row>
+    <row r="38" ht="31.5" customHeight="1" s="49">
+      <c r="C38" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" s="18" t="n"/>
+      <c r="E38" s="18" t="n"/>
+      <c r="F38" s="18" t="n"/>
+      <c r="G38" s="114" t="n"/>
+      <c r="H38" s="6" t="n"/>
+      <c r="I38" s="18" t="n"/>
+      <c r="J38" s="18" t="n"/>
+      <c r="K38" s="66" t="n"/>
+      <c r="L38" s="6" t="n"/>
     </row>
     <row r="39" ht="31.5" customHeight="1" s="49">
       <c r="C39" s="22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D39" s="18" t="n"/>
       <c r="E39" s="18" t="n"/>
@@ -3556,7 +3436,7 @@
     </row>
     <row r="40" ht="31.5" customHeight="1" s="49">
       <c r="C40" s="22" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D40" s="18" t="n"/>
       <c r="E40" s="18" t="n"/>
@@ -3568,55 +3448,70 @@
       <c r="K40" s="66" t="n"/>
       <c r="L40" s="6" t="n"/>
     </row>
-    <row r="41" ht="31.5" customHeight="1" s="49">
-      <c r="C41" s="22" t="n">
-        <v>3</v>
-      </c>
-      <c r="D41" s="18" t="n"/>
-      <c r="E41" s="18" t="n"/>
-      <c r="F41" s="18" t="n"/>
-      <c r="G41" s="114" t="n"/>
-      <c r="H41" s="6" t="n"/>
-      <c r="I41" s="18" t="n"/>
-      <c r="J41" s="18" t="n"/>
-      <c r="K41" s="66" t="n"/>
-      <c r="L41" s="6" t="n"/>
-    </row>
-    <row r="42" ht="31.5" customHeight="1" s="49">
-      <c r="C42" s="22" t="n">
-        <v>4</v>
-      </c>
-      <c r="D42" s="18" t="n"/>
-      <c r="E42" s="18" t="n"/>
-      <c r="F42" s="18" t="n"/>
-      <c r="G42" s="114" t="n"/>
-      <c r="H42" s="6" t="n"/>
-      <c r="I42" s="18" t="n"/>
-      <c r="J42" s="18" t="n"/>
-      <c r="K42" s="66" t="n"/>
-      <c r="L42" s="6" t="n"/>
+    <row r="41" ht="25.5" customHeight="1" s="49">
+      <c r="C41" s="45" t="n"/>
+      <c r="D41" s="43" t="n"/>
+      <c r="J41" s="58" t="n"/>
+    </row>
+    <row r="42" ht="19.5" customHeight="1" s="49">
+      <c r="C42" s="48" t="inlineStr">
+        <is>
+          <t>5. 자기점검 및 대표 검수</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="25.5" customHeight="1" s="49">
-      <c r="C43" s="45" t="n"/>
-      <c r="D43" s="43" t="n"/>
-      <c r="J43" s="58" t="n"/>
-    </row>
-    <row r="44" ht="19.5" customHeight="1" s="49">
-      <c r="C44" s="48" t="inlineStr">
-        <is>
-          <t>5. 자기점검 및 대표 검수</t>
-        </is>
-      </c>
+      <c r="C43" s="45" t="inlineStr">
+        <is>
+          <t>이번 주 가장 잘한 것</t>
+        </is>
+      </c>
+      <c r="D43" s="43" t="inlineStr">
+        <is>
+          <t>결과로 증명되는 것 1개만</t>
+        </is>
+      </c>
+      <c r="E43" s="41" t="n"/>
+      <c r="F43" s="41" t="n"/>
+      <c r="G43" s="41" t="n"/>
+      <c r="H43" s="41" t="n"/>
+      <c r="I43" s="42" t="n"/>
+      <c r="J43" s="58" t="inlineStr">
+        <is>
+          <t>[대표 검수 의견]</t>
+        </is>
+      </c>
+      <c r="K43" s="59" t="n"/>
+      <c r="L43" s="60" t="n"/>
+    </row>
+    <row r="44" ht="25.5" customHeight="1" s="49">
+      <c r="C44" s="45" t="inlineStr">
+        <is>
+          <t>이번 주 가장 부족한 것</t>
+        </is>
+      </c>
+      <c r="D44" s="43" t="inlineStr">
+        <is>
+          <t>변명 말고 사실만</t>
+        </is>
+      </c>
+      <c r="E44" s="41" t="n"/>
+      <c r="F44" s="41" t="n"/>
+      <c r="G44" s="41" t="n"/>
+      <c r="H44" s="41" t="n"/>
+      <c r="I44" s="42" t="n"/>
+      <c r="J44" s="61" t="n"/>
+      <c r="L44" s="62" t="n"/>
     </row>
     <row r="45" ht="25.5" customHeight="1" s="49">
       <c r="C45" s="45" t="inlineStr">
         <is>
-          <t>이번 주 가장 잘한 것</t>
+          <t>다음 주 개선 액션 1개</t>
         </is>
       </c>
       <c r="D45" s="43" t="inlineStr">
         <is>
-          <t>결과로 증명되는 것 1개만</t>
+          <t>실행 가능한 행동으로</t>
         </is>
       </c>
       <c r="E45" s="41" t="n"/>
@@ -3624,128 +3519,85 @@
       <c r="G45" s="41" t="n"/>
       <c r="H45" s="41" t="n"/>
       <c r="I45" s="42" t="n"/>
-      <c r="J45" s="58" t="inlineStr">
-        <is>
-          <t>[대표 검수 의견]</t>
-        </is>
-      </c>
-      <c r="K45" s="59" t="n"/>
-      <c r="L45" s="60" t="n"/>
-    </row>
-    <row r="46" ht="25.5" customHeight="1" s="49">
-      <c r="C46" s="45" t="inlineStr">
-        <is>
-          <t>이번 주 가장 부족한 것</t>
-        </is>
-      </c>
-      <c r="D46" s="43" t="inlineStr">
-        <is>
-          <t>변명 말고 사실만</t>
-        </is>
-      </c>
-      <c r="E46" s="41" t="n"/>
-      <c r="F46" s="41" t="n"/>
-      <c r="G46" s="41" t="n"/>
-      <c r="H46" s="41" t="n"/>
-      <c r="I46" s="42" t="n"/>
-      <c r="J46" s="61" t="n"/>
-      <c r="L46" s="62" t="n"/>
-    </row>
-    <row r="47" ht="25.5" customHeight="1" s="49">
+      <c r="J45" s="63" t="n"/>
+      <c r="K45" s="64" t="n"/>
+      <c r="L45" s="65" t="n"/>
+    </row>
+    <row r="47" ht="33.75" customHeight="1" s="49">
       <c r="C47" s="45" t="inlineStr">
         <is>
-          <t>다음 주 개선 액션 1개</t>
-        </is>
-      </c>
-      <c r="D47" s="43" t="inlineStr">
-        <is>
-          <t>실행 가능한 행동으로</t>
-        </is>
-      </c>
+          <t>제출자</t>
+        </is>
+      </c>
+      <c r="D47" s="47" t="n"/>
       <c r="E47" s="41" t="n"/>
-      <c r="F47" s="41" t="n"/>
-      <c r="G47" s="41" t="n"/>
-      <c r="H47" s="41" t="n"/>
+      <c r="F47" s="42" t="n"/>
+      <c r="G47" s="45" t="inlineStr">
+        <is>
+          <t>검수자</t>
+        </is>
+      </c>
+      <c r="H47" s="66" t="n"/>
       <c r="I47" s="42" t="n"/>
-      <c r="J47" s="63" t="n"/>
-      <c r="K47" s="64" t="n"/>
-      <c r="L47" s="65" t="n"/>
-    </row>
-    <row r="49" ht="33.75" customHeight="1" s="49">
-      <c r="C49" s="45" t="inlineStr">
-        <is>
-          <t>제출자</t>
-        </is>
-      </c>
-      <c r="D49" s="47" t="n"/>
-      <c r="E49" s="41" t="n"/>
-      <c r="F49" s="42" t="n"/>
-      <c r="G49" s="45" t="inlineStr">
-        <is>
-          <t>검수자</t>
-        </is>
-      </c>
-      <c r="H49" s="66" t="n"/>
-      <c r="I49" s="42" t="n"/>
-      <c r="J49" s="45" t="inlineStr">
+      <c r="J47" s="45" t="inlineStr">
         <is>
           <t>최종 판정</t>
         </is>
       </c>
-      <c r="K49" s="56" t="n"/>
-      <c r="L49" s="42" t="n"/>
+      <c r="K47" s="56" t="n"/>
+      <c r="L47" s="42" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="K49:L49"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="D20:H20"/>
     <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D47:I47"/>
+    <mergeCell ref="D47:F47"/>
     <mergeCell ref="D7:L7"/>
-    <mergeCell ref="C37:L37"/>
-    <mergeCell ref="J45:L47"/>
+    <mergeCell ref="D43:I43"/>
+    <mergeCell ref="C19:L19"/>
+    <mergeCell ref="D21:H21"/>
+    <mergeCell ref="K47:L47"/>
     <mergeCell ref="J24:K24"/>
-    <mergeCell ref="H49:I49"/>
     <mergeCell ref="D27:H27"/>
     <mergeCell ref="J27:K27"/>
+    <mergeCell ref="C42:L42"/>
+    <mergeCell ref="D17:E17"/>
     <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J20:K20"/>
     <mergeCell ref="J25:K25"/>
-    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="C29:L29"/>
+    <mergeCell ref="C35:L35"/>
+    <mergeCell ref="J43:L45"/>
+    <mergeCell ref="J17:L17"/>
+    <mergeCell ref="D44:I44"/>
     <mergeCell ref="J22:K22"/>
+    <mergeCell ref="H47:I47"/>
     <mergeCell ref="C1:L1"/>
-    <mergeCell ref="C44:L44"/>
+    <mergeCell ref="J21:K21"/>
     <mergeCell ref="D25:H25"/>
-    <mergeCell ref="C31:L31"/>
-    <mergeCell ref="D46:I46"/>
     <mergeCell ref="C9:L9"/>
     <mergeCell ref="D24:H24"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="C21:L21"/>
     <mergeCell ref="D45:I45"/>
     <mergeCell ref="D23:H23"/>
     <mergeCell ref="J23:K23"/>
     <mergeCell ref="C2:L2"/>
     <mergeCell ref="D6:L6"/>
-    <mergeCell ref="D49:F49"/>
     <mergeCell ref="D26:H26"/>
   </mergeCells>
   <dataValidations count="5">
-    <dataValidation sqref="I23:I29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I21:I27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"충족,미충족"</formula1>
     </dataValidation>
-    <dataValidation sqref="L23:L29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L21:L27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"합격,보완,불합격"</formula1>
     </dataValidation>
-    <dataValidation sqref="K39:K42 L33:L35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K37:K40 L31:L33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"승인,보류,반려"</formula1>
     </dataValidation>
-    <dataValidation sqref="K49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"합격,조건부합격,보완요청,불합격"</formula1>
     </dataValidation>
-    <dataValidation sqref="G12:G18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G12:G16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"완료,진행중,미착수,보류,취소"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Revise 황우중 W30 task 1 to follow TRL report writing guide
Drop the guide-reconciliation (room/window→entrance) step; task 1 now
directs writing the report body per the company's TRL1 writing guide
with thorough research, and states the report's purpose (surface gaps,
supplement, clarify, evidence base). Tasks 2-5 unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPtt2MinYXH5T7wMFXyfVt
</commit_message>
<xml_diff>
--- a/out/BRING_주간_황우중_2026-W30.xlsx
+++ b/out/BRING_주간_황우중_2026-W30.xlsx
@@ -1694,8 +1694,8 @@
       <c r="C8" s="70" t="inlineStr">
         <is>
           <t>대표가 제1장에서 회사의 기술개발 방향을 확정하였습니다. 확정된 방향은 '노후 소형건축물의 입구 1개소'를 처음 적용 대상으로 하여, 현장을 3D로 실측하고 그 형상에 맞춰 표준 프레임과 맞춤형 연결부, 탈부착이 가능한 기능 카세트를 공장에서 미리 만들어 현장에 조립·설치하는 리트로핏(개선) 기술입니다.
-다만 예전에 만들어 둔 TRL1 보고서 작성 가이드는 '방 1개·창문 1~2개'와 센서 중심으로 쓰여 있어, 지금 확정된 '건물 입구' 방향과 맞지 않는 부분이 많습니다. 이 상태로 본문을 쓰면 옛 방향(방·창문)이 그대로 섞여 나옵니다.
-따라서 이번 주에는 이 보고서의 본문을 실제로 쓰는 일을 최우선으로 하고, 거기서 나온 내용이 나머지 산출물(표·그림·연구가설·위험요소 등)로 이어지도록 진행합니다.</t>
+이번 주에는 이 방향을 담은 TRL1 연구개발보고서의 본문을 실제로 작성하는 일을 최우선으로 합니다. 이 보고서는 단순한 서류가 아니라 ① 우리가 미처 생각하지 못한 부분을 짚어보고 ② 부족한 부분을 보완하며 ③ 명확히 해야 할 것을 정리하고 ④ 앞으로 대외적으로 설명할 때 근거가 되는 자료입니다.
+따라서 관련 자료·사례·기술을 최대한 많이 찾아보고 공부하여, 회사의 TRL1 보고서 작성 요령에 따라 충실히 작성하는 것이 목적입니다.</t>
         </is>
       </c>
       <c r="D8" s="41" t="n"/>
@@ -1716,7 +1716,7 @@
       </c>
       <c r="C9" s="73" t="inlineStr">
         <is>
-          <t>제1장에서 확정된 '건물 입구 1개소' 중심 리트로핏 방향을 기준으로 TRL1 연구개발보고서의 본문을 작성하고, 그 내용을 뒷받침하는 표·그림·연구가설·위험요소를 함께 정리하는 것입니다.</t>
+          <t>제1장에서 확정된 방향을 기준으로, 회사의 TRL1 보고서 작성 요령에 따라 연구개발보고서 본문을 충실히 작성하고, 그 내용을 뒷받침하는 표·그림·연구가설·위험요소를 함께 정리하는 것입니다.</t>
         </is>
       </c>
       <c r="D9" s="41" t="n"/>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="C10" s="73" t="inlineStr">
         <is>
-          <t>보고서가 옛 방향(방·창문)과 섞이면, 이후 모든 장의 논리가 흔들리고 다시 써야 합니다. 또한 문제→기술→구조→검증으로 이어지는 논리가 정리되지 않으면, 다음 단계(TRL2)의 개념검증·시제품 일정이 함께 미뤄지고 재작업 부담이 커집니다.</t>
+          <t>보고서의 논리(문제 → 기술 → 구조 → 검증)가 제대로 정리되지 않으면, 이후 모든 장을 다시 써야 하고 다음 단계(TRL2)의 개념검증·시제품 일정이 함께 미뤄집니다. 또한 대외적으로 설명할 때 근거로 삼을 자료가 부실해집니다.</t>
         </is>
       </c>
       <c r="D10" s="41" t="n"/>
@@ -1808,7 +1808,7 @@
       <c r="B15" s="112" t="n"/>
       <c r="C15" s="111" t="inlineStr">
         <is>
-          <t>예전 작성 가이드의 '방·창문·외벽' 중심 표현을 '건물 입구' 기준으로 고쳐 맞춘 뒤 본문 작성</t>
+          <t>회사 TRL1 보고서 작성 요령(장·절 구성 방법)에 따라 본문 작성</t>
         </is>
       </c>
       <c r="D15" s="41" t="n"/>
@@ -1824,7 +1824,7 @@
       <c r="B16" s="112" t="n"/>
       <c r="C16" s="111" t="inlineStr">
         <is>
-          <t>TRL1 연구개발보고서 본문(문제 정의 → 기술 개념 → 시스템·제품 구조) 초안 작성</t>
+          <t>관련 자료·사례·기술을 충분히 조사하여 근거와 출처 확보</t>
         </is>
       </c>
       <c r="D16" s="41" t="n"/>
@@ -1840,7 +1840,7 @@
       <c r="B17" s="112" t="n"/>
       <c r="C17" s="111" t="inlineStr">
         <is>
-          <t>본문을 뒷받침하는 핵심 표·그림을 발표용 슬라이드(PPT)로 제작</t>
+          <t>TRL1 연구개발보고서 본문(문제 정의 → 기술 개념 → 시스템·제품 구조) 초안 작성</t>
         </is>
       </c>
       <c r="D17" s="41" t="n"/>
@@ -1856,7 +1856,7 @@
       <c r="B18" s="112" t="n"/>
       <c r="C18" s="111" t="inlineStr">
         <is>
-          <t>연구가설과 다음 단계 검증계획 정리</t>
+          <t>본문을 뒷받침하는 핵심 표·그림을 발표용 슬라이드(PPT)로 제작</t>
         </is>
       </c>
       <c r="D18" s="41" t="n"/>
@@ -1872,7 +1872,7 @@
       <c r="B19" s="112" t="n"/>
       <c r="C19" s="113" t="inlineStr">
         <is>
-          <t>위험요소와 나중에 측정할 성능지표 후보 정리</t>
+          <t>연구가설과 다음 단계 검증계획 정리</t>
         </is>
       </c>
       <c r="D19" s="41" t="n"/>
@@ -1888,7 +1888,7 @@
       <c r="B20" s="112" t="n"/>
       <c r="C20" s="111" t="inlineStr">
         <is>
-          <t>확인되지 않은 가정·대표 검토가 필요한 쟁점·용어 정리</t>
+          <t>위험요소와 나중에 측정할 성능지표 후보 정리</t>
         </is>
       </c>
       <c r="D20" s="41" t="n"/>
@@ -1902,7 +1902,11 @@
     </row>
     <row r="21" ht="33.75" customHeight="1" s="49">
       <c r="B21" s="112" t="n"/>
-      <c r="C21" s="113" t="n"/>
+      <c r="C21" s="113" t="inlineStr">
+        <is>
+          <t>확인되지 않은 가정·대표 검토가 필요한 쟁점·용어 정리</t>
+        </is>
+      </c>
       <c r="D21" s="41" t="n"/>
       <c r="E21" s="41" t="n"/>
       <c r="F21" s="41" t="n"/>
@@ -1951,7 +1955,7 @@
 · TRL1 단계에 맞춰, 문제 관찰·기술 원리·개념 정의·연구가설·적용/제외 조건·후보 성능지표·다음 단계 계획까지만 작성합니다
 · '이미 성능을 달성했다 / 스마트공장을 지금 구축한다 / 자동설계가 완성됐다 / 원가를 이미 절감했다'와 같은 완성형 표현은 지양해 주시기 바랍니다
 · 서술은 □ 큰 주제 / ○ 세부 주제 / • 현황·원인·필요성·대응방향·이번 단계 정립사항 순서로 정리해 주시면 읽기 쉽습니다
-· 첨부된 예전 가이드는 참고자료이며, 입구 방향과 다를 경우 입구 방향을 우선합니다</t>
+· 회사 TRL1 보고서 작성 요령을 기준으로 삼아 작성합니다</t>
         </is>
       </c>
       <c r="D23" s="41" t="n"/>
@@ -2074,14 +2078,14 @@
       </c>
       <c r="D28" s="47" t="inlineStr">
         <is>
-          <t>보고서를 쓰기 전에, 예전 작성 가이드에서 '방·창문·외벽' 기준으로 된 부분을 지금 확정된 '건물 입구' 기준으로 먼저 고쳐 맞춘 뒤, 핵심 문제와 연구가설을 정하고 본문을 하나의 논리로 작성해 주시면 됩니다.</t>
+          <t>제1장에서 확정된 방향을 기준으로, 회사 TRL1 보고서 작성 요령에 따라 본문을 작성해 주시면 됩니다. 이 보고서는 단순 서류가 아니라 우리가 미처 생각하지 못한 점을 짚어 보완하고, 명확히 할 것을 정리하며, 앞으로 대외적으로 설명할 때 근거가 되는 자료입니다. 그러니 관련 자료를 최대한 많이 찾아보고 공부해서 충실히 작성해 주시면 됩니다.</t>
         </is>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>① 예전 가이드에서 '방·창문·외벽'으로 된 표현을 찾아 '건물 입구' 기준으로 어떻게 바꿀지 대조표(위치 / 기존 표현 / 수정 표현 / 초기적용·후속확장 구분)로 먼저 정리해 주시면 됩니다.
-② 보고서 전체가 답할 '핵심 문제 한 문장'과 그 아래 세부 문제들을 먼저 확정해 주시면 됩니다.
-③ 이어서 본문 초안을 (가)문제 정의 (나)기술 개념·전체 흐름 (다)시스템·제품 구조 순서로, 서로 연결되게 작성해 주시면 됩니다.
+          <t>① 회사 TRL1 보고서 작성 요령의 장·절 구성에 따라 본문(문제 정의 → 기술 개념·전체 흐름 → 시스템·제품 구조)을 서로 연결되게 작성해 주시면 됩니다.
+② 관련 자료·사례·기술을 충분히 조사하고, 근거와 출처를 함께 적어 주시면 됩니다.
+③ 우리가 놓쳤을 수 있는 점, 보완이 필요한 점, 명확히 정리해야 할 점을 찾아 함께 정리해 주시면 됩니다.
 ④ 아직 확인되지 않은 성능·효과는 '이미 달성'이 아니라 '다음 단계(TRL2)에서 확인할 항목'으로 적어 주시면 됩니다.</t>
         </is>
       </c>

</xml_diff>